<commit_message>
Acid/base regen loop write-convergence (completes Step 1 + balance --write restoration): o2_close write-path fixes - IA-VS-NAOH spent-return term added to the IA-BMED-04 purge (the base twin the assert diagnosed), stale x_par_12_base re-stamps retired (write_graph owns IA-EVAP_*-COND; they created a repulsive fixed point at 439.4 diverging +13.8 kg/d/pass), rounding-grid ping-pong resolved via solver.evap single-writer with 1 g/d epsilon, note-churn attractors guarded (S17-BMED/IA-BASE-PPT). IA-ACID-01 re-sized to the leach HCl demand per its own AQS-DUTY-011/X-RSZ-01 basis (439.61; misfit 0.00%). Convergence proven by sha: settle stable 7cd234ce, full regen converged in 2 passes at f4ef1fb7, --quick byte-stable. balance --write restored in the manifest. Tests 42P/1F (envelopes LFS-pointer only); tree golden at PV 405.3506; 700 files 0 stale; authority PASS.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -564,7 +564,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 b5f3c191a2f62c081c5312e6ced4676012463738b70786b3fb9406a5ff347a8a</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 f4ef1fb78bd813d7cade94d0ef3c343ac1bd731a6fd017218ec7f9ff4f5671ed</t>
         </is>
       </c>
     </row>
@@ -2032,7 +2032,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>1.975396</v>
+        <v>1.975408</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -2422,7 +2422,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>22.876312</v>
+        <v>22.876217</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -2662,7 +2662,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.975396</v>
+        <v>1.975408</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2842,7 +2842,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33.195596</v>
+        <v>33.195501</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -12410,7 +12410,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.360759</v>
+        <v>9.360747</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -12440,7 +12440,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>83.647854</v>
+        <v>83.647747</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -12470,7 +12470,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>74.28709499999999</v>
+        <v>74.28700000000001</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -12530,7 +12530,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.03208</v>
+        <v>0.032086</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -12620,7 +12620,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.032272</v>
+        <v>0.032278</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -12980,7 +12980,7 @@
         </is>
       </c>
       <c r="D50" t="n">
-        <v>22.876312</v>
+        <v>22.876217</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -13040,7 +13040,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>22.876312</v>
+        <v>22.876217</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -13370,7 +13370,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.975396</v>
+        <v>1.975408</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -13580,7 +13580,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>33.195596</v>
+        <v>33.195501</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -14507,7 +14507,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>83.647854</v>
+        <v>83.647747</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -14837,7 +14837,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>168.058609</v>
+        <v>168.058502</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -15039,7 +15039,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>165.23317</v>
+        <v>165.233063</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -15159,7 +15159,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>175.233209</v>
+        <v>175.233102</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -15489,7 +15489,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>308.578609</v>
+        <v>308.578502</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -15939,7 +15939,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>405.4928</v>
+        <v>405.3506</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -16725,7 +16725,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>405.4928</v>
+        <v>405.3506</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -17407,7 +17407,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1093.561663</v>
+        <v>1092.975294</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -17437,7 +17437,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1093.561663</v>
+        <v>1092.975294</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -44758,7 +44758,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>64.81344300000001</v>
+        <v>64.813948</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -44908,7 +44908,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>22.876312</v>
+        <v>22.876217</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -47368,7 +47368,7 @@
         <v>9</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>578.987</v>
+        <v>578.8448</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -47602,7 +47602,7 @@
         <v>3</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>409.501</v>
+        <v>409.3588</v>
       </c>
       <c r="I63" t="n">
         <v>3</v>
@@ -47719,7 +47719,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>405.4928</v>
+        <v>405.3506</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -55084,7 +55084,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>405.4928</v>
+        <v>405.3506</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -58928,7 +58928,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>439.6125</v>
+        <v>439.6127</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -59078,7 +59078,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>450.163884</v>
+        <v>450.164184</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -59678,7 +59678,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>865.1442</v>
+        <v>865.1446</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -59708,7 +59708,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1304.786</v>
+        <v>1304.7866</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -59918,7 +59918,7 @@
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3909.915497</v>
+        <v>3909.914016</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -59948,7 +59948,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>3896.339738</v>
+        <v>3896.338257</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -59978,7 +59978,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>3719.792521</v>
+        <v>3719.79104</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -60008,7 +60008,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>3707.26014</v>
+        <v>3707.257179</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -60038,7 +60038,7 @@
         </is>
       </c>
       <c r="D83" t="n">
-        <v>3520.31431</v>
+        <v>3520.311349</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -60668,7 +60668,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>7.40552</v>
+        <v>7.406995</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -60698,7 +60698,7 @@
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.03208</v>
+        <v>0.032086</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -60848,7 +60848,7 @@
         </is>
       </c>
       <c r="D110" t="n">
-        <v>7.44975</v>
+        <v>7.451224</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -60878,7 +60878,7 @@
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.032272</v>
+        <v>0.032278</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -61058,7 +61058,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>64.81344300000001</v>
+        <v>64.813948</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -61448,7 +61448,7 @@
         </is>
       </c>
       <c r="D130" t="n">
-        <v>168.058609</v>
+        <v>168.058502</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -61650,7 +61650,7 @@
         </is>
       </c>
       <c r="D137" t="n">
-        <v>3302.944317</v>
+        <v>3302.941356</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -61710,7 +61710,7 @@
         </is>
       </c>
       <c r="D139" t="n">
-        <v>3302.944317</v>
+        <v>3302.941356</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
T03 at scale: P&ID coverage switched to graph-derived - all 174 present non-boundary units (963 edges, 619 valves, 549 instruments across the set); task-03 evidence ticks plant-wide via file-existence detection. EVAP_ACID_VS sector stamp WET->DIGESTER (the ghost-sector exception closed; tree test 178). Suite 43/43; check green.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -120,7 +120,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="12">
+  <cellXfs count="11">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="0" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
@@ -133,7 +133,6 @@
     </xf>
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
-    <xf numFmtId="0" fontId="0" fillId="5" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="164" fontId="1" fillId="2" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
   </cellXfs>
   <cellStyles count="1">
@@ -564,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 c1fd2bec1b943618c9607755b0877923a16474da6cd9ae87a03eff07a08299bb</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 bf8e0f2444c6a4c8237645caaf2f45175ee024ff66edac433c45382b7037c818</t>
         </is>
       </c>
     </row>
@@ -1341,7 +1340,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <f>SUM(B2:B11)</f>
         <v/>
       </c>
@@ -3525,7 +3524,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B20" s="11">
+      <c r="B20" s="10">
         <f>SUM(B2:B18)</f>
         <v/>
       </c>
@@ -5170,7 +5169,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <f>SUM(B2:B11)</f>
         <v/>
       </c>
@@ -7545,7 +7544,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B30" s="11">
+      <c r="B30" s="10">
         <f>SUM(B2:B28)</f>
         <v/>
       </c>
@@ -9320,7 +9319,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <f>SUM(B2:B2)</f>
         <v/>
       </c>
@@ -9822,7 +9821,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <f>SUM(B2:B3)</f>
         <v/>
       </c>
@@ -10537,7 +10536,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B6" s="11">
+      <c r="B6" s="10">
         <f>SUM(B2:B4)</f>
         <v/>
       </c>
@@ -12077,7 +12076,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B17" s="11">
+      <c r="B17" s="10">
         <f>SUM(B2:B15)</f>
         <v/>
       </c>
@@ -14233,7 +14232,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B11" s="11">
+      <c r="B11" s="10">
         <f>SUM(B2:B9)</f>
         <v/>
       </c>
@@ -16143,7 +16142,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B12" s="11">
+      <c r="B12" s="10">
         <f>SUM(B2:B10)</f>
         <v/>
       </c>
@@ -41213,7 +41212,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B15" s="11">
+      <c r="B15" s="10">
         <f>SUM(B2:B13)</f>
         <v/>
       </c>
@@ -43079,7 +43078,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
@@ -43906,7 +43905,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B4" s="11">
+      <c r="B4" s="10">
         <f>SUM(B2:B2)</f>
         <v/>
       </c>
@@ -44172,7 +44171,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B7" s="11">
+      <c r="B7" s="10">
         <f>SUM(B2:B5)</f>
         <v/>
       </c>
@@ -44601,7 +44600,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B5" s="11">
+      <c r="B5" s="10">
         <f>SUM(B2:B3)</f>
         <v/>
       </c>
@@ -57758,7 +57757,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H172"/>
+  <dimension ref="A1:H180"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -57996,9 +57995,9 @@
       <c r="G7" t="b">
         <v>1</v>
       </c>
-      <c r="H7" s="10" t="inlineStr">
-        <is>
-          <t>WET</t>
+      <c r="H7" t="inlineStr">
+        <is>
+          <t>DIGESTER</t>
         </is>
       </c>
     </row>
@@ -58517,7 +58516,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B28" s="11">
+      <c r="B28" s="10">
         <f>SUM(B2:B26)</f>
         <v/>
       </c>
@@ -59778,21 +59777,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IA-EVAP_BASE-COND</t>
+          <t>IA-EVAP_ACID-VENT</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>EVAP_BASE</t>
+          <t>EVAP_ACID</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>BMED_BASE</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>801.8559</v>
+        <v>0.0293</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -59808,21 +59807,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IA-EVAP_BASE-FEED</t>
+          <t>IA-EVAP_BASE-COND</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>EVAP_BASE</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
           <t>BMED_BASE</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>EVAP_BASE</t>
-        </is>
-      </c>
       <c r="D74" t="n">
-        <v>1301.7164</v>
+        <v>801.8559</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -59838,21 +59837,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>IA-EW-01</t>
+          <t>IA-EVAP_BASE-FEED</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>BMED_BASE</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>EW_2</t>
+          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>4139.222213</v>
+        <v>1301.7164</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -59868,21 +59867,21 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>IA-EW-02</t>
+          <t>IA-EW-01</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
         <is>
+          <t>EW_1</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
           <t>EW_2</t>
         </is>
       </c>
-      <c r="C76" t="inlineStr">
-        <is>
-          <t>EW_3</t>
-        </is>
-      </c>
       <c r="D76" t="n">
-        <v>3990.594815</v>
+        <v>4139.222213</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -59898,21 +59897,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>IA-EW-03</t>
+          <t>IA-EW-02</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
+          <t>EW_2</t>
+        </is>
+      </c>
+      <c r="C77" t="inlineStr">
+        <is>
           <t>EW_3</t>
         </is>
       </c>
-      <c r="C77" t="inlineStr">
-        <is>
-          <t>EW_4</t>
-        </is>
-      </c>
       <c r="D77" t="n">
-        <v>3934.805911</v>
+        <v>3990.594815</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -59928,21 +59927,21 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IA-EW-04</t>
+          <t>IA-EW-03</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>EW_3</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>EW_4</t>
         </is>
       </c>
       <c r="D78" t="n">
-        <v>4287.799997</v>
+        <v>3934.805911</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -59958,21 +59957,21 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IA-EW-05</t>
+          <t>IA-EW-04</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
         <is>
-          <t>EW_5</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>EW_6</t>
+          <t>EW_1</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>3909.914016</v>
+        <v>4287.799997</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -59988,21 +59987,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>IA-EW-06</t>
+          <t>IA-EW-05</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
+          <t>EW_5</t>
+        </is>
+      </c>
+      <c r="C80" t="inlineStr">
+        <is>
           <t>EW_6</t>
         </is>
       </c>
-      <c r="C80" t="inlineStr">
-        <is>
-          <t>EW_7</t>
-        </is>
-      </c>
       <c r="D80" t="n">
-        <v>3896.338257</v>
+        <v>3909.914016</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -60018,21 +60017,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IA-EW-07</t>
+          <t>IA-EW-06</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
+          <t>EW_6</t>
+        </is>
+      </c>
+      <c r="C81" t="inlineStr">
+        <is>
           <t>EW_7</t>
         </is>
       </c>
-      <c r="C81" t="inlineStr">
-        <is>
-          <t>EW_8</t>
-        </is>
-      </c>
       <c r="D81" t="n">
-        <v>3719.79104</v>
+        <v>3896.338257</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -60048,21 +60047,21 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IA-EW-08</t>
+          <t>IA-EW-07</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
         <is>
+          <t>EW_7</t>
+        </is>
+      </c>
+      <c r="C82" t="inlineStr">
+        <is>
           <t>EW_8</t>
         </is>
       </c>
-      <c r="C82" t="inlineStr">
-        <is>
-          <t>EW_9</t>
-        </is>
-      </c>
       <c r="D82" t="n">
-        <v>3707.257179</v>
+        <v>3719.79104</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -60078,21 +60077,21 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IA-EW-09</t>
+          <t>IA-EW-08</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
+          <t>EW_8</t>
+        </is>
+      </c>
+      <c r="C83" t="inlineStr">
+        <is>
           <t>EW_9</t>
         </is>
       </c>
-      <c r="C83" t="inlineStr">
-        <is>
-          <t>POLISH_BANK</t>
-        </is>
-      </c>
       <c r="D83" t="n">
-        <v>3520.311349</v>
+        <v>3707.257179</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
@@ -60108,21 +60107,21 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IA-EW-10</t>
+          <t>IA-EW-09</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
         <is>
-          <t>EW_4</t>
+          <t>EW_9</t>
         </is>
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>EW_5</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>3922.373456</v>
+        <v>3520.311349</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
@@ -60138,21 +60137,21 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IA-EW-MET-1</t>
+          <t>IA-EW-10</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>EW_4</t>
         </is>
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>EW_5</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>59.869999</v>
+        <v>3922.373456</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -60168,12 +60167,12 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IA-EW-MET-2</t>
+          <t>IA-EW-MET-1</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
         <is>
-          <t>EW_2</t>
+          <t>EW_1</t>
         </is>
       </c>
       <c r="C86" t="inlineStr">
@@ -60182,7 +60181,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>59.889999</v>
+        <v>59.869999</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -60198,12 +60197,12 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>IA-EW-MET-3</t>
+          <t>IA-EW-MET-2</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
         <is>
-          <t>EW_3</t>
+          <t>EW_2</t>
         </is>
       </c>
       <c r="C87" t="inlineStr">
@@ -60212,7 +60211,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>22.480359</v>
+        <v>59.889999</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -60228,12 +60227,12 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>IA-EW-MET-4</t>
+          <t>IA-EW-MET-3</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
-          <t>EW_4</t>
+          <t>EW_3</t>
         </is>
       </c>
       <c r="C88" t="inlineStr">
@@ -60242,7 +60241,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>4.85</v>
+        <v>22.480359</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -60258,12 +60257,12 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>IA-EW-MET-5</t>
+          <t>IA-EW-MET-4</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>EW_5</t>
+          <t>EW_4</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
@@ -60272,7 +60271,7 @@
         </is>
       </c>
       <c r="D89" t="n">
-        <v>5.020359</v>
+        <v>4.85</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -60288,12 +60287,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>IA-EW-MET-6</t>
+          <t>IA-EW-MET-5</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>EW_6</t>
+          <t>EW_5</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -60302,7 +60301,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>5.470359</v>
+        <v>5.020359</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -60318,12 +60317,12 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>IA-EW-MET-7</t>
+          <t>IA-EW-MET-6</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>EW_7</t>
+          <t>EW_6</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
@@ -60332,7 +60331,7 @@
         </is>
       </c>
       <c r="D91" t="n">
-        <v>71.139999</v>
+        <v>5.470359</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -60348,12 +60347,12 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>IA-EW-MET-8</t>
+          <t>IA-EW-MET-7</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
         <is>
-          <t>EW_8</t>
+          <t>EW_7</t>
         </is>
       </c>
       <c r="C92" t="inlineStr">
@@ -60362,7 +60361,7 @@
         </is>
       </c>
       <c r="D92" t="n">
-        <v>5.050359</v>
+        <v>71.139999</v>
       </c>
       <c r="E92" t="inlineStr">
         <is>
@@ -60378,12 +60377,12 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>IA-EW-MET-9</t>
+          <t>IA-EW-MET-8</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>EW_9</t>
+          <t>EW_8</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
@@ -60392,7 +60391,7 @@
         </is>
       </c>
       <c r="D93" t="n">
-        <v>61.341099</v>
+        <v>5.050359</v>
       </c>
       <c r="E93" t="inlineStr">
         <is>
@@ -60408,7 +60407,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>IA-EW-SHEET</t>
+          <t>IA-EW-MET-9</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -60418,11 +60417,11 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>MET_MELT</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D94" t="n">
-        <v>13.9889</v>
+        <v>61.341099</v>
       </c>
       <c r="E94" t="inlineStr">
         <is>
@@ -60438,21 +60437,21 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>IA-EW1-CL2</t>
+          <t>IA-EW-SHEET</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>EW_9</t>
         </is>
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MET_MELT</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>88.32517</v>
+        <v>13.9889</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -60468,7 +60467,7 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>IA-EW1-H2</t>
+          <t>IA-EW1-CL2</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
@@ -60478,11 +60477,11 @@
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>0</v>
+        <v>88.32517</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -60498,21 +60497,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>IA-EW2-CL2</t>
+          <t>IA-EW1-H2</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>EW_2</t>
+          <t>EW_1</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>88.35465600000001</v>
+        <v>0</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -60528,7 +60527,7 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>IA-EW2-H2</t>
+          <t>IA-EW2-CL2</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
@@ -60538,11 +60537,11 @@
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>0</v>
+        <v>88.35465600000001</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
@@ -60558,21 +60557,21 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>IA-EW3-CL2</t>
+          <t>IA-EW2-H2</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
         <is>
-          <t>EW_3</t>
+          <t>EW_2</t>
         </is>
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>33.164878</v>
+        <v>0</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -60588,7 +60587,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>IA-EW3-H2B</t>
+          <t>IA-EW3-CL2</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -60598,11 +60597,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.143667</v>
+        <v>33.164878</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -60618,21 +60617,21 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>IA-EW4-CL2</t>
+          <t>IA-EW3-H2B</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
         <is>
-          <t>EW_4</t>
+          <t>EW_3</t>
         </is>
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>7.154886</v>
+        <v>0.143667</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -60648,7 +60647,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>IA-EW4-H2</t>
+          <t>IA-EW4-CL2</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -60658,11 +60657,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0.030994</v>
+        <v>7.154886</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -60678,7 +60677,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>IA-EW4-N2</t>
+          <t>IA-EW4-H2</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -60688,11 +60687,11 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>HDR_N2</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D103" t="n">
-        <v>0.396575</v>
+        <v>0.030994</v>
       </c>
       <c r="E103" t="inlineStr">
         <is>
@@ -60708,21 +60707,21 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>IA-EW5-CL2</t>
+          <t>IA-EW4-N2</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
         <is>
-          <t>EW_5</t>
+          <t>EW_4</t>
         </is>
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_N2</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>7.406995</v>
+        <v>0.396575</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -60738,7 +60737,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>IA-EW5-H2B</t>
+          <t>IA-EW5-CL2</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -60748,11 +60747,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0.032086</v>
+        <v>7.406995</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -60768,21 +60767,21 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>IA-EW6-CL2</t>
+          <t>IA-EW5-H2B</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
         <is>
-          <t>EW_6</t>
+          <t>EW_5</t>
         </is>
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>8.07044</v>
+        <v>0.032086</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -60798,7 +60797,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>IA-EW6-H2B</t>
+          <t>IA-EW6-CL2</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -60808,11 +60807,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.03496</v>
+        <v>8.07044</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -60828,21 +60827,21 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>IA-EW7-CL2</t>
+          <t>IA-EW6-H2B</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
         <is>
-          <t>EW_7</t>
+          <t>EW_6</t>
         </is>
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>104.952575</v>
+        <v>0.03496</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -60858,7 +60857,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>IA-EW7-H2B</t>
+          <t>IA-EW7-CL2</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -60868,11 +60867,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.454643</v>
+        <v>104.952575</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -60888,21 +60887,21 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>IA-EW8-CL2</t>
+          <t>IA-EW7-H2B</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
         <is>
-          <t>EW_8</t>
+          <t>EW_7</t>
         </is>
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>7.451224</v>
+        <v>0.454643</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -60918,7 +60917,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>IA-EW8-H2B</t>
+          <t>IA-EW8-CL2</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -60928,11 +60927,11 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D111" t="n">
-        <v>0.032278</v>
+        <v>7.451224</v>
       </c>
       <c r="E111" t="inlineStr">
         <is>
@@ -60948,21 +60947,21 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>IA-EW9-CL2</t>
+          <t>IA-EW8-H2B</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
         <is>
-          <t>EW_9</t>
+          <t>EW_8</t>
         </is>
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>111.134409</v>
+        <v>0.032278</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -60978,12 +60977,12 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>IA-FAB-SPENT</t>
+          <t>IA-EW9-CL2</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>EW_9</t>
         </is>
       </c>
       <c r="C113" t="inlineStr">
@@ -60992,7 +60991,7 @@
         </is>
       </c>
       <c r="D113" t="n">
-        <v>66.502511</v>
+        <v>111.134409</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -61008,12 +61007,12 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>IA-FC-LEACH</t>
+          <t>IA-FAB-SPENT</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C114" t="inlineStr">
@@ -61022,7 +61021,7 @@
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.323377</v>
+        <v>66.502511</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -61038,12 +61037,12 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>IA-FEED-01</t>
+          <t>IA-FC-LEACH</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="C115" t="inlineStr">
@@ -61052,7 +61051,7 @@
         </is>
       </c>
       <c r="D115" t="n">
-        <v>102.680001</v>
+        <v>0.323377</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -61068,12 +61067,12 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>IA-GREY-01</t>
+          <t>IA-FEED-01</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="C116" t="inlineStr">
@@ -61082,7 +61081,7 @@
         </is>
       </c>
       <c r="D116" t="n">
-        <v>244.641602</v>
+        <v>102.680001</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -61098,12 +61097,12 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>IA-H2O-MU</t>
+          <t>IA-GREY-01</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C117" t="inlineStr">
@@ -61112,7 +61111,7 @@
         </is>
       </c>
       <c r="D117" t="n">
-        <v>64.813948</v>
+        <v>244.641602</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -61128,21 +61127,21 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>IA-HDR-H2-01</t>
+          <t>IA-H2O-MU</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D118" t="n">
-        <v>0.382615</v>
+        <v>64.813948</v>
       </c>
       <c r="E118" t="inlineStr">
         <is>
@@ -61158,12 +61157,12 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>IA-HDR-H2-03</t>
+          <t>IA-HDR-H2-01</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
         <is>
-          <t>EW_2</t>
+          <t>EW_1</t>
         </is>
       </c>
       <c r="C119" t="inlineStr">
@@ -61172,7 +61171,7 @@
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.382743</v>
+        <v>0.382615</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -61188,12 +61187,12 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>IA-HDR-H2-04</t>
+          <t>IA-HDR-H2-03</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>EW_9</t>
+          <t>EW_2</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
@@ -61202,7 +61201,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>0.481422</v>
+        <v>0.382743</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -61218,21 +61217,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>IA-HF-SRC</t>
+          <t>IA-HDR-H2-04</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>EW_9</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>WS_HF_ED</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>1.5</v>
+        <v>0.481422</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -61248,21 +61247,21 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>IA-HOP-01</t>
+          <t>IA-HF-SRC</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>WS_HF_ED</t>
         </is>
       </c>
       <c r="D122" t="n">
-        <v>530.73594</v>
+        <v>1.5</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -61278,25 +61277,25 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>IA-HX8</t>
+          <t>IA-HOP-01</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>EW_1</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>HX8</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>4.572</v>
+        <v>530.73594</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F123" t="inlineStr">
@@ -61308,25 +61307,25 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>IA-LEACH-ASU</t>
+          <t>IA-HX8</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>EW_1</t>
         </is>
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>HX8</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>0</v>
+        <v>4.572</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F124" t="inlineStr">
@@ -61338,7 +61337,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>IA-LEACH-BD</t>
+          <t>IA-LEACH-ASU</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -61348,11 +61347,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>109.63</v>
+        <v>0</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -61368,7 +61367,7 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>IA-LEACH-FLUE</t>
+          <t>IA-LEACH-BD</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
@@ -61378,11 +61377,11 @@
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>FLUE_KO</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="D126" t="n">
-        <v>135.9019</v>
+        <v>109.63</v>
       </c>
       <c r="E126" t="inlineStr">
         <is>
@@ -61398,7 +61397,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>IA-LEACH-H2</t>
+          <t>IA-LEACH-FLUE</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -61408,11 +61407,11 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>FLUE_KO</t>
         </is>
       </c>
       <c r="D127" t="n">
-        <v>0</v>
+        <v>135.9019</v>
       </c>
       <c r="E127" t="inlineStr">
         <is>
@@ -61428,7 +61427,7 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>IA-LEACH-HOP</t>
+          <t>IA-LEACH-H2</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
@@ -61438,11 +61437,11 @@
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>35.355</v>
+        <v>0</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
@@ -61458,7 +61457,7 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>IA-LEACH-NOX</t>
+          <t>IA-LEACH-HOP</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
@@ -61468,11 +61467,11 @@
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>195.024701</v>
+        <v>35.355</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
@@ -61488,7 +61487,7 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>IA-LEACH-VCD</t>
+          <t>IA-LEACH-NOX</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
@@ -61498,11 +61497,11 @@
       </c>
       <c r="C130" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>NOX_SCRUB</t>
         </is>
       </c>
       <c r="D130" t="n">
-        <v>168.058502</v>
+        <v>195.024701</v>
       </c>
       <c r="E130" t="inlineStr">
         <is>
@@ -61518,7 +61517,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>IA-NA-PURGE</t>
+          <t>IA-LEACH-VCD</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -61528,11 +61527,11 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D131" t="n">
-        <v>4.3936</v>
+        <v>168.058502</v>
       </c>
       <c r="E131" t="inlineStr">
         <is>
@@ -61548,17 +61547,17 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>IA-NAOH-MU</t>
+          <t>IA-NA-PURGE</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="C132" t="inlineStr">
+        <is>
           <t>NORTH_DOCK</t>
-        </is>
-      </c>
-      <c r="C132" t="inlineStr">
-        <is>
-          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="D132" t="n">
@@ -61578,21 +61577,21 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>IA-NUT-LEACH</t>
+          <t>IA-NAOH-MU</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>82.317318</v>
+        <v>4.3936</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -61608,21 +61607,21 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
-          <t>IA-PHOS-SRC</t>
+          <t>IA-NUT-LEACH</t>
         </is>
       </c>
       <c r="B134" t="inlineStr">
         <is>
+          <t>NUTRIENT_DOSE</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
-        <is>
-          <t>WS_PHOS</t>
-        </is>
-      </c>
       <c r="D134" t="n">
-        <v>0.62</v>
+        <v>82.317318</v>
       </c>
       <c r="E134" t="inlineStr">
         <is>
@@ -61638,21 +61637,21 @@
     <row r="135">
       <c r="A135" t="inlineStr">
         <is>
-          <t>IA-PLAST-01</t>
+          <t>IA-PHOS-SRC</t>
         </is>
       </c>
       <c r="B135" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C135" t="inlineStr">
         <is>
-          <t>OIL_DRYER</t>
+          <t>WS_PHOS</t>
         </is>
       </c>
       <c r="D135" t="n">
-        <v>33</v>
+        <v>0.62</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -61668,29 +61667,37 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IA-POL-01</t>
+          <t>IA-PLAST-01</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>OIL_DRYER</t>
+        </is>
+      </c>
+      <c r="D136" t="n">
+        <v>33</v>
+      </c>
+      <c r="E136" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F136" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>IA-POL-02</t>
+          <t>IA-POL-01</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
@@ -61700,27 +61707,19 @@
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>CONTINUOUS_RECYCLE</t>
-        </is>
-      </c>
-      <c r="D137" t="n">
-        <v>3302.941356</v>
-      </c>
-      <c r="E137" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="F137" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>IA-POL-CAKE</t>
+          <t>IA-POL-02</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -61730,11 +61729,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>CONTINUOUS_RECYCLE</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>217.369993</v>
+        <v>3302.941356</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -61750,21 +61749,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IA-REC-01</t>
+          <t>IA-POL-CAKE</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
-          <t>CONTINUOUS_RECYCLE</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="C139" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D139" t="n">
-        <v>3302.941356</v>
+        <v>217.369993</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -61780,21 +61779,21 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>IA-SCRUB-SRC</t>
+          <t>IA-REC-01</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
         <is>
+          <t>CONTINUOUS_RECYCLE</t>
+        </is>
+      </c>
+      <c r="C140" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C140" t="inlineStr">
-        <is>
-          <t>ACID_POLISH_SCRUB</t>
-        </is>
-      </c>
       <c r="D140" t="n">
-        <v>27.342833</v>
+        <v>3302.941356</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -61810,21 +61809,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IA-SIC-RET</t>
+          <t>IA-SCRUB-SRC</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ACID_POLISH_SCRUB</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.466189</v>
+        <v>27.342833</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -61840,21 +61839,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IA-SINK-01</t>
+          <t>IA-SIC-RET</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
+          <t>NUTRIENT_DOSE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>FLOAT_SINK</t>
-        </is>
-      </c>
       <c r="D142" t="n">
-        <v>376.1</v>
+        <v>0.466189</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -61870,25 +61869,25 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>IA-TRIM-HX5</t>
+          <t>IA-SINK-01</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>RECTIFIER</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="D143" t="n">
-        <v>15.882</v>
+        <v>376.1</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F143" t="inlineStr">
@@ -61900,12 +61899,12 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>IA-UPW-REJ</t>
+          <t>IA-TRIM-HX5</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>RECTIFIER</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
@@ -61914,11 +61913,11 @@
         </is>
       </c>
       <c r="D144" t="n">
-        <v>6.045005</v>
+        <v>15.882</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F144" t="inlineStr">
@@ -61930,12 +61929,12 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IA-VCD-BD</t>
+          <t>IA-UPW-REJ</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C145" t="inlineStr">
@@ -61944,7 +61943,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>6.709424</v>
+        <v>6.045005</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -61960,12 +61959,12 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IA-WET-FLOAT-01</t>
+          <t>IA-VCD-BD</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
@@ -61974,7 +61973,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>343.1</v>
+        <v>6.709424</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -61990,21 +61989,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>IA-ZNBR-MU</t>
+          <t>IA-VS-NAOH</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BMED_BASE</t>
         </is>
       </c>
       <c r="C147" t="inlineStr">
         <is>
-          <t>ZNBR2</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="D147" t="n">
-        <v>8.486482000000001</v>
+        <v>0.0005</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -62020,43 +62019,51 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>LI_TO_GREASE</t>
+          <t>IA-VS-OFF</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>LI_RECOVER</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>GREASE_LI</t>
+          <t>ALK_SCRUBBER</t>
+        </is>
+      </c>
+      <c r="D148" t="n">
+        <v>0.0292</v>
+      </c>
+      <c r="E148" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F148" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>MG_POT_CL2</t>
+          <t>IA-VS-SPENT</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="D149" t="n">
-        <v>0</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E149" t="inlineStr">
         <is>
@@ -62072,21 +62079,21 @@
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
+          <t>IA-WET-FLOAT-01</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D150" t="n">
-        <v>0</v>
+        <v>343.1</v>
       </c>
       <c r="E150" t="inlineStr">
         <is>
@@ -62102,21 +62109,21 @@
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>MO_CELL_RAFFINATE</t>
+          <t>IA-ZNBR-MU</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>ZNBR2</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>0</v>
+        <v>8.486482000000001</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -62132,17 +62139,17 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>PCA_TO_GREASE</t>
+          <t>LI_TO_GREASE</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>P_CA</t>
+          <t>LI_RECOVER</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>GREASE_CA</t>
+          <t>GREASE_LI</t>
         </is>
       </c>
       <c r="F152" t="inlineStr">
@@ -62154,43 +62161,51 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>POLISH_TO_LI</t>
+          <t>MG_POT_CL2</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="C153" t="inlineStr">
         <is>
-          <t>LI_RECOVER</t>
+          <t>CRU</t>
+        </is>
+      </c>
+      <c r="D153" t="n">
+        <v>0</v>
+      </c>
+      <c r="E153" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F153" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>POLY_TO_WET</t>
+          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>POLY_STOCK</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.037719</v>
+        <v>0</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -62206,21 +62221,21 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>MO_CELL_RAFFINATE</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="D155" t="n">
-        <v>41.996408</v>
+        <v>0</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -62236,72 +62251,56 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>PCA_TO_GREASE</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>P_CA</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
-        </is>
-      </c>
-      <c r="D156" t="n">
-        <v>9.277184</v>
-      </c>
-      <c r="E156" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREASE_CA</t>
         </is>
       </c>
       <c r="F156" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>POLISH_TO_LI</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="C157" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
-      <c r="D157" t="n">
-        <v>79.11577699999999</v>
-      </c>
-      <c r="E157" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>LI_RECOVER</t>
         </is>
       </c>
       <c r="F157" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>S100</t>
+          <t>POLY_TO_WET</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
@@ -62310,11 +62309,11 @@
         </is>
       </c>
       <c r="D158" t="n">
-        <v>0.5322</v>
+        <v>0.037719</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -62326,21 +62325,21 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>S16</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="C159" t="inlineStr">
+        <is>
           <t>MFG_SHOP</t>
         </is>
       </c>
-      <c r="C159" t="inlineStr">
-        <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
       <c r="D159" t="n">
-        <v>12.299499</v>
+        <v>41.996408</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
@@ -62356,25 +62355,25 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>S17-BMED</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>5.6267</v>
+        <v>9.277184</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F160" t="inlineStr">
@@ -62386,12 +62385,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>S19</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>BAGHOUSE</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -62400,7 +62399,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0</v>
+        <v>79.11577699999999</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -62416,12 +62415,12 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>S28</t>
+          <t>S100</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
@@ -62430,11 +62429,11 @@
         </is>
       </c>
       <c r="D162" t="n">
-        <v>17.877059</v>
+        <v>0.5322</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F162" t="inlineStr">
@@ -62446,12 +62445,12 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="C163" t="inlineStr">
@@ -62460,7 +62459,7 @@
         </is>
       </c>
       <c r="D163" t="n">
-        <v>3.310001</v>
+        <v>12.299499</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -62476,25 +62475,25 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>S66</t>
+          <t>S17-BMED</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
         <is>
-          <t>ACID_POLISH_SCRUB</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>27.372033</v>
+        <v>5.6267</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F164" t="inlineStr">
@@ -62506,12 +62505,12 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>S68</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>BAGHOUSE</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
@@ -62520,7 +62519,7 @@
         </is>
       </c>
       <c r="D165" t="n">
-        <v>78.98790099999999</v>
+        <v>0</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -62536,12 +62535,12 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>S72</t>
+          <t>S28</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
-          <t>MET_SCRUB</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C166" t="inlineStr">
@@ -62550,7 +62549,7 @@
         </is>
       </c>
       <c r="D166" t="n">
-        <v>2.4442</v>
+        <v>17.877059</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -62566,21 +62565,21 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>SALT_TO_FLUX</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>SALT_FEED</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D167" t="n">
-        <v>0</v>
+        <v>3.310001</v>
       </c>
       <c r="E167" t="inlineStr">
         <is>
@@ -62596,25 +62595,25 @@
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>SF-EVAP_ACID</t>
+          <t>S66</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>ACID_POLISH_SCRUB</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>EVAP_ACID</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D168" t="n">
-        <v>1.498</v>
+        <v>27.372033</v>
       </c>
       <c r="E168" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
@@ -62626,25 +62625,25 @@
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>SF-EVAP_BASE</t>
+          <t>S68</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
         <is>
-          <t>EVAP_BASE</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D169" t="n">
-        <v>1.328</v>
+        <v>78.98790099999999</v>
       </c>
       <c r="E169" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F169" t="inlineStr">
@@ -62656,12 +62655,12 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>SF-LEACH_CSTR_1</t>
+          <t>S72</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>MET_SCRUB</t>
         </is>
       </c>
       <c r="C170" t="inlineStr">
@@ -62670,11 +62669,11 @@
         </is>
       </c>
       <c r="D170" t="n">
-        <v>0.75</v>
+        <v>2.4442</v>
       </c>
       <c r="E170" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F170" t="inlineStr">
@@ -62686,17 +62685,17 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>TI_CELL_CL2_TO_CRU</t>
+          <t>SALT_TO_FLUX</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>SALT_FEED</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>FLUX_PREP</t>
         </is>
       </c>
       <c r="D171" t="n">
@@ -62716,28 +62715,268 @@
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
+          <t>SF-EVAP_ACID</t>
+        </is>
+      </c>
+      <c r="B172" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C172" t="inlineStr">
+        <is>
+          <t>EVAP_ACID</t>
+        </is>
+      </c>
+      <c r="D172" t="n">
+        <v>1.498</v>
+      </c>
+      <c r="E172" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F172" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="173">
+      <c r="A173" t="inlineStr">
+        <is>
+          <t>SF-EVAP_ACID_VS</t>
+        </is>
+      </c>
+      <c r="B173" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C173" t="inlineStr">
+        <is>
+          <t>EVAP_ACID_VS</t>
+        </is>
+      </c>
+      <c r="D173" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="E173" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F173" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="174">
+      <c r="A174" t="inlineStr">
+        <is>
+          <t>SF-EVAP_BASE</t>
+        </is>
+      </c>
+      <c r="B174" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C174" t="inlineStr">
+        <is>
+          <t>EVAP_BASE</t>
+        </is>
+      </c>
+      <c r="D174" t="n">
+        <v>1.328</v>
+      </c>
+      <c r="E174" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F174" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="175">
+      <c r="A175" t="inlineStr">
+        <is>
+          <t>SF-LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="B175" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="D175" t="n">
+        <v>0.75</v>
+      </c>
+      <c r="E175" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F175" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="176">
+      <c r="A176" t="inlineStr">
+        <is>
+          <t>SQ-EVAP_ACID</t>
+        </is>
+      </c>
+      <c r="B176" t="inlineStr">
+        <is>
+          <t>EVAP_ACID</t>
+        </is>
+      </c>
+      <c r="C176" t="inlineStr">
+        <is>
+          <t>HEAT_SINK</t>
+        </is>
+      </c>
+      <c r="D176" t="n">
+        <v>1.498</v>
+      </c>
+      <c r="E176" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F176" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="177">
+      <c r="A177" t="inlineStr">
+        <is>
+          <t>SQ-EVAP_ACID_VS</t>
+        </is>
+      </c>
+      <c r="B177" t="inlineStr">
+        <is>
+          <t>EVAP_ACID_VS</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
+          <t>HEAT_SINK</t>
+        </is>
+      </c>
+      <c r="D177" t="n">
+        <v>0.0238</v>
+      </c>
+      <c r="E177" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F177" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="178">
+      <c r="A178" t="inlineStr">
+        <is>
+          <t>SQ-EVAP_BASE</t>
+        </is>
+      </c>
+      <c r="B178" t="inlineStr">
+        <is>
+          <t>EVAP_BASE</t>
+        </is>
+      </c>
+      <c r="C178" t="inlineStr">
+        <is>
+          <t>HEAT_SINK</t>
+        </is>
+      </c>
+      <c r="D178" t="n">
+        <v>1.328</v>
+      </c>
+      <c r="E178" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F178" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="179">
+      <c r="A179" t="inlineStr">
+        <is>
+          <t>TI_CELL_CL2_TO_CRU</t>
+        </is>
+      </c>
+      <c r="B179" t="inlineStr">
+        <is>
+          <t>TI_CELL</t>
+        </is>
+      </c>
+      <c r="C179" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
+      <c r="D179" t="n">
+        <v>0</v>
+      </c>
+      <c r="E179" t="inlineStr">
+        <is>
+          <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F179" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="180">
+      <c r="A180" t="inlineStr">
+        <is>
           <t>TI_CELL_SLAG_RETURN</t>
         </is>
       </c>
-      <c r="B172" t="inlineStr">
+      <c r="B180" t="inlineStr">
         <is>
           <t>TI_CELL</t>
         </is>
       </c>
-      <c r="C172" t="inlineStr">
+      <c r="C180" t="inlineStr">
         <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="D172" t="n">
+      <c r="D180" t="n">
         <v>0</v>
       </c>
-      <c r="E172" t="inlineStr">
+      <c r="E180" t="inlineStr">
         <is>
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F172" t="inlineStr">
+      <c r="F180" t="inlineStr">
         <is>
           <t>study</t>
         </is>
@@ -63167,7 +63406,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B16" s="11">
+      <c r="B16" s="10">
         <f>SUM(B2:B14)</f>
         <v/>
       </c>
@@ -64806,7 +65045,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B8" s="11">
+      <c r="B8" s="10">
         <f>SUM(B2:B6)</f>
         <v/>
       </c>
@@ -65740,7 +65979,7 @@
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B13" s="11">
+      <c r="B13" s="10">
         <f>SUM(B2:B11)</f>
         <v/>
       </c>

</xml_diff>

<commit_message>
Generator templates and source data free of working jargon
Text that generators write, and the data they read, no longer use the banned
terms of DOC_STYLE (AQS-DOC-002):

- DERIVED_REVISIONS rows read 'regenerated, no change'; the media manifest
  row says what the manifest is.
- Work orders written by models/mfg/foundry.py and polymers.py say which
  stream is connected instead of 'landed'.
- Duty sheets say the STL is the outer envelope only and nothing inside it is
  modelled yet (worded so the internals register does not read it as a
  basis).
- 're-derived' becomes 'derived again' in generators, graph notes and the
  assumptions data; assumption task labels and notes drop 'lane', 'wave'
  and who asked.
- Pack export, PFD label, insulation and FreeCAD docstrings reworded.

Pages that are now clean are removed from the pending list.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 8f5733d774593ecaaf06d17bf01fb43b70529b6b6b78f803488da3498e90b6f1</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 180a5b333e041348b5a4cea18b4a3ff4e231255fd7049bb9761faeb787887bb2</t>
         </is>
       </c>
     </row>
@@ -63218,7 +63218,7 @@
     <row r="11">
       <c r="A11" s="7" t="inlineStr">
         <is>
-          <t>write_graph power() (single writer, D1/D2/D4): need/target/PV/storage chain re-derived per A-M-234 replaced_by / A-M-258 from docs-authority/_power_sizing.py (demand = max(node continuous_kw, SOL_ARK feed) + RECT-EW bounding AC, A-M-231) and solver.roof_close; pv_module_kw x pv_count = PV_ARRAY.params.nameplate_kw; znbr_* = the SOL_ARK hybrid-inverter block the ZNBR2 store is distributed over; rect_count = the single nine-channel RECTIFIER (Rev AC; RECT_EW remap, A-M-255).</t>
+          <t>write_graph power() (single writer, D1/D2/D4): need/target/PV/storage chain derived again per A-M-234 replaced_by / A-M-258 from docs-authority/_power_sizing.py (demand = max(node continuous_kw, SOL_ARK feed) + RECT-EW bounding AC, A-M-231) and solver.roof_close; pv_module_kw x pv_count = PV_ARRAY.params.nameplate_kw; znbr_* = the SOL_ARK hybrid-inverter block the ZNBR2 store is distributed over; rect_count = the single nine-channel RECTIFIER (Rev AC; RECT_EW remap, A-M-255).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Code editions: latest published edition of every standard (Q-018 closed by the owner); CODE_BASIS Table 3.1 is the single edition source, test_code_editions.py rejects any other edition; edition-bearing reference keys renamed; clauses carried from earlier editions recorded as assumptions A-M-333 onward
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 180a5b333e041348b5a4cea18b4a3ff4e231255fd7049bb9761faeb787887bb2</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 9bffd7c81c83fa7e8acb973528cc08647f5bd03a58fea6dcfd338168c2f9bb87</t>
         </is>
       </c>
     </row>
@@ -26596,7 +26596,7 @@
       </c>
       <c r="D120" t="inlineStr">
         <is>
-          <t>NEC2023</t>
+          <t>NEC2026</t>
         </is>
       </c>
       <c r="H120" t="inlineStr">
@@ -26680,7 +26680,7 @@
       </c>
       <c r="D122" t="inlineStr">
         <is>
-          <t>NEC2023_240</t>
+          <t>NEC2026_240</t>
         </is>
       </c>
       <c r="H122" t="inlineStr">
@@ -27240,7 +27240,7 @@
       </c>
       <c r="D137" t="inlineStr">
         <is>
-          <t>NFPA110_2022</t>
+          <t>NFPA110_2025</t>
         </is>
       </c>
       <c r="H137" t="inlineStr">
@@ -27280,7 +27280,7 @@
       </c>
       <c r="D138" t="inlineStr">
         <is>
-          <t>NFPA110_2022</t>
+          <t>NFPA110_2025</t>
         </is>
       </c>
       <c r="H138" t="inlineStr">
@@ -27360,7 +27360,7 @@
       </c>
       <c r="D140" t="inlineStr">
         <is>
-          <t>NFPA69_2019</t>
+          <t>NFPA69_2024</t>
         </is>
       </c>
       <c r="H140" t="inlineStr">
@@ -37497,7 +37497,7 @@
       </c>
       <c r="D404" t="inlineStr">
         <is>
-          <t>NFPA110_2022</t>
+          <t>NFPA110_2025</t>
         </is>
       </c>
       <c r="F404" t="b">
@@ -38691,7 +38691,7 @@
       </c>
       <c r="D453" t="inlineStr">
         <is>
-          <t>NEC2023</t>
+          <t>NEC2026</t>
         </is>
       </c>
     </row>
@@ -40623,7 +40623,7 @@
       </c>
       <c r="D525" t="inlineStr">
         <is>
-          <t>NFPA13_2022</t>
+          <t>NFPA13_2025</t>
         </is>
       </c>
     </row>
@@ -40645,7 +40645,7 @@
       </c>
       <c r="D526" t="inlineStr">
         <is>
-          <t>NFPA13_2022</t>
+          <t>NFPA13_2025</t>
         </is>
       </c>
     </row>
@@ -40667,7 +40667,7 @@
       </c>
       <c r="D527" t="inlineStr">
         <is>
-          <t>NFPA13_2022</t>
+          <t>NFPA13_2025</t>
         </is>
       </c>
     </row>
@@ -40687,7 +40687,7 @@
       </c>
       <c r="D528" t="inlineStr">
         <is>
-          <t>NFPA20_2022</t>
+          <t>NFPA20_2025</t>
         </is>
       </c>
     </row>
@@ -40707,7 +40707,7 @@
       </c>
       <c r="D529" t="inlineStr">
         <is>
-          <t>NFPA20_2022</t>
+          <t>NFPA20_2025</t>
         </is>
       </c>
     </row>
@@ -40727,7 +40727,7 @@
       </c>
       <c r="D530" t="inlineStr">
         <is>
-          <t>NFPA20_2022</t>
+          <t>NFPA20_2025</t>
         </is>
       </c>
     </row>
@@ -40777,7 +40777,7 @@
       </c>
       <c r="D532" t="inlineStr">
         <is>
-          <t>NFPA20_2022</t>
+          <t>NFPA20_2025</t>
         </is>
       </c>
     </row>
@@ -40869,7 +40869,7 @@
       </c>
       <c r="D536" t="inlineStr">
         <is>
-          <t>NFPA13_2022</t>
+          <t>NFPA13_2025</t>
         </is>
       </c>
     </row>
@@ -41558,7 +41558,7 @@
       </c>
       <c r="D562" t="inlineStr">
         <is>
-          <t>NFPA69_2019</t>
+          <t>NFPA69_2024</t>
         </is>
       </c>
     </row>
@@ -42628,7 +42628,7 @@
       </c>
       <c r="D605" t="inlineStr">
         <is>
-          <t>IFC2021_1205</t>
+          <t>IFC2027_1205</t>
         </is>
       </c>
       <c r="F605" t="b">
@@ -42656,7 +42656,7 @@
       </c>
       <c r="D606" t="inlineStr">
         <is>
-          <t>IFC2021_1205</t>
+          <t>IFC2027_1205</t>
         </is>
       </c>
       <c r="F606" t="b">
@@ -42684,7 +42684,7 @@
       </c>
       <c r="D607" t="inlineStr">
         <is>
-          <t>IFC2021_1205</t>
+          <t>IFC2027_1205</t>
         </is>
       </c>
       <c r="F607" t="b">
@@ -42712,7 +42712,7 @@
       </c>
       <c r="D608" t="inlineStr">
         <is>
-          <t>IFC2021_1205</t>
+          <t>IFC2027_1205</t>
         </is>
       </c>
       <c r="F608" t="b">
@@ -42740,7 +42740,7 @@
       </c>
       <c r="D609" t="inlineStr">
         <is>
-          <t>IFC2021_1205</t>
+          <t>IFC2027_1205</t>
         </is>
       </c>
       <c r="F609" t="b">
@@ -46693,7 +46693,7 @@
       </c>
       <c r="D774" t="inlineStr">
         <is>
-          <t>NEC2023_240</t>
+          <t>NEC2026_240</t>
         </is>
       </c>
       <c r="F774" t="b">
@@ -46764,7 +46764,7 @@
       </c>
       <c r="D777" t="inlineStr">
         <is>
-          <t>IBC2021_1806</t>
+          <t>IBC2027_1806</t>
         </is>
       </c>
       <c r="F777" t="b">

</xml_diff>

<commit_message>
Regenerate outputs for profile gravity and air density (Q-032)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 07baa51a068d02113977edac6338b19d56d0f4048a03bbf3001ce3c259774160</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 ed22ff1bb3835551b4aa1d64459cb688a3688229d7ac1f18f05386b0cb165366</t>
         </is>
       </c>
     </row>
@@ -1039,7 +1039,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -1102,7 +1102,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -3021,7 +3021,7 @@
         </is>
       </c>
       <c r="D71" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -3051,7 +3051,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -5443,7 +5443,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>2.1234</v>
+        <v>2.1232</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -7131,7 +7131,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>2.1234</v>
+        <v>2.1232</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -17946,7 +17946,7 @@
         </is>
       </c>
       <c r="B6" s="8" t="n">
-        <v>336.8121</v>
+        <v>336.8116</v>
       </c>
       <c r="C6" t="inlineStr">
         <is>
@@ -18047,7 +18047,7 @@
         </is>
       </c>
       <c r="B9" s="8" t="n">
-        <v>179.7338</v>
+        <v>179.7238</v>
       </c>
       <c r="C9" t="inlineStr">
         <is>
@@ -18732,7 +18732,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>336.8121</v>
+        <v>336.8116</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -19414,7 +19414,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>752.788322</v>
+        <v>755.229337</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -19444,7 +19444,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>752.788322</v>
+        <v>755.229337</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -19504,7 +19504,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -19534,7 +19534,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -20254,7 +20254,7 @@
         </is>
       </c>
       <c r="D86" t="n">
-        <v>0.1258</v>
+        <v>0.1257</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -20704,7 +20704,7 @@
         </is>
       </c>
       <c r="D101" t="n">
-        <v>2.1234</v>
+        <v>2.1232</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -27467,20 +27467,28 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>ELEC.storage-train.ZNBR2.purge_air_rho_kg_m3</t>
+          <t>ELEC.storage-train.ZNBR2.purge_air_T_C</t>
         </is>
       </c>
       <c r="B143" s="4" t="n">
-        <v>1.18</v>
+        <v>25</v>
       </c>
       <c r="C143" t="inlineStr">
         <is>
-          <t>kg/m3 purge air density</t>
+          <t>C purge air temperature</t>
         </is>
       </c>
       <c r="E143" t="inlineStr">
         <is>
-          <t>A-M-135 (X-PAR-02 ZNBR2 purge basis)</t>
+          <t>A-M-384</t>
+        </is>
+      </c>
+      <c r="F143" t="b">
+        <v>1</v>
+      </c>
+      <c r="G143" t="inlineStr">
+        <is>
+          <t>Compare with the HVAC design room and line temperatures</t>
         </is>
       </c>
       <c r="H143" t="inlineStr">
@@ -27500,7 +27508,7 @@
       </c>
       <c r="K143" t="inlineStr">
         <is>
-          <t>purge_air_rho_kg_m3</t>
+          <t>purge_air_T_C</t>
         </is>
       </c>
     </row>
@@ -31521,20 +31529,28 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_cp_water_kJ_kgK</t>
+          <t>HDR.headers-train.hdr_air_T_C</t>
         </is>
       </c>
       <c r="B241" s="4" t="n">
-        <v>4.186</v>
+        <v>20</v>
       </c>
       <c r="C241" t="inlineStr">
         <is>
-          <t>kJ/kg K water</t>
-        </is>
-      </c>
-      <c r="D241" t="inlineStr">
-        <is>
-          <t>IAPWS_IF97</t>
+          <t>C air / N2 class gas temperature for header density</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>A-M-384</t>
+        </is>
+      </c>
+      <c r="F241" t="b">
+        <v>1</v>
+      </c>
+      <c r="G241" t="inlineStr">
+        <is>
+          <t>Compare with the HVAC design room and line temperatures</t>
         </is>
       </c>
       <c r="H241" t="inlineStr">
@@ -31549,35 +31565,27 @@
       </c>
       <c r="J241" t="inlineStr">
         <is>
-          <t>hdr_cp_water_kJ_kgK</t>
+          <t>hdr_air_T_C</t>
         </is>
       </c>
     </row>
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_min_DN_flue</t>
+          <t>HDR.headers-train.hdr_cp_water_kJ_kgK</t>
         </is>
       </c>
       <c r="B242" s="4" t="n">
-        <v>100</v>
+        <v>4.186</v>
       </c>
       <c r="C242" t="inlineStr">
         <is>
-          <t>DN minimum, afterburner flue</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>A-M-304</t>
-        </is>
-      </c>
-      <c r="F242" t="b">
-        <v>1</v>
-      </c>
-      <c r="G242" t="inlineStr">
-        <is>
-          <t>Natural-draft and condensate-drainage check on the flue routing drawing</t>
+          <t>kJ/kg K water</t>
+        </is>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>IAPWS_IF97</t>
         </is>
       </c>
       <c r="H242" t="inlineStr">
@@ -31592,27 +31600,27 @@
       </c>
       <c r="J242" t="inlineStr">
         <is>
-          <t>hdr_min_DN_flue</t>
+          <t>hdr_cp_water_kJ_kgK</t>
         </is>
       </c>
     </row>
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_min_DN_gas</t>
+          <t>HDR.headers-train.hdr_min_DN_flue</t>
         </is>
       </c>
       <c r="B243" s="4" t="n">
-        <v>25</v>
+        <v>100</v>
       </c>
       <c r="C243" t="inlineStr">
         <is>
-          <t>DN minimum, gas headers</t>
+          <t>DN minimum, afterburner flue</t>
         </is>
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>A-M-303</t>
+          <t>A-M-304</t>
         </is>
       </c>
       <c r="F243" t="b">
@@ -31620,7 +31628,7 @@
       </c>
       <c r="G243" t="inlineStr">
         <is>
-          <t>Take-off and instrument tapping check on the header GA at unit task 05</t>
+          <t>Natural-draft and condensate-drainage check on the flue routing drawing</t>
         </is>
       </c>
       <c r="H243" t="inlineStr">
@@ -31635,14 +31643,14 @@
       </c>
       <c r="J243" t="inlineStr">
         <is>
-          <t>hdr_min_DN_gas</t>
+          <t>hdr_min_DN_flue</t>
         </is>
       </c>
     </row>
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_min_DN_water</t>
+          <t>HDR.headers-train.hdr_min_DN_gas</t>
         </is>
       </c>
       <c r="B244" s="4" t="n">
@@ -31650,7 +31658,7 @@
       </c>
       <c r="C244" t="inlineStr">
         <is>
-          <t>DN minimum, water headers</t>
+          <t>DN minimum, gas headers</t>
         </is>
       </c>
       <c r="E244" t="inlineStr">
@@ -31658,6 +31666,14 @@
           <t>A-M-303</t>
         </is>
       </c>
+      <c r="F244" t="b">
+        <v>1</v>
+      </c>
+      <c r="G244" t="inlineStr">
+        <is>
+          <t>Take-off and instrument tapping check on the header GA at unit task 05</t>
+        </is>
+      </c>
       <c r="H244" t="inlineStr">
         <is>
           <t>HDR</t>
@@ -31670,27 +31686,27 @@
       </c>
       <c r="J244" t="inlineStr">
         <is>
-          <t>hdr_min_DN_water</t>
+          <t>hdr_min_DN_gas</t>
         </is>
       </c>
     </row>
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_rho_CO2</t>
+          <t>HDR.headers-train.hdr_min_DN_water</t>
         </is>
       </c>
       <c r="B245" s="4" t="n">
-        <v>1.84</v>
+        <v>25</v>
       </c>
       <c r="C245" t="inlineStr">
         <is>
-          <t>kg/m3 CO2 at 20 C 1 atm</t>
-        </is>
-      </c>
-      <c r="D245" t="inlineStr">
-        <is>
-          <t>NIST_WEBBOOK</t>
+          <t>DN minimum, water headers</t>
+        </is>
+      </c>
+      <c r="E245" t="inlineStr">
+        <is>
+          <t>A-M-303</t>
         </is>
       </c>
       <c r="H245" t="inlineStr">
@@ -31705,22 +31721,22 @@
       </c>
       <c r="J245" t="inlineStr">
         <is>
-          <t>hdr_rho_CO2</t>
+          <t>hdr_min_DN_water</t>
         </is>
       </c>
     </row>
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_rho_H2</t>
+          <t>HDR.headers-train.hdr_rho_CO2</t>
         </is>
       </c>
       <c r="B246" s="4" t="n">
-        <v>0.08400000000000001</v>
+        <v>1.84</v>
       </c>
       <c r="C246" t="inlineStr">
         <is>
-          <t>kg/m3 hydrogen at 20 C 1 atm</t>
+          <t>kg/m3 CO2 at 20 C 1 atm</t>
         </is>
       </c>
       <c r="D246" t="inlineStr">
@@ -31740,22 +31756,22 @@
       </c>
       <c r="J246" t="inlineStr">
         <is>
-          <t>hdr_rho_H2</t>
+          <t>hdr_rho_CO2</t>
         </is>
       </c>
     </row>
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>HDR.headers-train.hdr_rho_air</t>
+          <t>HDR.headers-train.hdr_rho_H2</t>
         </is>
       </c>
       <c r="B247" s="4" t="n">
-        <v>1.2</v>
+        <v>0.08400000000000001</v>
       </c>
       <c r="C247" t="inlineStr">
         <is>
-          <t>kg/m3 air / N2 class at 20 C</t>
+          <t>kg/m3 hydrogen at 20 C 1 atm</t>
         </is>
       </c>
       <c r="D247" t="inlineStr">
@@ -31775,7 +31791,7 @@
       </c>
       <c r="J247" t="inlineStr">
         <is>
-          <t>hdr_rho_air</t>
+          <t>hdr_rho_H2</t>
         </is>
       </c>
     </row>
@@ -35789,20 +35805,28 @@
     <row r="351">
       <c r="A351" t="inlineStr">
         <is>
-          <t>WTR.grey-black-train.san_air_rho20_kg_m3</t>
+          <t>WTR.grey-black-train.san_air_T_C</t>
         </is>
       </c>
       <c r="B351" s="4" t="n">
-        <v>1.2</v>
+        <v>20</v>
       </c>
       <c r="C351" t="inlineStr">
         <is>
-          <t>kg/m3 air density at 20 C (flue and vent superficials)</t>
+          <t>C reference air temperature for the NOX_SCRUB superficial</t>
         </is>
       </c>
       <c r="E351" t="inlineStr">
         <is>
-          <t>A-M-118</t>
+          <t>A-M-384</t>
+        </is>
+      </c>
+      <c r="F351" t="b">
+        <v>1</v>
+      </c>
+      <c r="G351" t="inlineStr">
+        <is>
+          <t>Compare with the HVAC design room and line temperatures</t>
         </is>
       </c>
       <c r="H351" t="inlineStr">
@@ -35817,7 +35841,7 @@
       </c>
       <c r="J351" t="inlineStr">
         <is>
-          <t>san_air_rho20_kg_m3</t>
+          <t>san_air_T_C</t>
         </is>
       </c>
     </row>
@@ -51590,7 +51614,7 @@
         </is>
       </c>
       <c r="B4" s="8" t="n">
-        <v>0.1258</v>
+        <v>0.1257</v>
       </c>
       <c r="C4" t="inlineStr">
         <is>
@@ -51891,7 +51915,7 @@
         </is>
       </c>
       <c r="D17" t="n">
-        <v>0.1258</v>
+        <v>0.1257</v>
       </c>
       <c r="E17" t="inlineStr">
         <is>
@@ -55598,7 +55622,7 @@
         <v>9</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>600.8379</v>
+        <v>600.8274</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -55832,7 +55856,7 @@
         <v>3</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>340.8203</v>
+        <v>340.8198</v>
       </c>
       <c r="I63" t="n">
         <v>3</v>
@@ -55949,7 +55973,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>336.8121</v>
+        <v>336.8116</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -55988,7 +56012,7 @@
         <v>2</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>179.7338</v>
+        <v>179.7238</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
@@ -56027,7 +56051,7 @@
         <v>1</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>179.7338</v>
+        <v>179.7238</v>
       </c>
       <c r="I68" t="n">
         <v>1</v>
@@ -58474,7 +58498,7 @@
         <v>10</v>
       </c>
       <c r="H131" s="5" t="n">
-        <v>2.2836</v>
+        <v>2.2834</v>
       </c>
       <c r="I131" t="n">
         <v>4</v>
@@ -58513,7 +58537,7 @@
         <v>10</v>
       </c>
       <c r="H132" s="5" t="n">
-        <v>2.2836</v>
+        <v>2.2834</v>
       </c>
       <c r="I132" t="n">
         <v>4</v>
@@ -58747,7 +58771,7 @@
         <v>6</v>
       </c>
       <c r="H138" s="5" t="n">
-        <v>2.2631</v>
+        <v>2.2629</v>
       </c>
       <c r="I138" t="n">
         <v>3</v>
@@ -58786,7 +58810,7 @@
         <v>1</v>
       </c>
       <c r="H139" s="5" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="I139" t="n">
         <v>1</v>
@@ -58864,7 +58888,7 @@
         <v>1</v>
       </c>
       <c r="H141" s="5" t="n">
-        <v>1.1123</v>
+        <v>1.1122</v>
       </c>
       <c r="I141" t="n">
         <v>1</v>
@@ -59015,7 +59039,7 @@
         <v>4</v>
       </c>
       <c r="H145" s="5" t="n">
-        <v>0.8124</v>
+        <v>0.8123</v>
       </c>
       <c r="I145" t="n">
         <v>2</v>
@@ -59054,7 +59078,7 @@
         <v>4</v>
       </c>
       <c r="H146" s="5" t="n">
-        <v>0.8124</v>
+        <v>0.8123</v>
       </c>
       <c r="I146" t="n">
         <v>2</v>
@@ -59171,7 +59195,7 @@
         <v>1</v>
       </c>
       <c r="H149" s="5" t="n">
-        <v>0.1258</v>
+        <v>0.1257</v>
       </c>
       <c r="I149" t="n">
         <v>1</v>
@@ -60628,7 +60652,7 @@
         <v>10</v>
       </c>
       <c r="H187" s="5" t="n">
-        <v>5.4747</v>
+        <v>5.4745</v>
       </c>
       <c r="I187" t="n">
         <v>8</v>
@@ -60667,7 +60691,7 @@
         <v>10</v>
       </c>
       <c r="H188" s="5" t="n">
-        <v>5.4747</v>
+        <v>5.4745</v>
       </c>
       <c r="I188" t="n">
         <v>8</v>
@@ -60706,7 +60730,7 @@
         <v>4</v>
       </c>
       <c r="H189" s="5" t="n">
-        <v>4.6734</v>
+        <v>4.6732</v>
       </c>
       <c r="I189" t="n">
         <v>2</v>
@@ -60823,7 +60847,7 @@
         <v>1</v>
       </c>
       <c r="H192" s="5" t="n">
-        <v>2.1234</v>
+        <v>2.1232</v>
       </c>
       <c r="I192" t="n">
         <v>1</v>
@@ -63138,7 +63162,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>179.73</v>
+        <v>179.72</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -63168,7 +63192,7 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>449.33</v>
+        <v>449.31</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -63314,7 +63338,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>336.8121</v>
+        <v>336.8116</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -63339,7 +63363,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>179.7338</v>
+        <v>179.7238</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Death Valley locale run, site basis AQS-SITE-006; single-branch note
The first locale run (270 differing outputs, untracked under sites/) closes
the mass balance at coverage 1.09 and records its one design-check finding
(QC-09, site H2 bank 17.406 kg vs the 19 kg Q-004 basis) plus the absent
groundwater intake unit. X-LOC-07 stays open until both close. Dated record
extended.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -45266,7 +45266,7 @@
       </c>
       <c r="C715" t="inlineStr">
         <is>
-          <t>kPa flat-roof snow (study)</t>
+          <t>kPa flat-roof snow</t>
         </is>
       </c>
       <c r="E715" t="inlineStr">
@@ -46863,7 +46863,7 @@
       </c>
       <c r="C779" t="inlineStr">
         <is>
-          <t>kPa allowable bearing, presumptive clay (CL/ML/MH/CH)</t>
+          <t>kPa allowable bearing, presumptive</t>
         </is>
       </c>
       <c r="D779" t="inlineStr">
@@ -46891,7 +46891,7 @@
       </c>
       <c r="C780" t="inlineStr">
         <is>
-          <t>kN/m3 moist clay</t>
+          <t>kN/m3 moist soil</t>
         </is>
       </c>
       <c r="E780" t="inlineStr">
@@ -47718,7 +47718,7 @@
       </c>
       <c r="C812" t="inlineStr">
         <is>
-          <t>g design 1 s spectral acceleration = 2/3 Fv S1, AQS-SITE-002 S1 0.05 g, site class D, Fv 2.4 (ASCE 7-22 Table 11.4-2)</t>
+          <t>g design 1 s spectral acceleration = 2/3 Fv S1</t>
         </is>
       </c>
       <c r="D812" t="inlineStr">
@@ -47746,7 +47746,7 @@
       </c>
       <c r="C813" t="inlineStr">
         <is>
-          <t>g design short-period spectral acceleration = 2/3 Fa Ss, AQS-SITE-002 Ss 0.10 g, site class D, Fa 1.6 (ASCE 7-22 Table 11.4-1)</t>
+          <t>g design short-period spectral acceleration = 2/3 Fa Ss</t>
         </is>
       </c>
       <c r="D813" t="inlineStr">

</xml_diff>

<commit_message>
GW_INTAKE: groundwater intake unit joins the water cycle; QC-09 reads the sized store
New WTR unit (well pump, sand separator, RO rack; PVC-U/FRP/316L selections
issued in duty section 3; USGS_DV_GW quality basis; RO reject a defined plant
stream) feeding ROOF_TANK with make-up by difference, parallel to the AHU
condensate harvest. Rate solves to zero at the baseline; the instrument index
authors its FT/PT/CT loops; the sizing sweep, P&ID, envelope STL, tree leaf and
task chain follow the standard new-unit induction (tree test count pins updated
with the growth). QC-09 now checks the rack against the graph's sized H2 store
(AQS-ELEC-007 / X-PAR-12, 17 kg) instead of a frozen 19 kg constant, which the
store basis superseded; the check passes honestly at both sites.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -34,7 +34,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DRIVERS'!$A$1:$L$832</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TREE'!$A$1:$J$250</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TREE'!$A$1:$J$251</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DIGESTER'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'OIL'!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'GLASS'!$A$1:$H$6</definedName>
@@ -47,7 +47,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'FARM'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'HAB'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CRYO'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'WTR'!$A$1:$H$9</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'WTR'!$A$1:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'ELEC'!$A$1:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'HEAT'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'MEOH'!$A$1:$H$6</definedName>
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 ed22ff1bb3835551b4aa1d64459cb688a3688229d7ac1f18f05386b0cb165366</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 54183eb7f6220988cb4882e0ae030912ef889f3bc72c0389ee168c5ffc1e0a7d</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>178 units across 19 sectors; the tree leaf set equals the graph unit set (drift guard: pytest flow_graph/param/test_system_tree.py).</t>
+          <t>179 units across 19 sectors; the tree leaf set equals the graph unit set (drift guard: pytest flow_graph/param/test_system_tree.py).</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>249 system-tree nodes: level, parent, type, unit counts, rolled-up kW (SystemTree.aggregate)</t>
+          <t>250 system-tree nodes: level, parent, type, unit counts, rolled-up kW (SystemTree.aggregate)</t>
         </is>
       </c>
     </row>
@@ -15856,7 +15856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H66"/>
+  <dimension ref="A1:H68"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -16040,7 +16040,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>header</t>
+          <t>intake</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -16065,20 +16065,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>REMIN</t>
-        </is>
-      </c>
-      <c r="B7" s="8" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="C7" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="D7" t="inlineStr">
-        <is>
-          <t>study</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -16088,7 +16075,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>header</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -16103,7 +16090,20 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>REMIN</t>
+        </is>
+      </c>
+      <c r="B8" s="8" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="C8" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D8" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -16113,7 +16113,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -16128,147 +16128,150 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
+          <t>ROOF_TANK</t>
+        </is>
+      </c>
+      <c r="E9" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="F9" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="G9" t="b">
+        <v>1</v>
+      </c>
+      <c r="H9" t="inlineStr">
+        <is>
+          <t>WTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="10">
+      <c r="A10" t="inlineStr">
+        <is>
           <t>VCD_TRAIN</t>
         </is>
       </c>
-      <c r="B9" s="8" t="n">
+      <c r="B10" s="8" t="n">
         <v>0.2359</v>
       </c>
-      <c r="C9" t="inlineStr">
+      <c r="C10" t="inlineStr">
         <is>
           <t>kW</t>
         </is>
       </c>
-      <c r="D9" t="inlineStr">
-        <is>
-          <t>study</t>
-        </is>
-      </c>
-      <c r="E9" t="inlineStr">
+      <c r="D10" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
         <is>
           <t>present</t>
         </is>
       </c>
-      <c r="F9" t="inlineStr">
+      <c r="F10" t="inlineStr">
         <is>
           <t>evaporator</t>
         </is>
       </c>
-      <c r="G9" t="b">
-        <v>1</v>
-      </c>
-      <c r="H9" t="inlineStr">
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
         <is>
           <t>WTR</t>
         </is>
       </c>
     </row>
-    <row r="11">
-      <c r="A11" s="1" t="inlineStr">
+    <row r="12">
+      <c r="A12" s="1" t="inlineStr">
         <is>
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B11" s="10">
-        <f>SUM(B2:B9)</f>
+      <c r="B12" s="10">
+        <f>SUM(B2:B10)</f>
         <v/>
       </c>
     </row>
-    <row r="13">
-      <c r="A13" s="9" t="inlineStr">
+    <row r="14">
+      <c r="A14" s="9" t="inlineStr">
         <is>
           <t>EDGES TOUCHING THIS SECTOR (from or to)</t>
         </is>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="3" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="3" t="inlineStr">
         <is>
           <t>stream_id</t>
         </is>
       </c>
-      <c r="B14" s="3" t="inlineStr">
+      <c r="B15" s="3" t="inlineStr">
         <is>
           <t>from_unit</t>
         </is>
       </c>
-      <c r="C14" s="3" t="inlineStr">
+      <c r="C15" s="3" t="inlineStr">
         <is>
           <t>to_unit</t>
         </is>
       </c>
-      <c r="D14" s="3" t="inlineStr">
+      <c r="D15" s="3" t="inlineStr">
         <is>
           <t>rate</t>
         </is>
       </c>
-      <c r="E14" s="3" t="inlineStr">
+      <c r="E15" s="3" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="F14" s="3" t="inlineStr">
+      <c r="F15" s="3" t="inlineStr">
         <is>
           <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="15">
-      <c r="A15" t="inlineStr">
-        <is>
-          <t>DIGEST_TO_POLY</t>
-        </is>
-      </c>
-      <c r="B15" t="inlineStr">
-        <is>
-          <t>BLACK_DIGEST</t>
-        </is>
-      </c>
-      <c r="C15" t="inlineStr">
-        <is>
-          <t>POLY_COND</t>
-        </is>
-      </c>
-      <c r="D15" t="n">
-        <v>0</v>
-      </c>
-      <c r="E15" t="inlineStr">
-        <is>
-          <t>kg/d</t>
-        </is>
-      </c>
-      <c r="F15" t="inlineStr">
-        <is>
-          <t>study</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>HAB_BLACK</t>
+          <t>DIGEST_TO_POLY</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>POLY_COND</t>
+        </is>
+      </c>
+      <c r="D16" t="n">
+        <v>0</v>
+      </c>
+      <c r="E16" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F16" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HAB_GREY</t>
+          <t>HAB_BLACK</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
@@ -16278,7 +16281,7 @@
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
@@ -16290,51 +16293,43 @@
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>IA-BED-H2O</t>
+          <t>HAB_GREY</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
-        </is>
-      </c>
-      <c r="D18" t="n">
-        <v>42.138417</v>
-      </c>
-      <c r="E18" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IA-BLK-01</t>
+          <t>IA-BED-H2O</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="D19" t="n">
-        <v>19.644</v>
+        <v>42.138417</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -16350,21 +16345,21 @@
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IA-BLK-CAKE</t>
+          <t>IA-BLK-01</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
+          <t>HABITATION</t>
+        </is>
+      </c>
+      <c r="C20" t="inlineStr">
+        <is>
           <t>BLACK_DIGEST</t>
         </is>
       </c>
-      <c r="C20" t="inlineStr">
-        <is>
-          <t>AFTERBURNER</t>
-        </is>
-      </c>
       <c r="D20" t="n">
-        <v>0.67</v>
+        <v>19.644</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -16380,7 +16375,7 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IA-BLK-GAS</t>
+          <t>IA-BLK-CAKE</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
@@ -16394,7 +16389,7 @@
         </is>
       </c>
       <c r="D21" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -16410,7 +16405,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IA-BLK-GREY</t>
+          <t>IA-BLK-GAS</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -16420,11 +16415,11 @@
       </c>
       <c r="C22" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="D22" t="n">
-        <v>21.0508</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -16440,7 +16435,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IA-BLK-NUT</t>
+          <t>IA-BLK-GREY</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -16450,11 +16445,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.9</v>
+        <v>21.0508</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -16470,21 +16465,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IA-ELY-H2O</t>
+          <t>IA-BLK-NUT</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>H2O_ELYZ</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>83.620295</v>
+        <v>0.9</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -16500,21 +16495,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IA-ESS-HYDRO-CHG</t>
+          <t>IA-ELY-H2O</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>H2O_ELYZ</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0</v>
+        <v>83.620295</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -16530,17 +16525,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IA-ESS-HYDRO-DIS</t>
+          <t>IA-ESS-HYDRO-CHG</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>CATCH_TANK</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>ROOF_TANK</t>
-        </is>
-      </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -16560,21 +16555,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IA-FEC-01</t>
+          <t>IA-ESS-HYDRO-DIS</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.13</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -16590,12 +16585,12 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IA-FERM-DIG</t>
+          <t>IA-FEC-01</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>MEOH_FERM</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
@@ -16604,7 +16599,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.3454</v>
+        <v>0.13</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -16620,21 +16615,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IA-FLUE-QUENCH</t>
+          <t>IA-FERM-DIG</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>MEOH_FERM</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>FLUE_KO</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>24.31</v>
+        <v>0.3454</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -16650,21 +16645,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IA-GAL</t>
+          <t>IA-FLUE-QUENCH</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>FLUE_KO</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>1.18</v>
+        <v>24.31</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -16680,21 +16675,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IA-GREY-01</t>
+          <t>IA-GAL</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>244.641602</v>
+        <v>1.18</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -16710,7 +16705,7 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IA-GREY-RET</t>
+          <t>IA-GREY-01</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
@@ -16720,11 +16715,11 @@
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0</v>
+        <v>244.641602</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -16740,17 +16735,17 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IA-H2P-H2O</t>
+          <t>IA-GREY-RET</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>H2_DRYER</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D33" t="n">
@@ -16770,12 +16765,12 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IA-HVAC-COND</t>
+          <t>IA-GW-MAKEUP</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
@@ -16784,28 +16779,23 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>67.443215</v>
+        <v>0</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>kg/d</t>
-        </is>
-      </c>
-      <c r="F34" t="inlineStr">
-        <is>
-          <t>study</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IA-LEACH-VCD</t>
+          <t>IA-H2P-H2O</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>H2_DRYER</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
@@ -16814,7 +16804,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>167.999678</v>
+        <v>0</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -16830,12 +16820,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IA-MEOH-COND</t>
+          <t>IA-HVAC-COND</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>MEOH_COND</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -16844,7 +16834,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>26.652161</v>
+        <v>67.443215</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -16860,21 +16850,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IA-NOX-H2O</t>
+          <t>IA-LEACH-VCD</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>221.583096</v>
+        <v>167.999678</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -16890,21 +16880,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-NOX-HAB</t>
+          <t>IA-MEOH-COND</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
+          <t>MEOH_COND</t>
+        </is>
+      </c>
+      <c r="C38" t="inlineStr">
+        <is>
           <t>ROOF_TANK</t>
         </is>
       </c>
-      <c r="C38" t="inlineStr">
-        <is>
-          <t>HABITATION</t>
-        </is>
-      </c>
       <c r="D38" t="n">
-        <v>207.279999</v>
+        <v>26.652161</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -16920,21 +16910,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IA-NUT-01</t>
+          <t>IA-NOX-H2O</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>NOX_SCRUB</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>13.930007</v>
+        <v>221.583096</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -16950,7 +16940,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IA-PEROX-H2O</t>
+          <t>IA-NOX-HAB</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -16960,11 +16950,11 @@
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>WS_PEROX</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>2.824</v>
+        <v>207.279999</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -16980,43 +16970,51 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IA-POL-01</t>
+          <t>IA-NUT-01</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>VCD_TRAIN</t>
+        </is>
+      </c>
+      <c r="D41" t="n">
+        <v>13.930007</v>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F41" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IA-POT-01</t>
+          <t>IA-PEROX-H2O</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>WS_PEROX</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>165.174239</v>
+        <v>2.824</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -17032,51 +17030,43 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IA-UPW-FAB</t>
+          <t>IA-POL-01</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>POLISH_BANK</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>BMED_UPW_POLISH</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>FAB_UPW_TANK</t>
-        </is>
-      </c>
-      <c r="D43" t="n">
-        <v>60.000181</v>
-      </c>
-      <c r="E43" t="inlineStr">
-        <is>
-          <t>kg/d</t>
-        </is>
-      </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IA-UPW-HAB</t>
+          <t>IA-POT-01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.800001</v>
+        <v>165.174239</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -17092,7 +17082,7 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IA-UPW-REJ</t>
+          <t>IA-UPW-FAB</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
@@ -17102,11 +17092,11 @@
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>FAB_UPW_TANK</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>6.045005</v>
+        <v>60.000181</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -17122,21 +17112,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IA-UPW-REMIN</t>
+          <t>IA-UPW-HAB</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>175.174278</v>
+        <v>0.800001</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -17152,21 +17142,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IA-UPW-USE</t>
+          <t>IA-UPW-REJ</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>66.500213</v>
+        <v>6.045005</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -17182,21 +17172,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IA-URINE</t>
+          <t>IA-UPW-REMIN</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>1.42</v>
+        <v>175.174278</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -17212,21 +17202,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IA-VCD-BD</t>
+          <t>IA-UPW-USE</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>6.709424</v>
+        <v>66.500213</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -17242,21 +17232,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IA-ZNBR-BD</t>
+          <t>IA-URINE</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>ZNBR2</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>8.486841</v>
+        <v>1.42</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -17272,21 +17262,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>IA-VCD-BD</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>67.300214</v>
+        <v>6.709424</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -17302,12 +17292,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>IA-ZNBR-BD</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ZNBR2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -17316,7 +17306,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>319.60396</v>
+        <v>8.486841</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -17332,21 +17322,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>3.799494</v>
+        <v>67.300214</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -17362,21 +17352,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S21</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>120.68</v>
+        <v>319.60396</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -17392,21 +17382,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S22</t>
+          <t>S13</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0</v>
+        <v>3.799494</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -17422,21 +17412,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S23</t>
+          <t>S21</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>120.68</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -17452,21 +17442,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S25</t>
+          <t>S22</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>308.519678</v>
+        <v>0</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -17482,21 +17472,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S23</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -17512,7 +17502,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S28</t>
+          <t>S25</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -17522,11 +17512,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>17.877059</v>
+        <v>308.519678</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -17542,21 +17532,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>104.499999</v>
+        <v>10</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -17572,34 +17562,42 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>S28</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="D61" t="n">
+        <v>17.877059</v>
+      </c>
+      <c r="E61" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F61" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
@@ -17608,7 +17606,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>42.876623</v>
+        <v>104.499999</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -17624,55 +17622,47 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>SF-BLACK_DIGEST</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>0.1052</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>kW</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>SF-BMED_UPW_POLISH</t>
+          <t>S52</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.018</v>
+        <v>42.876623</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F64" t="inlineStr">
@@ -17684,7 +17674,7 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SF-REMIN</t>
+          <t>SF-BLACK_DIGEST</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
@@ -17694,11 +17684,11 @@
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.046</v>
+        <v>0.1052</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -17714,27 +17704,87 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
+          <t>SF-BMED_UPW_POLISH</t>
+        </is>
+      </c>
+      <c r="B66" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
+          <t>BMED_UPW_POLISH</t>
+        </is>
+      </c>
+      <c r="D66" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E66" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F66" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="67">
+      <c r="A67" t="inlineStr">
+        <is>
+          <t>SF-REMIN</t>
+        </is>
+      </c>
+      <c r="B67" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C67" t="inlineStr">
+        <is>
+          <t>REMIN</t>
+        </is>
+      </c>
+      <c r="D67" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="E67" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F67" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="68">
+      <c r="A68" t="inlineStr">
+        <is>
           <t>UPW_TO_FAB</t>
         </is>
       </c>
-      <c r="B66" t="inlineStr">
+      <c r="B68" t="inlineStr">
         <is>
           <t>HDR_UPW</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
+      <c r="C68" t="inlineStr">
         <is>
           <t>FAB_UPW_TANK</t>
         </is>
       </c>
-      <c r="F66" t="inlineStr">
+      <c r="F68" t="inlineStr">
         <is>
           <t>null</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H9"/>
+  <autoFilter ref="A1:H10"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -53397,7 +53447,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J250"/>
+  <dimension ref="A1:J251"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -62691,7 +62741,7 @@
         </is>
       </c>
       <c r="G240" t="n">
-        <v>8</v>
+        <v>9</v>
       </c>
       <c r="H240" s="5" t="n">
         <v>0.4051</v>
@@ -62847,7 +62897,7 @@
         </is>
       </c>
       <c r="G244" t="n">
-        <v>6</v>
+        <v>7</v>
       </c>
       <c r="H244" s="5" t="n">
         <v>0.2999</v>
@@ -62942,7 +62992,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.HDR_UPW</t>
+          <t>WTR.potable-upw-train.GW_INTAKE</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -62960,7 +63010,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="G247" t="n">
@@ -62981,7 +63031,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.REMIN</t>
+          <t>WTR.potable-upw-train.HDR_UPW</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -62999,17 +63049,17 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="G248" t="n">
         <v>1</v>
       </c>
       <c r="H248" s="5" t="n">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="I248" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J248" t="inlineStr">
         <is>
@@ -63020,7 +63070,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.ROOF_TANK</t>
+          <t>WTR.potable-upw-train.REMIN</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -63038,17 +63088,17 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="G249" t="n">
         <v>1</v>
       </c>
       <c r="H249" s="5" t="n">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="I249" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -63059,7 +63109,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.VCD_TRAIN</t>
+          <t>WTR.potable-upw-train.ROOF_TANK</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -63077,26 +63127,65 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
+          <t>ROOF_TANK</t>
+        </is>
+      </c>
+      <c r="G250" t="n">
+        <v>1</v>
+      </c>
+      <c r="H250" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I250" t="n">
+        <v>0</v>
+      </c>
+      <c r="J250" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="251">
+      <c r="A251" t="inlineStr">
+        <is>
+          <t>WTR.potable-upw-train.VCD_TRAIN</t>
+        </is>
+      </c>
+      <c r="B251" t="inlineStr">
+        <is>
+          <t>WTR.potable-upw-train</t>
+        </is>
+      </c>
+      <c r="C251" t="n">
+        <v>2</v>
+      </c>
+      <c r="D251" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E251" t="inlineStr">
+        <is>
           <t>VCD_TRAIN</t>
         </is>
       </c>
-      <c r="G250" t="n">
-        <v>1</v>
-      </c>
-      <c r="H250" s="5" t="n">
+      <c r="G251" t="n">
+        <v>1</v>
+      </c>
+      <c r="H251" s="5" t="n">
         <v>0.2359</v>
       </c>
-      <c r="I250" t="n">
-        <v>1</v>
-      </c>
-      <c r="J250" t="inlineStr">
+      <c r="I251" t="n">
+        <v>1</v>
+      </c>
+      <c r="J251" t="inlineStr">
         <is>
           <t>present</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J250"/>
+  <autoFilter ref="A1:J251"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
X-LOC-13: site evaporative rejection charge on the water balance
ATMOS (bookkeeping boundary) + the spray/evaporation edge pair join the graph
at zero; balance.physics books the charge where the site's low-grade rejection
mode is evaporative: spray = rejected kW x 86400 s x 1000 W/kW / 2.454 MJ/kg
(NIST_WEBBOOK), the evaporated fraction leaves to ATMOS, and the groundwater
intake closes the roof-tank balance by difference. Design pass notes: every
write_graph_heat sizing stage precedes balance_report in the regeneration
order, so the mass closure reads final heat-edge rates; GW_INTAKE and ATMOS
join the boundary-meter exemption set (in != out by design). Baseline solved
values unchanged (the edges book zero at air-rejection sites); tree count pins
follow the new leaf. GW_INTAKE/ATMOS duty sheets, P&ID and task chain follow
the standard induction.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -34,7 +34,7 @@
   </sheets>
   <definedNames>
     <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DRIVERS'!$A$1:$L$832</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TREE'!$A$1:$J$251</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TREE'!$A$1:$J$252</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DIGESTER'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'OIL'!$A$1:$H$14</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="7" hidden="1">'GLASS'!$A$1:$H$6</definedName>
@@ -47,7 +47,7 @@
     <definedName name="_xlnm._FilterDatabase" localSheetId="14" hidden="1">'FARM'!$A$1:$H$3</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="15" hidden="1">'HAB'!$A$1:$H$4</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="16" hidden="1">'CRYO'!$A$1:$H$15</definedName>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'WTR'!$A$1:$H$10</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="17" hidden="1">'WTR'!$A$1:$H$11</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="18" hidden="1">'ELEC'!$A$1:$H$10</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="19" hidden="1">'HEAT'!$A$1:$H$13</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="20" hidden="1">'MEOH'!$A$1:$H$6</definedName>
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 54183eb7f6220988cb4882e0ae030912ef889f3bc72c0389ee168c5ffc1e0a7d</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 9479193fdc0f246bab571ab1df72f066c22c2e6c585ed4301b6911d7c62f7f4e</t>
         </is>
       </c>
     </row>
@@ -607,7 +607,7 @@
       </c>
       <c r="B8" t="inlineStr">
         <is>
-          <t>179 units across 19 sectors; the tree leaf set equals the graph unit set (drift guard: pytest flow_graph/param/test_system_tree.py).</t>
+          <t>180 units across 19 sectors; the tree leaf set equals the graph unit set (drift guard: pytest flow_graph/param/test_system_tree.py).</t>
         </is>
       </c>
     </row>
@@ -710,7 +710,7 @@
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>250 system-tree nodes: level, parent, type, unit counts, rolled-up kW (SystemTree.aggregate)</t>
+          <t>251 system-tree nodes: level, parent, type, unit counts, rolled-up kW (SystemTree.aggregate)</t>
         </is>
       </c>
     </row>
@@ -15856,7 +15856,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H68"/>
+  <dimension ref="A1:H71"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -15914,20 +15914,7 @@
     <row r="2">
       <c r="A2" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
-        </is>
-      </c>
-      <c r="B2" s="8" t="n">
-        <v>0.1052</v>
-      </c>
-      <c r="C2" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="D2" t="inlineStr">
-        <is>
-          <t>study</t>
+          <t>ATMOS</t>
         </is>
       </c>
       <c r="E2" t="inlineStr">
@@ -15937,7 +15924,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>digest</t>
+          <t>boundary</t>
         </is>
       </c>
       <c r="G2" t="b">
@@ -15952,11 +15939,11 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>0.018</v>
+        <v>0.1052</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -15975,7 +15962,7 @@
       </c>
       <c r="F3" t="inlineStr">
         <is>
-          <t>skid</t>
+          <t>digest</t>
         </is>
       </c>
       <c r="G3" t="b">
@@ -15990,7 +15977,20 @@
     <row r="4">
       <c r="A4" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>BMED_UPW_POLISH</t>
+        </is>
+      </c>
+      <c r="B4" s="8" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="C4" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D4" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
       <c r="E4" t="inlineStr">
@@ -16000,7 +16000,7 @@
       </c>
       <c r="F4" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>skid</t>
         </is>
       </c>
       <c r="G4" t="b">
@@ -16015,7 +16015,7 @@
     <row r="5">
       <c r="A5" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="E5" t="inlineStr">
@@ -16025,7 +16025,7 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>treat</t>
+          <t>tank</t>
         </is>
       </c>
       <c r="G5" t="b">
@@ -16040,7 +16040,7 @@
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>GW_INTAKE</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -16050,7 +16050,7 @@
       </c>
       <c r="F6" t="inlineStr">
         <is>
-          <t>intake</t>
+          <t>treat</t>
         </is>
       </c>
       <c r="G6" t="b">
@@ -16065,7 +16065,7 @@
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="E7" t="inlineStr">
@@ -16075,7 +16075,7 @@
       </c>
       <c r="F7" t="inlineStr">
         <is>
-          <t>header</t>
+          <t>intake</t>
         </is>
       </c>
       <c r="G7" t="b">
@@ -16090,20 +16090,7 @@
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>REMIN</t>
-        </is>
-      </c>
-      <c r="B8" s="8" t="n">
-        <v>0.046</v>
-      </c>
-      <c r="C8" t="inlineStr">
-        <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="D8" t="inlineStr">
-        <is>
-          <t>study</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="E8" t="inlineStr">
@@ -16113,7 +16100,7 @@
       </c>
       <c r="F8" t="inlineStr">
         <is>
-          <t>dose</t>
+          <t>header</t>
         </is>
       </c>
       <c r="G8" t="b">
@@ -16128,7 +16115,20 @@
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>REMIN</t>
+        </is>
+      </c>
+      <c r="B9" s="8" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
       <c r="E9" t="inlineStr">
@@ -16138,7 +16138,7 @@
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>tank</t>
+          <t>dose</t>
         </is>
       </c>
       <c r="G9" t="b">
@@ -16153,147 +16153,150 @@
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
+          <t>ROOF_TANK</t>
+        </is>
+      </c>
+      <c r="E10" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+      <c r="F10" t="inlineStr">
+        <is>
+          <t>tank</t>
+        </is>
+      </c>
+      <c r="G10" t="b">
+        <v>1</v>
+      </c>
+      <c r="H10" t="inlineStr">
+        <is>
+          <t>WTR</t>
+        </is>
+      </c>
+    </row>
+    <row r="11">
+      <c r="A11" t="inlineStr">
+        <is>
           <t>VCD_TRAIN</t>
         </is>
       </c>
-      <c r="B10" s="8" t="n">
+      <c r="B11" s="8" t="n">
         <v>0.2359</v>
       </c>
-      <c r="C10" t="inlineStr">
+      <c r="C11" t="inlineStr">
         <is>
           <t>kW</t>
         </is>
       </c>
-      <c r="D10" t="inlineStr">
-        <is>
-          <t>study</t>
-        </is>
-      </c>
-      <c r="E10" t="inlineStr">
+      <c r="D11" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+      <c r="E11" t="inlineStr">
         <is>
           <t>present</t>
         </is>
       </c>
-      <c r="F10" t="inlineStr">
+      <c r="F11" t="inlineStr">
         <is>
           <t>evaporator</t>
         </is>
       </c>
-      <c r="G10" t="b">
-        <v>1</v>
-      </c>
-      <c r="H10" t="inlineStr">
+      <c r="G11" t="b">
+        <v>1</v>
+      </c>
+      <c r="H11" t="inlineStr">
         <is>
           <t>WTR</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="1" t="inlineStr">
+    <row r="13">
+      <c r="A13" s="1" t="inlineStr">
         <is>
           <t>SUBTOTAL continuous kW (SUM)</t>
         </is>
       </c>
-      <c r="B12" s="10">
-        <f>SUM(B2:B10)</f>
+      <c r="B13" s="10">
+        <f>SUM(B2:B11)</f>
         <v/>
       </c>
     </row>
-    <row r="14">
-      <c r="A14" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>EDGES TOUCHING THIS SECTOR (from or to)</t>
         </is>
       </c>
     </row>
-    <row r="15">
-      <c r="A15" s="3" t="inlineStr">
+    <row r="16">
+      <c r="A16" s="3" t="inlineStr">
         <is>
           <t>stream_id</t>
         </is>
       </c>
-      <c r="B15" s="3" t="inlineStr">
+      <c r="B16" s="3" t="inlineStr">
         <is>
           <t>from_unit</t>
         </is>
       </c>
-      <c r="C15" s="3" t="inlineStr">
+      <c r="C16" s="3" t="inlineStr">
         <is>
           <t>to_unit</t>
         </is>
       </c>
-      <c r="D15" s="3" t="inlineStr">
+      <c r="D16" s="3" t="inlineStr">
         <is>
           <t>rate</t>
         </is>
       </c>
-      <c r="E15" s="3" t="inlineStr">
+      <c r="E16" s="3" t="inlineStr">
         <is>
           <t>unit</t>
         </is>
       </c>
-      <c r="F15" s="3" t="inlineStr">
+      <c r="F16" s="3" t="inlineStr">
         <is>
           <t>status</t>
-        </is>
-      </c>
-    </row>
-    <row r="16">
-      <c r="A16" t="inlineStr">
-        <is>
-          <t>DIGEST_TO_POLY</t>
-        </is>
-      </c>
-      <c r="B16" t="inlineStr">
-        <is>
-          <t>BLACK_DIGEST</t>
-        </is>
-      </c>
-      <c r="C16" t="inlineStr">
-        <is>
-          <t>POLY_COND</t>
-        </is>
-      </c>
-      <c r="D16" t="n">
-        <v>0</v>
-      </c>
-      <c r="E16" t="inlineStr">
-        <is>
-          <t>kg/d</t>
-        </is>
-      </c>
-      <c r="F16" t="inlineStr">
-        <is>
-          <t>study</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>HAB_BLACK</t>
+          <t>DIGEST_TO_POLY</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>POLY_COND</t>
+        </is>
+      </c>
+      <c r="D17" t="n">
+        <v>0</v>
+      </c>
+      <c r="E17" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F17" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>HAB_GREY</t>
+          <t>HAB_BLACK</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
@@ -16303,7 +16306,7 @@
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="F18" t="inlineStr">
@@ -16315,51 +16318,43 @@
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>IA-BED-H2O</t>
+          <t>HAB_GREY</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
-        </is>
-      </c>
-      <c r="D19" t="n">
-        <v>42.138417</v>
-      </c>
-      <c r="E19" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>IA-BLK-01</t>
+          <t>IA-BED-H2O</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C20" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="D20" t="n">
-        <v>19.644</v>
+        <v>42.138417</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -16375,21 +16370,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>IA-BLK-CAKE</t>
+          <t>IA-BLK-01</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
+          <t>HABITATION</t>
+        </is>
+      </c>
+      <c r="C21" t="inlineStr">
+        <is>
           <t>BLACK_DIGEST</t>
         </is>
       </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>AFTERBURNER</t>
-        </is>
-      </c>
       <c r="D21" t="n">
-        <v>0.67</v>
+        <v>19.644</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -16405,7 +16400,7 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>IA-BLK-GAS</t>
+          <t>IA-BLK-CAKE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
@@ -16419,7 +16414,7 @@
         </is>
       </c>
       <c r="D22" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="E22" t="inlineStr">
         <is>
@@ -16435,7 +16430,7 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>IA-BLK-GREY</t>
+          <t>IA-BLK-GAS</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
@@ -16445,11 +16440,11 @@
       </c>
       <c r="C23" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="D23" t="n">
-        <v>21.0508</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -16465,7 +16460,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IA-BLK-NUT</t>
+          <t>IA-BLK-GREY</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -16475,11 +16470,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.9</v>
+        <v>21.0508</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -16495,21 +16490,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IA-ELY-H2O</t>
+          <t>IA-BLK-NUT</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>H2O_ELYZ</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>83.620295</v>
+        <v>0.9</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -16525,17 +16520,17 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IA-ESS-HYDRO-CHG</t>
+          <t>IA-DC-EVAP</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>DRY_COOLER</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>ATMOS</t>
         </is>
       </c>
       <c r="D26" t="n">
@@ -16546,16 +16541,11 @@
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F26" t="inlineStr">
-        <is>
-          <t>study</t>
-        </is>
-      </c>
     </row>
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IA-ESS-HYDRO-DIS</t>
+          <t>IA-DC-SPRAY</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
@@ -16565,7 +16555,7 @@
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>DRY_COOLER</t>
         </is>
       </c>
       <c r="D27" t="n">
@@ -16576,30 +16566,25 @@
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F27" t="inlineStr">
-        <is>
-          <t>study</t>
-        </is>
-      </c>
     </row>
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IA-FEC-01</t>
+          <t>IA-ELY-H2O</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>H2O_ELYZ</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.13</v>
+        <v>83.620295</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -16615,21 +16600,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IA-FERM-DIG</t>
+          <t>IA-ESS-HYDRO-CHG</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>MEOH_FERM</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.3454</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -16645,7 +16630,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IA-FLUE-QUENCH</t>
+          <t>IA-ESS-HYDRO-DIS</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -16655,11 +16640,11 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>FLUE_KO</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>24.31</v>
+        <v>0</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -16675,7 +16660,7 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IA-GAL</t>
+          <t>IA-FEC-01</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
@@ -16689,7 +16674,7 @@
         </is>
       </c>
       <c r="D31" t="n">
-        <v>1.18</v>
+        <v>0.13</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -16705,21 +16690,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IA-GREY-01</t>
+          <t>IA-FERM-DIG</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>MEOH_FERM</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>244.641602</v>
+        <v>0.3454</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -16735,21 +16720,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IA-GREY-RET</t>
+          <t>IA-FLUE-QUENCH</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>FLUE_KO</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0</v>
+        <v>24.31</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -16765,46 +16750,51 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IA-GW-MAKEUP</t>
+          <t>IA-GAL</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>GW_INTAKE</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>1.18</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
           <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F34" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IA-H2P-H2O</t>
+          <t>IA-GREY-01</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>H2_DRYER</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>244.641602</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -16820,12 +16810,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IA-HVAC-COND</t>
+          <t>IA-GREY-RET</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -16834,7 +16824,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>67.443215</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -16850,51 +16840,46 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IA-LEACH-VCD</t>
+          <t>IA-GW-MAKEUP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>167.999678</v>
+        <v>0</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
           <t>kg/d</t>
-        </is>
-      </c>
-      <c r="F37" t="inlineStr">
-        <is>
-          <t>study</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-MEOH-COND</t>
+          <t>IA-H2P-H2O</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MEOH_COND</t>
+          <t>H2_DRYER</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>26.652161</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -16910,12 +16895,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IA-NOX-H2O</t>
+          <t>IA-HVAC-COND</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -16924,7 +16909,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>221.583096</v>
+        <v>67.443215</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -16940,21 +16925,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IA-NOX-HAB</t>
+          <t>IA-LEACH-VCD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>207.279999</v>
+        <v>167.999678</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -16970,21 +16955,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IA-NUT-01</t>
+          <t>IA-MEOH-COND</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>MEOH_COND</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>13.930007</v>
+        <v>26.652161</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -17000,21 +16985,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IA-PEROX-H2O</t>
+          <t>IA-NOX-H2O</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
+          <t>NOX_SCRUB</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
           <t>ROOF_TANK</t>
         </is>
       </c>
-      <c r="C42" t="inlineStr">
-        <is>
-          <t>WS_PEROX</t>
-        </is>
-      </c>
       <c r="D42" t="n">
-        <v>2.824</v>
+        <v>221.583096</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -17030,43 +17015,51 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IA-POL-01</t>
+          <t>IA-NOX-HAB</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>HABITATION</t>
+        </is>
+      </c>
+      <c r="D43" t="n">
+        <v>207.279999</v>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F43" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IA-POT-01</t>
+          <t>IA-NUT-01</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>165.174239</v>
+        <v>13.930007</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -17082,21 +17075,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IA-UPW-FAB</t>
+          <t>IA-PEROX-H2O</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>FAB_UPW_TANK</t>
+          <t>WS_PEROX</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>60.000181</v>
+        <v>2.824</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -17112,51 +17105,43 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IA-UPW-HAB</t>
+          <t>IA-POL-01</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>HABITATION</t>
-        </is>
-      </c>
-      <c r="D46" t="n">
-        <v>0.800001</v>
-      </c>
-      <c r="E46" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="F46" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IA-UPW-REJ</t>
+          <t>IA-POT-01</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>6.045005</v>
+        <v>165.174239</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -17172,7 +17157,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IA-UPW-REMIN</t>
+          <t>IA-UPW-FAB</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -17182,11 +17167,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>FAB_UPW_TANK</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>175.174278</v>
+        <v>60.000181</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -17202,7 +17187,7 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IA-UPW-USE</t>
+          <t>IA-UPW-HAB</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
@@ -17212,11 +17197,11 @@
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>66.500213</v>
+        <v>0.800001</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -17232,21 +17217,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IA-URINE</t>
+          <t>IA-UPW-REJ</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>1.42</v>
+        <v>6.045005</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -17262,21 +17247,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IA-VCD-BD</t>
+          <t>IA-UPW-REMIN</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>6.709424</v>
+        <v>175.174278</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -17292,21 +17277,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IA-ZNBR-BD</t>
+          <t>IA-UPW-USE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>ZNBR2</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>8.486841</v>
+        <v>66.500213</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -17322,21 +17307,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S01</t>
+          <t>IA-URINE</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>67.300214</v>
+        <v>1.42</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -17352,21 +17337,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S12</t>
+          <t>IA-VCD-BD</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>319.60396</v>
+        <v>6.709424</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -17382,21 +17367,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S13</t>
+          <t>IA-ZNBR-BD</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>ZNBR2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>3.799494</v>
+        <v>8.486841</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -17412,21 +17397,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S21</t>
+          <t>S01</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>120.68</v>
+        <v>67.300214</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -17442,21 +17427,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S22</t>
+          <t>S12</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>319.60396</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -17472,21 +17457,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S23</t>
+          <t>S13</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0</v>
+        <v>3.799494</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -17502,21 +17487,21 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S25</t>
+          <t>S21</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>308.519678</v>
+        <v>120.68</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -17532,21 +17517,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S26</t>
+          <t>S22</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -17562,21 +17547,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S28</t>
+          <t>S23</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>17.877059</v>
+        <v>0</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -17592,21 +17577,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S29</t>
+          <t>S25</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>104.499999</v>
+        <v>308.519678</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -17622,43 +17607,51 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S30</t>
+          <t>S26</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>HABITATION</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>10</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S52</t>
+          <t>S28</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>42.876623</v>
+        <v>17.877059</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -17674,25 +17667,25 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>SF-BLACK_DIGEST</t>
+          <t>S29</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.1052</v>
+        <v>104.499999</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F65" t="inlineStr">
@@ -17704,55 +17697,47 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>SF-BMED_UPW_POLISH</t>
+          <t>S30</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
-        </is>
-      </c>
-      <c r="D66" t="n">
-        <v>0.018</v>
-      </c>
-      <c r="E66" t="inlineStr">
-        <is>
-          <t>kW</t>
+          <t>NUTRIENT_DOSE</t>
         </is>
       </c>
       <c r="F66" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SF-REMIN</t>
+          <t>S52</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.046</v>
+        <v>42.876623</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -17764,27 +17749,117 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
+          <t>SF-BLACK_DIGEST</t>
+        </is>
+      </c>
+      <c r="B68" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C68" t="inlineStr">
+        <is>
+          <t>BLACK_DIGEST</t>
+        </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0.1052</v>
+      </c>
+      <c r="E68" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F68" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="69">
+      <c r="A69" t="inlineStr">
+        <is>
+          <t>SF-BMED_UPW_POLISH</t>
+        </is>
+      </c>
+      <c r="B69" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C69" t="inlineStr">
+        <is>
+          <t>BMED_UPW_POLISH</t>
+        </is>
+      </c>
+      <c r="D69" t="n">
+        <v>0.018</v>
+      </c>
+      <c r="E69" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F69" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" t="inlineStr">
+        <is>
+          <t>SF-REMIN</t>
+        </is>
+      </c>
+      <c r="B70" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C70" t="inlineStr">
+        <is>
+          <t>REMIN</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>0.046</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F70" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="71">
+      <c r="A71" t="inlineStr">
+        <is>
           <t>UPW_TO_FAB</t>
         </is>
       </c>
-      <c r="B68" t="inlineStr">
+      <c r="B71" t="inlineStr">
         <is>
           <t>HDR_UPW</t>
         </is>
       </c>
-      <c r="C68" t="inlineStr">
+      <c r="C71" t="inlineStr">
         <is>
           <t>FAB_UPW_TANK</t>
         </is>
       </c>
-      <c r="F68" t="inlineStr">
+      <c r="F71" t="inlineStr">
         <is>
           <t>null</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:H10"/>
+  <autoFilter ref="A1:H11"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
@@ -48309,7 +48384,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H71"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -49691,81 +49766,71 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IA-MAU-AIR</t>
+          <t>IA-DC-EVAP</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>MAU_HX</t>
+          <t>DRY_COOLER</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>ATMOS</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>12</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="F52" t="inlineStr">
-        <is>
-          <t>study</t>
+          <t>kg/d</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IA-Q1A-LOSS</t>
+          <t>IA-DC-SPRAY</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>Q1_A</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>BOUNDARY_EXPORT</t>
+          <t>DRY_COOLER</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.25</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>kW</t>
-        </is>
-      </c>
-      <c r="F53" t="inlineStr">
-        <is>
-          <t>study</t>
+          <t>kg/d</t>
         </is>
       </c>
     </row>
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IA-Q1B-LOSS</t>
+          <t>IA-MAU-AIR</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Q1_B</t>
+          <t>MAU_HX</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>BOUNDARY_EXPORT</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.25</v>
+        <v>12</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -49781,12 +49846,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IA-Q2A-LOSS</t>
+          <t>IA-Q1A-LOSS</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>Q2_A</t>
+          <t>Q1_A</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -49795,7 +49860,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -49811,12 +49876,12 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IA-Q2B-LOSS</t>
+          <t>IA-Q1B-LOSS</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>Q2_B</t>
+          <t>Q1_B</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
@@ -49825,7 +49890,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.17</v>
+        <v>0.25</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -49841,21 +49906,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IA-Q4-ADS</t>
+          <t>IA-Q2A-LOSS</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>Q2_A</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>ADS_CHILL</t>
+          <t>BOUNDARY_EXPORT</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>5</v>
+        <v>0.17</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -49871,21 +49936,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IA-Q4-LIFE</t>
+          <t>IA-Q2B-LOSS</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>Q2_B</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>BOUNDARY_EXPORT</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>3</v>
+        <v>0.17</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -49901,7 +49966,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IA-Q4-MAU</t>
+          <t>IA-Q4-ADS</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -49911,11 +49976,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>MAU_HX</t>
+          <t>ADS_CHILL</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>12</v>
+        <v>5</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -49931,21 +49996,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IA-Q4A-TRIM</t>
+          <t>IA-Q4-LIFE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>RECTIFIER</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>Q4_A</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>1.61</v>
+        <v>3</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -49961,21 +50026,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>IA-Q4B-TRIM</t>
+          <t>IA-Q4-MAU</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>RECTIFIER</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>Q4_B</t>
+          <t>MAU_HX</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>1.61</v>
+        <v>12</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -49991,7 +50056,7 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>IA-RECT-Q4</t>
+          <t>IA-Q4A-TRIM</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
@@ -50001,11 +50066,11 @@
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>Q4_A</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1</v>
+        <v>1.61</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -50021,21 +50086,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>IA-ZNBR-HEAT</t>
+          <t>IA-Q4B-TRIM</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>ZNBR2</t>
+          <t>RECTIFIER</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>Q4_B</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>1.67</v>
+        <v>1.61</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -50051,21 +50116,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S100</t>
+          <t>IA-RECT-Q4</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>RECTIFIER</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
           <t>Q4_BUS</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
       <c r="D64" t="n">
-        <v>0.5322</v>
+        <v>1</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -50081,21 +50146,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S101</t>
+          <t>IA-ZNBR-HEAT</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>ZNBR2</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
           <t>Q4_BUS</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>GLASS_DIGEST</t>
-        </is>
-      </c>
       <c r="D65" t="n">
-        <v>0.2822</v>
+        <v>1.67</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -50111,21 +50176,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S44</t>
+          <t>S100</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>GEO_HP</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>2.1972</v>
+        <v>0.5322</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -50141,21 +50206,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S53</t>
+          <t>S101</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>GLASS_DIGEST</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.1419</v>
+        <v>0.2822</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -50171,12 +50236,12 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S54</t>
+          <t>S44</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CRYO_HX_Q4</t>
+          <t>GEO_HP</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
@@ -50185,7 +50250,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.5448</v>
+        <v>2.1972</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -50201,12 +50266,12 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S63</t>
+          <t>S53</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>MET_HX_Q4</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
@@ -50215,7 +50280,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.0171</v>
+        <v>1.1419</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -50231,12 +50296,12 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S80</t>
+          <t>S54</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MEOH_FC</t>
+          <t>CRYO_HX_Q4</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
@@ -50245,7 +50310,7 @@
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.3689</v>
+        <v>0.5448</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -50261,28 +50326,88 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
+          <t>S63</t>
+        </is>
+      </c>
+      <c r="B71" t="inlineStr">
+        <is>
+          <t>MET_HX_Q4</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
+          <t>Q4_BUS</t>
+        </is>
+      </c>
+      <c r="D71" t="n">
+        <v>0.0171</v>
+      </c>
+      <c r="E71" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F71" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="72">
+      <c r="A72" t="inlineStr">
+        <is>
+          <t>S80</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>MEOH_FC</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>Q4_BUS</t>
+        </is>
+      </c>
+      <c r="D72" t="n">
+        <v>0.3689</v>
+      </c>
+      <c r="E72" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>SQ-H2O_ELYZ-Q4</t>
         </is>
       </c>
-      <c r="B71" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>H2O_ELYZ</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>Q4_BUS</t>
         </is>
       </c>
-      <c r="D71" t="n">
+      <c r="D73" t="n">
         <v>6.0825</v>
       </c>
-      <c r="E71" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>kW</t>
         </is>
       </c>
-      <c r="F71" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>study</t>
         </is>
@@ -53447,7 +53572,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J251"/>
+  <dimension ref="A1:J252"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="52" customWidth="1" min="1" max="1"/>
@@ -62741,7 +62866,7 @@
         </is>
       </c>
       <c r="G240" t="n">
-        <v>9</v>
+        <v>10</v>
       </c>
       <c r="H240" s="5" t="n">
         <v>0.4051</v>
@@ -62758,7 +62883,7 @@
     <row r="241">
       <c r="A241" t="inlineStr">
         <is>
-          <t>WTR.grey-black-train</t>
+          <t>WTR.ATMOS</t>
         </is>
       </c>
       <c r="B241" t="inlineStr">
@@ -62771,22 +62896,22 @@
       </c>
       <c r="D241" t="inlineStr">
         <is>
-          <t>train</t>
-        </is>
-      </c>
-      <c r="F241" t="inlineStr">
-        <is>
-          <t>Grey treatment and the blackwater barrier digest (vacuum toilet, urine, fecal, galley).</t>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E241" t="inlineStr">
+        <is>
+          <t>ATMOS</t>
         </is>
       </c>
       <c r="G241" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="H241" s="5" t="n">
-        <v>0.1052</v>
+        <v>0</v>
       </c>
       <c r="I241" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J241" t="inlineStr">
         <is>
@@ -62797,29 +62922,29 @@
     <row r="242">
       <c r="A242" t="inlineStr">
         <is>
-          <t>WTR.grey-black-train.BLACK_DIGEST</t>
+          <t>WTR.grey-black-train</t>
         </is>
       </c>
       <c r="B242" t="inlineStr">
         <is>
-          <t>WTR.grey-black-train</t>
+          <t>WTR</t>
         </is>
       </c>
       <c r="C242" t="n">
+        <v>1</v>
+      </c>
+      <c r="D242" t="inlineStr">
+        <is>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="F242" t="inlineStr">
+        <is>
+          <t>Grey treatment and the blackwater barrier digest (vacuum toilet, urine, fecal, galley).</t>
+        </is>
+      </c>
+      <c r="G242" t="n">
         <v>2</v>
-      </c>
-      <c r="D242" t="inlineStr">
-        <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="E242" t="inlineStr">
-        <is>
-          <t>BLACK_DIGEST</t>
-        </is>
-      </c>
-      <c r="G242" t="n">
-        <v>1</v>
       </c>
       <c r="H242" s="5" t="n">
         <v>0.1052</v>
@@ -62836,7 +62961,7 @@
     <row r="243">
       <c r="A243" t="inlineStr">
         <is>
-          <t>WTR.grey-black-train.GREY_TREAT</t>
+          <t>WTR.grey-black-train.BLACK_DIGEST</t>
         </is>
       </c>
       <c r="B243" t="inlineStr">
@@ -62854,17 +62979,17 @@
       </c>
       <c r="E243" t="inlineStr">
         <is>
-          <t>GREY_TREAT</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="G243" t="n">
         <v>1</v>
       </c>
       <c r="H243" s="5" t="n">
-        <v>0</v>
+        <v>0.1052</v>
       </c>
       <c r="I243" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J243" t="inlineStr">
         <is>
@@ -62875,35 +63000,35 @@
     <row r="244">
       <c r="A244" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train</t>
+          <t>WTR.grey-black-train.GREY_TREAT</t>
         </is>
       </c>
       <c r="B244" t="inlineStr">
         <is>
-          <t>WTR</t>
+          <t>WTR.grey-black-train</t>
         </is>
       </c>
       <c r="C244" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="D244" t="inlineStr">
         <is>
-          <t>train</t>
-        </is>
-      </c>
-      <c r="F244" t="inlineStr">
-        <is>
-          <t>Roof and catch tanks (pumped-hydro penstock peers), VCD, BMED UPW polish, UPW header, remineralizer to potable.</t>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E244" t="inlineStr">
+        <is>
+          <t>GREY_TREAT</t>
         </is>
       </c>
       <c r="G244" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="H244" s="5" t="n">
-        <v>0.2999</v>
+        <v>0</v>
       </c>
       <c r="I244" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="J244" t="inlineStr">
         <is>
@@ -62914,35 +63039,35 @@
     <row r="245">
       <c r="A245" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.BMED_UPW_POLISH</t>
+          <t>WTR.potable-upw-train</t>
         </is>
       </c>
       <c r="B245" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train</t>
+          <t>WTR</t>
         </is>
       </c>
       <c r="C245" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="D245" t="inlineStr">
         <is>
-          <t>unit</t>
-        </is>
-      </c>
-      <c r="E245" t="inlineStr">
-        <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>train</t>
+        </is>
+      </c>
+      <c r="F245" t="inlineStr">
+        <is>
+          <t>Roof and catch tanks (pumped-hydro penstock peers), VCD, BMED UPW polish, UPW header, remineralizer to potable.</t>
         </is>
       </c>
       <c r="G245" t="n">
-        <v>1</v>
+        <v>7</v>
       </c>
       <c r="H245" s="5" t="n">
-        <v>0.018</v>
+        <v>0.2999</v>
       </c>
       <c r="I245" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -62953,7 +63078,7 @@
     <row r="246">
       <c r="A246" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.CATCH_TANK</t>
+          <t>WTR.potable-upw-train.BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="B246" t="inlineStr">
@@ -62971,17 +63096,17 @@
       </c>
       <c r="E246" t="inlineStr">
         <is>
-          <t>CATCH_TANK</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="G246" t="n">
         <v>1</v>
       </c>
       <c r="H246" s="5" t="n">
-        <v>0</v>
+        <v>0.018</v>
       </c>
       <c r="I246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -62992,7 +63117,7 @@
     <row r="247">
       <c r="A247" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.GW_INTAKE</t>
+          <t>WTR.potable-upw-train.CATCH_TANK</t>
         </is>
       </c>
       <c r="B247" t="inlineStr">
@@ -63010,7 +63135,7 @@
       </c>
       <c r="E247" t="inlineStr">
         <is>
-          <t>GW_INTAKE</t>
+          <t>CATCH_TANK</t>
         </is>
       </c>
       <c r="G247" t="n">
@@ -63031,7 +63156,7 @@
     <row r="248">
       <c r="A248" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.HDR_UPW</t>
+          <t>WTR.potable-upw-train.GW_INTAKE</t>
         </is>
       </c>
       <c r="B248" t="inlineStr">
@@ -63049,7 +63174,7 @@
       </c>
       <c r="E248" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>GW_INTAKE</t>
         </is>
       </c>
       <c r="G248" t="n">
@@ -63070,7 +63195,7 @@
     <row r="249">
       <c r="A249" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.REMIN</t>
+          <t>WTR.potable-upw-train.HDR_UPW</t>
         </is>
       </c>
       <c r="B249" t="inlineStr">
@@ -63088,17 +63213,17 @@
       </c>
       <c r="E249" t="inlineStr">
         <is>
-          <t>REMIN</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="G249" t="n">
         <v>1</v>
       </c>
       <c r="H249" s="5" t="n">
-        <v>0.046</v>
+        <v>0</v>
       </c>
       <c r="I249" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J249" t="inlineStr">
         <is>
@@ -63109,7 +63234,7 @@
     <row r="250">
       <c r="A250" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.ROOF_TANK</t>
+          <t>WTR.potable-upw-train.REMIN</t>
         </is>
       </c>
       <c r="B250" t="inlineStr">
@@ -63127,17 +63252,17 @@
       </c>
       <c r="E250" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>REMIN</t>
         </is>
       </c>
       <c r="G250" t="n">
         <v>1</v>
       </c>
       <c r="H250" s="5" t="n">
-        <v>0</v>
+        <v>0.046</v>
       </c>
       <c r="I250" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J250" t="inlineStr">
         <is>
@@ -63148,7 +63273,7 @@
     <row r="251">
       <c r="A251" t="inlineStr">
         <is>
-          <t>WTR.potable-upw-train.VCD_TRAIN</t>
+          <t>WTR.potable-upw-train.ROOF_TANK</t>
         </is>
       </c>
       <c r="B251" t="inlineStr">
@@ -63166,26 +63291,65 @@
       </c>
       <c r="E251" t="inlineStr">
         <is>
+          <t>ROOF_TANK</t>
+        </is>
+      </c>
+      <c r="G251" t="n">
+        <v>1</v>
+      </c>
+      <c r="H251" s="5" t="n">
+        <v>0</v>
+      </c>
+      <c r="I251" t="n">
+        <v>0</v>
+      </c>
+      <c r="J251" t="inlineStr">
+        <is>
+          <t>present</t>
+        </is>
+      </c>
+    </row>
+    <row r="252">
+      <c r="A252" t="inlineStr">
+        <is>
+          <t>WTR.potable-upw-train.VCD_TRAIN</t>
+        </is>
+      </c>
+      <c r="B252" t="inlineStr">
+        <is>
+          <t>WTR.potable-upw-train</t>
+        </is>
+      </c>
+      <c r="C252" t="n">
+        <v>2</v>
+      </c>
+      <c r="D252" t="inlineStr">
+        <is>
+          <t>unit</t>
+        </is>
+      </c>
+      <c r="E252" t="inlineStr">
+        <is>
           <t>VCD_TRAIN</t>
         </is>
       </c>
-      <c r="G251" t="n">
-        <v>1</v>
-      </c>
-      <c r="H251" s="5" t="n">
+      <c r="G252" t="n">
+        <v>1</v>
+      </c>
+      <c r="H252" s="5" t="n">
         <v>0.2359</v>
       </c>
-      <c r="I251" t="n">
-        <v>1</v>
-      </c>
-      <c r="J251" t="inlineStr">
+      <c r="I252" t="n">
+        <v>1</v>
+      </c>
+      <c r="J252" t="inlineStr">
         <is>
           <t>present</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:J251"/>
+  <autoFilter ref="A1:J252"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
X-UI-002 follow-up: the internals duty-quote scan stops eating the envelope filename; the placement-routes artifacts and the MF-28/WF-30 design files join the tracked set
- _internals.py: the unit-id strip governs the keyword scan only - the quoted
  fragment now comes from the original duty text, so the envelope citation
  cad/stl/<UNIT>.stl survives (the strip had eaten the filename into
  cad/stl/.stl, dangling the citation on every new internals row).
- The same fix cascades to the fab sheets (they quote the internals register).
- The placement-routes artifacts (ISO_ROUTES.md/.json, ISO_SHEETS.md/.csv) and
  the generator join the tracked set; _doc_register refreshes.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 978d0c66abb9bc99fdd646b48da1bf02f27eb3eb24f3b11481a568af3d3d4d32</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 79339916a4ef21d586f3fc367adc1d954b703f2585b42895e9ebdcb3e136397e</t>
         </is>
       </c>
     </row>
@@ -19174,6 +19174,19 @@
           <t>GW_INTAKE</t>
         </is>
       </c>
+      <c r="B9" s="8" t="n">
+        <v>0.37</v>
+      </c>
+      <c r="C9" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D9" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
       <c r="E9" t="inlineStr">
         <is>
           <t>present</t>
@@ -21466,7 +21479,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>68.2838</v>
+        <v>72.90009999999999</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -21592,7 +21605,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>337.8116</v>
+        <v>342.4279</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -21693,7 +21706,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>180.7538</v>
+        <v>191.3901</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -22498,7 +22511,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>337.8116</v>
+        <v>342.4279</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -23180,7 +23193,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>759.5575689999999</v>
+        <v>804.2529950000001</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -23210,7 +23223,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>759.5575689999999</v>
+        <v>804.2529950000001</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -23840,7 +23853,7 @@
         </is>
       </c>
       <c r="D85" t="n">
-        <v>68.2838</v>
+        <v>72.90009999999999</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -55573,6 +55586,19 @@
           <t>DRY_COOLER</t>
         </is>
       </c>
+      <c r="B3" s="8" t="n">
+        <v>0.15</v>
+      </c>
+      <c r="C3" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D3" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
       <c r="E3" t="inlineStr">
         <is>
           <t>present</t>
@@ -61681,10 +61707,10 @@
         <v>25</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>14.4748</v>
+        <v>14.5748</v>
       </c>
       <c r="I21" t="n">
-        <v>6</v>
+        <v>8</v>
       </c>
       <c r="J21" t="inlineStr">
         <is>
@@ -62227,10 +62253,10 @@
         <v>15</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>9.2265</v>
+        <v>9.326499999999999</v>
       </c>
       <c r="I35" t="n">
-        <v>5</v>
+        <v>7</v>
       </c>
       <c r="J35" t="inlineStr">
         <is>
@@ -62500,10 +62526,10 @@
         <v>10</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>0.75</v>
+        <v>0.85</v>
       </c>
       <c r="I42" t="n">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="J42" t="inlineStr">
         <is>
@@ -62734,10 +62760,10 @@
         <v>1</v>
       </c>
       <c r="H48" s="5" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="I48" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J48" t="inlineStr">
         <is>
@@ -62812,10 +62838,10 @@
         <v>1</v>
       </c>
       <c r="H50" s="5" t="n">
-        <v>0</v>
+        <v>0.05</v>
       </c>
       <c r="I50" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J50" t="inlineStr">
         <is>
@@ -63075,7 +63101,7 @@
         <v>10</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>602.8574</v>
+        <v>622.7263</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -63114,7 +63140,7 @@
         <v>4</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>80.2838</v>
+        <v>84.90009999999999</v>
       </c>
       <c r="I58" t="n">
         <v>2</v>
@@ -63153,7 +63179,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>68.2838</v>
+        <v>72.90009999999999</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -63309,7 +63335,7 @@
         <v>3</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>341.8198</v>
+        <v>346.4361</v>
       </c>
       <c r="I63" t="n">
         <v>3</v>
@@ -63426,7 +63452,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>337.8116</v>
+        <v>342.4279</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -63465,7 +63491,7 @@
         <v>3</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>180.7538</v>
+        <v>191.3901</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
@@ -63543,7 +63569,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="5" t="n">
-        <v>180.7538</v>
+        <v>191.3901</v>
       </c>
       <c r="I69" t="n">
         <v>1</v>
@@ -67540,10 +67566,10 @@
         <v>5</v>
       </c>
       <c r="H172" s="5" t="n">
-        <v>0.09</v>
+        <v>5.09</v>
       </c>
       <c r="I172" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J172" t="inlineStr">
         <is>
@@ -67579,10 +67605,10 @@
         <v>5</v>
       </c>
       <c r="H173" s="5" t="n">
-        <v>0.09</v>
+        <v>5.09</v>
       </c>
       <c r="I173" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="J173" t="inlineStr">
         <is>
@@ -67618,10 +67644,10 @@
         <v>1</v>
       </c>
       <c r="H174" s="5" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="I174" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J174" t="inlineStr">
         <is>
@@ -68310,10 +68336,10 @@
         <v>13</v>
       </c>
       <c r="H192" s="5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I192" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J192" t="inlineStr">
         <is>
@@ -68349,10 +68375,10 @@
         <v>13</v>
       </c>
       <c r="H193" s="5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I193" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J193" t="inlineStr">
         <is>
@@ -68388,10 +68414,10 @@
         <v>4</v>
       </c>
       <c r="H194" s="5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I194" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J194" t="inlineStr">
         <is>
@@ -68466,10 +68492,10 @@
         <v>1</v>
       </c>
       <c r="H196" s="5" t="n">
-        <v>0</v>
+        <v>0.15</v>
       </c>
       <c r="I196" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J196" t="inlineStr">
         <is>
@@ -69928,10 +69954,10 @@
         <v>14</v>
       </c>
       <c r="H234" s="5" t="n">
-        <v>1.7972</v>
+        <v>2.1972</v>
       </c>
       <c r="I234" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J234" t="inlineStr">
         <is>
@@ -69967,10 +69993,10 @@
         <v>14</v>
       </c>
       <c r="H235" s="5" t="n">
-        <v>1.7972</v>
+        <v>2.1972</v>
       </c>
       <c r="I235" t="n">
-        <v>2</v>
+        <v>4</v>
       </c>
       <c r="J235" t="inlineStr">
         <is>
@@ -70357,10 +70383,10 @@
         <v>2</v>
       </c>
       <c r="H245" s="5" t="n">
-        <v>0</v>
+        <v>0.4</v>
       </c>
       <c r="I245" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="J245" t="inlineStr">
         <is>
@@ -70396,10 +70422,10 @@
         <v>1</v>
       </c>
       <c r="H246" s="5" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I246" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J246" t="inlineStr">
         <is>
@@ -70435,10 +70461,10 @@
         <v>1</v>
       </c>
       <c r="H247" s="5" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="I247" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J247" t="inlineStr">
         <is>
@@ -71356,10 +71382,10 @@
         <v>18</v>
       </c>
       <c r="H271" s="5" t="n">
-        <v>0.4275</v>
+        <v>0.7975</v>
       </c>
       <c r="I271" t="n">
-        <v>4</v>
+        <v>5</v>
       </c>
       <c r="J271" t="inlineStr">
         <is>
@@ -71590,10 +71616,10 @@
         <v>14</v>
       </c>
       <c r="H277" s="5" t="n">
-        <v>0.3223</v>
+        <v>0.6923</v>
       </c>
       <c r="I277" t="n">
-        <v>3</v>
+        <v>4</v>
       </c>
       <c r="J277" t="inlineStr">
         <is>
@@ -71785,10 +71811,10 @@
         <v>1</v>
       </c>
       <c r="H282" s="5" t="n">
-        <v>0</v>
+        <v>0.37</v>
       </c>
       <c r="I282" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J282" t="inlineStr">
         <is>
@@ -72214,7 +72240,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>180.75</v>
+        <v>191.39</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -72228,7 +72254,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 29x23 bays, ext 68.28 kW).</t>
+          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 31x23 bays, ext 72.90 kW).</t>
         </is>
       </c>
     </row>
@@ -72244,7 +72270,7 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>451.88</v>
+        <v>478.48</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -72289,7 +72315,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>5012</v>
+        <v>5308</v>
       </c>
     </row>
     <row r="6">
@@ -72319,7 +72345,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="8">
@@ -72390,7 +72416,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>337.8116</v>
+        <v>342.4279</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -72415,7 +72441,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>180.7538</v>
+        <v>191.3901</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -72518,7 +72544,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>5012</v>
+        <v>5308</v>
       </c>
     </row>
     <row r="19">
@@ -72533,7 +72559,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2506</v>
+        <v>2654</v>
       </c>
     </row>
     <row r="20">
@@ -72548,7 +72574,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21986</v>
+        <v>23569</v>
       </c>
     </row>
     <row r="21">
@@ -72563,7 +72589,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1253</v>
+        <v>1327</v>
       </c>
     </row>
     <row r="22">
@@ -72593,7 +72619,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>822</v>
+        <v>870</v>
       </c>
     </row>
     <row r="24">
@@ -72608,7 +72634,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2531</v>
+        <v>2680</v>
       </c>
     </row>
     <row r="25">
@@ -72623,7 +72649,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>822</v>
+        <v>870</v>
       </c>
     </row>
     <row r="26">
@@ -72638,7 +72664,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>181</v>
+        <v>192</v>
       </c>
     </row>
     <row r="27">
@@ -72653,7 +72679,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2100</v>
+        <v>2220</v>
       </c>
     </row>
     <row r="28">
@@ -72668,7 +72694,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>35</v>
+        <v>37</v>
       </c>
     </row>
     <row r="29">
@@ -72698,7 +72724,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1919.2</v>
+        <v>2028.6</v>
       </c>
     </row>
     <row r="31">
@@ -75649,6 +75675,19 @@
           <t>LI_RECOVER</t>
         </is>
       </c>
+      <c r="B22" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D22" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
       <c r="E22" t="inlineStr">
         <is>
           <t>present</t>
@@ -75697,6 +75736,19 @@
       <c r="A24" t="inlineStr">
         <is>
           <t>P_CA</t>
+        </is>
+      </c>
+      <c r="B24" s="8" t="n">
+        <v>0.05</v>
+      </c>
+      <c r="C24" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D24" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
       <c r="E24" t="inlineStr">
@@ -79465,6 +79517,9 @@
           <t>GREASE_LI</t>
         </is>
       </c>
+      <c r="D154" t="n">
+        <v>0.5</v>
+      </c>
       <c r="F154" t="inlineStr">
         <is>
           <t>null</t>
@@ -79577,6 +79632,9 @@
           <t>GREASE_CA</t>
         </is>
       </c>
+      <c r="D158" t="n">
+        <v>0.025</v>
+      </c>
       <c r="F158" t="inlineStr">
         <is>
           <t>null</t>
@@ -79598,6 +79656,9 @@
         <is>
           <t>LI_RECOVER</t>
         </is>
+      </c>
+      <c r="D159" t="n">
+        <v>0.5</v>
       </c>
       <c r="F159" t="inlineStr">
         <is>
@@ -80546,6 +80607,19 @@
           <t>GREASE_CA</t>
         </is>
       </c>
+      <c r="B5" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C5" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D5" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
       <c r="E5" t="inlineStr">
         <is>
           <t>present</t>
@@ -80569,6 +80643,19 @@
       <c r="A6" t="inlineStr">
         <is>
           <t>GREASE_LI</t>
+        </is>
+      </c>
+      <c r="B6" s="8" t="n">
+        <v>0.2</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>study</t>
         </is>
       </c>
       <c r="E6" t="inlineStr">
@@ -80954,6 +81041,9 @@
           <t>SI_REDUCE</t>
         </is>
       </c>
+      <c r="D23" t="n">
+        <v>1.924</v>
+      </c>
       <c r="F23" t="inlineStr">
         <is>
           <t>null</t>
@@ -81920,6 +82010,9 @@
           <t>GREASE_LI</t>
         </is>
       </c>
+      <c r="D56" t="n">
+        <v>0.5</v>
+      </c>
       <c r="F56" t="inlineStr">
         <is>
           <t>null</t>
@@ -82002,6 +82095,9 @@
           <t>GREASE_CA</t>
         </is>
       </c>
+      <c r="D59" t="n">
+        <v>0.025</v>
+      </c>
       <c r="F59" t="inlineStr">
         <is>
           <t>null</t>
@@ -82234,6 +82330,9 @@
           <t>GREASE_CA</t>
         </is>
       </c>
+      <c r="D67" t="n">
+        <v>0.2</v>
+      </c>
       <c r="F67" t="inlineStr">
         <is>
           <t>null</t>
@@ -82255,6 +82354,9 @@
         <is>
           <t>GREASE_LI</t>
         </is>
+      </c>
+      <c r="D68" t="n">
+        <v>0.1</v>
       </c>
       <c r="F68" t="inlineStr">
         <is>
@@ -82478,6 +82580,19 @@
           <t>SI_REDUCE</t>
         </is>
       </c>
+      <c r="B6" s="8" t="n">
+        <v>5</v>
+      </c>
+      <c r="C6" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="D6" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
       <c r="E6" t="inlineStr">
         <is>
           <t>present</t>
@@ -82562,6 +82677,9 @@
         <is>
           <t>SI_REDUCE</t>
         </is>
+      </c>
+      <c r="D12" t="n">
+        <v>1.924</v>
       </c>
       <c r="F12" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Regenerate outputs for the rectifier trim heaters at rated load (batch 14)
The plant bus demand rises from 179.72 to 216.27 kW: the trim heaters add
23.26 kW and the extension hall that roofs the larger array adds 13.29 kW.
The array, storage, inverters and bus section rating follow. Change note
docs-authority/notes/2026-10-29-rewrite-batch-14.md; REWRITE_TODO Rev Q.
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 307200ce85a4b6e4ac802b198b2b61760112d5af88cc7956debf461181d0cd08</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 d47de7a2485991ce88edfc3bea99d6f9cb52c9dd2571e4c64069c2ec36446466</t>
         </is>
       </c>
     </row>
@@ -18270,7 +18270,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>68.2838</v>
+        <v>81.57170000000001</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -18396,7 +18396,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>336.8116</v>
+        <v>350.0995</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -18497,7 +18497,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>179.7238</v>
+        <v>216.2717</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -19182,7 +19182,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>336.8116</v>
+        <v>350.0995</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -19864,7 +19864,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>755.229337</v>
+        <v>908.809619</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -19894,7 +19894,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>755.229337</v>
+        <v>908.809619</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -20524,7 +20524,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>68.2838</v>
+        <v>81.57170000000001</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -56595,7 +56595,7 @@
         <v>10</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>600.8274</v>
+        <v>663.9511</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -56634,7 +56634,7 @@
         <v>4</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>80.2838</v>
+        <v>93.57170000000001</v>
       </c>
       <c r="I58" t="n">
         <v>2</v>
@@ -56673,7 +56673,7 @@
         <v>1</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>68.2838</v>
+        <v>81.57170000000001</v>
       </c>
       <c r="I59" t="n">
         <v>1</v>
@@ -56829,7 +56829,7 @@
         <v>3</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>340.8198</v>
+        <v>354.1077</v>
       </c>
       <c r="I63" t="n">
         <v>3</v>
@@ -56946,7 +56946,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>336.8116</v>
+        <v>350.0995</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -56985,7 +56985,7 @@
         <v>3</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>179.7238</v>
+        <v>216.2717</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
@@ -57063,7 +57063,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="5" t="n">
-        <v>179.7238</v>
+        <v>216.2717</v>
       </c>
       <c r="I69" t="n">
         <v>1</v>
@@ -64798,7 +64798,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>179.72</v>
+        <v>216.27</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -64812,7 +64812,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 29x23 bays, ext 68.28 kW).</t>
+          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 38x21 bays, ext 81.57 kW).</t>
         </is>
       </c>
     </row>
@@ -64828,7 +64828,7 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>449.31</v>
+        <v>540.6799999999999</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -64873,7 +64873,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>4984</v>
+        <v>5998</v>
       </c>
     </row>
     <row r="6">
@@ -64903,7 +64903,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -64974,7 +64974,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>336.8116</v>
+        <v>350.0995</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -64999,7 +64999,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>179.7238</v>
+        <v>216.2717</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -65102,7 +65102,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>4984</v>
+        <v>5998</v>
       </c>
     </row>
     <row r="19">
@@ -65117,7 +65117,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>2492</v>
+        <v>2999</v>
       </c>
     </row>
     <row r="20">
@@ -65132,7 +65132,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>21986</v>
+        <v>26315</v>
       </c>
     </row>
     <row r="21">
@@ -65147,7 +65147,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1246</v>
+        <v>1500</v>
       </c>
     </row>
     <row r="22">
@@ -65177,7 +65177,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>817</v>
+        <v>984</v>
       </c>
     </row>
     <row r="24">
@@ -65192,7 +65192,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>2517</v>
+        <v>3028</v>
       </c>
     </row>
     <row r="25">
@@ -65207,7 +65207,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>817</v>
+        <v>984</v>
       </c>
     </row>
     <row r="26">
@@ -65222,7 +65222,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>180</v>
+        <v>217</v>
       </c>
     </row>
     <row r="27">
@@ -65237,7 +65237,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2100</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="28">
@@ -65252,7 +65252,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>35</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29">
@@ -65282,7 +65282,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>1920.3</v>
+        <v>2303.7</v>
       </c>
     </row>
     <row r="31">

</xml_diff>

<commit_message>
Argon blanket gas for the CZ puller from the cold box in a closed loop; nitrogen refused for the melt (owner decision 2026-10-29, A-M-417)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 71bd267d2e8a5147eac04cbd777a3e2f1d7c2b2257a9e3b2ff987d35d89e0a20</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 b4b60a03b5946476c11f673c7a2d945019a336132256141029114900c0b12762</t>
         </is>
       </c>
     </row>
@@ -3186,7 +3186,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -3810,21 +3810,21 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>IA-BMED-01</t>
+          <t>IA-AR-CZ</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>WS_NITRIC</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>1.2456</v>
+        <v>0.535819</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -3840,21 +3840,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>IA-BMED-02</t>
+          <t>IA-AR-CZ-BACK</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>BMED_BASE</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>WS_KOH</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.2701</v>
+        <v>0.535819</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -3870,21 +3870,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IA-FAB-KERF</t>
+          <t>IA-BMED-01</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>WS_NITRIC</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.08745799999999999</v>
+        <v>1.2456</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -3900,21 +3900,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IA-FAB-LOSS</t>
+          <t>IA-BMED-02</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>BMED_BASE</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>BAGHOUSE</t>
+          <t>WS_KOH</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.51</v>
+        <v>0.2701</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -3930,7 +3930,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IA-FAB-PRODUCT</t>
+          <t>IA-FAB-KERF</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -3940,11 +3940,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.138904</v>
+        <v>0.08745799999999999</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -3960,7 +3960,7 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IA-FAB-SPENT</t>
+          <t>IA-FAB-LOSS</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
@@ -3970,11 +3970,11 @@
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BAGHOUSE</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>66.502511</v>
+        <v>0.51</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -3990,7 +3990,7 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IA-FAB-WAFER</t>
+          <t>IA-FAB-PRODUCT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
@@ -4000,7 +4000,7 @@
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>LITHO_COAT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D30" t="n">
@@ -4020,21 +4020,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IA-H2O2-SRC</t>
+          <t>IA-FAB-SPENT</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>HDR_O2</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>WS_PEROX</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>0.176</v>
+        <v>66.502511</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -4050,21 +4050,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IA-HF-PROD</t>
+          <t>IA-FAB-WAFER</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>HF_GEN</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>WS_HF_ED</t>
+          <t>LITHO_COAT</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>1.5</v>
+        <v>0.138904</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -4080,21 +4080,21 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IA-LITHO-CARRY</t>
+          <t>IA-H2O2-SRC</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>LITHO_COAT</t>
+          <t>HDR_O2</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>LITHO_DEV</t>
+          <t>WS_PEROX</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>0.987499</v>
+        <v>0.176</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -4110,21 +4110,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IA-LITHO-IN</t>
+          <t>IA-HF-PROD</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>HF_GEN</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>LITHO_COAT</t>
+          <t>WS_HF_ED</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.987499</v>
+        <v>1.5</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -4140,17 +4140,17 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IA-LITHO-OUT</t>
+          <t>IA-LITHO-CARRY</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
+          <t>LITHO_COAT</t>
+        </is>
+      </c>
+      <c r="C35" t="inlineStr">
+        <is>
           <t>LITHO_DEV</t>
-        </is>
-      </c>
-      <c r="C35" t="inlineStr">
-        <is>
-          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D35" t="n">
@@ -4170,21 +4170,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IA-LITHO-WAFER-A</t>
+          <t>IA-LITHO-IN</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
+          <t>WAFER_FAB</t>
+        </is>
+      </c>
+      <c r="C36" t="inlineStr">
+        <is>
           <t>LITHO_COAT</t>
         </is>
       </c>
-      <c r="C36" t="inlineStr">
-        <is>
-          <t>LITHO_ALIGN</t>
-        </is>
-      </c>
       <c r="D36" t="n">
-        <v>0.138904</v>
+        <v>0.987499</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -4200,21 +4200,21 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IA-LITHO-WAFER-B</t>
+          <t>IA-LITHO-OUT</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LITHO_ALIGN</t>
+          <t>LITHO_DEV</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>LITHO_DEV</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.138904</v>
+        <v>0.987499</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -4230,17 +4230,17 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-LITHO-WAFER-RET</t>
+          <t>IA-LITHO-WAFER-A</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>LITHO_DEV</t>
+          <t>LITHO_COAT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>LITHO_ALIGN</t>
         </is>
       </c>
       <c r="D38" t="n">
@@ -4260,21 +4260,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IA-NH3-SRC</t>
+          <t>IA-LITHO-WAFER-B</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>HDR_N2</t>
+          <t>LITHO_ALIGN</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>WS_AMMONIA</t>
+          <t>LITHO_DEV</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>3.008739</v>
+        <v>0.138904</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -4290,21 +4290,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IA-NIT-VENT</t>
+          <t>IA-LITHO-WAFER-RET</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>WS_NITRIC</t>
+          <t>LITHO_DEV</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>0.138904</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -4320,21 +4320,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IA-PEROX-H2O</t>
+          <t>IA-NH3-SRC</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>HDR_N2</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>WS_PEROX</t>
+          <t>WS_AMMONIA</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>2.824</v>
+        <v>3.008739</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -4350,21 +4350,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IA-PHOS-DOPE</t>
+          <t>IA-NIT-VENT</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>WS_PHOS</t>
+          <t>WS_NITRIC</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>WS_DOPE</t>
+          <t>NOX_SCRUB</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.01</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -4380,21 +4380,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IA-PHOS-SRC</t>
+          <t>IA-PEROX-H2O</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>WS_PHOS</t>
+          <t>WS_PEROX</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.62</v>
+        <v>2.824</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -4410,17 +4410,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IA-PV-IN</t>
+          <t>IA-PHOS-DOPE</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>WS_PHOS</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
           <t>WS_DOPE</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>SOLAR_PV_CELL</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -4440,21 +4440,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IA-PV-OUT</t>
+          <t>IA-PHOS-SRC</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>SOLAR_PV_CELL</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WS_PHOS</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.009998999999999999</v>
+        <v>0.62</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -4470,21 +4470,21 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IA-SIL-SRC</t>
+          <t>IA-PV-IN</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>GLASS_DIGEST</t>
+          <t>WS_DOPE</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>WS_SLURRY</t>
+          <t>SOLAR_PV_CELL</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>3.3</v>
+        <v>0.01</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -4500,21 +4500,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IA-SOLV-MU</t>
+          <t>IA-PV-OUT</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>SOLAR_PV_CELL</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>WS_SOLV</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.209973</v>
+        <v>0.009998999999999999</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -4530,21 +4530,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IA-SOLV-WB</t>
+          <t>IA-SIL-SRC</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>WS_SOLV</t>
+          <t>GLASS_DIGEST</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>WS_SLURRY</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.209973</v>
+        <v>3.3</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -4560,21 +4560,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IA-UPW-FAB</t>
+          <t>IA-SOLV-MU</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>FAB_UPW_TANK</t>
+          <t>WS_SOLV</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>60.000181</v>
+        <v>0.209973</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -4590,21 +4590,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IA-UPW-USE</t>
+          <t>IA-SOLV-WB</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HDR_UPW</t>
+          <t>WS_SOLV</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>66.500213</v>
+        <v>0.209973</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -4620,21 +4620,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POLY_TO_FAB</t>
+          <t>IA-UPW-FAB</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>POLY_STOCK</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>FAB_UPW_TANK</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>60.000181</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -4650,12 +4650,12 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>IA-UPW-USE</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CRYO_N2</t>
+          <t>HDR_UPW</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
@@ -4664,7 +4664,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>1.499799</v>
+        <v>66.500213</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -4680,21 +4680,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>POLY_TO_FAB</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>9.277184</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -4710,21 +4710,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>79.11577699999999</v>
+        <v>1.499799</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -4740,12 +4740,12 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S27</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>FAB_UPW_TANK</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
@@ -4754,7 +4754,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>60.000181</v>
+        <v>9.277184</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -4770,21 +4770,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S31</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>WS_HF_ED</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>1.5</v>
+        <v>79.11577699999999</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -4800,12 +4800,12 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S32</t>
+          <t>S27</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>WS_PEROX</t>
+          <t>FAB_UPW_TANK</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
@@ -4814,7 +4814,7 @@
         </is>
       </c>
       <c r="D57" t="n">
-        <v>3</v>
+        <v>60.000181</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -4830,12 +4830,12 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S33</t>
+          <t>S31</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>WS_AMMONIA</t>
+          <t>WS_HF_ED</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
@@ -4844,7 +4844,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>3.008739</v>
+        <v>1.5</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -4860,12 +4860,12 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S34</t>
+          <t>S32</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>WS_NITRIC</t>
+          <t>WS_PEROX</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
@@ -4874,7 +4874,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>1.2456</v>
+        <v>3</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -4890,12 +4890,12 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S34B</t>
+          <t>S33</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>WS_PHOS</t>
+          <t>WS_AMMONIA</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
@@ -4904,7 +4904,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.61</v>
+        <v>3.008739</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -4920,12 +4920,12 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S35</t>
+          <t>S34</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>WS_KOH</t>
+          <t>WS_NITRIC</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
@@ -4934,7 +4934,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.2701</v>
+        <v>1.2456</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -4950,21 +4950,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S36</t>
+          <t>S34B</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>WS_DOPE</t>
+          <t>WS_PHOS</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0</v>
+        <v>0.61</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -4980,21 +4980,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S37</t>
+          <t>S35</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>WS_SLURRY</t>
+          <t>WS_KOH</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>3.3</v>
+        <v>0.2701</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -5010,21 +5010,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S36</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>WS_DOPE</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -5040,21 +5040,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S37</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
+          <t>WS_SLURRY</t>
+        </is>
+      </c>
+      <c r="C65" t="inlineStr">
+        <is>
           <t>WAFER_FAB</t>
         </is>
       </c>
-      <c r="C65" t="inlineStr">
-        <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
       <c r="D65" t="n">
-        <v>3.310001</v>
+        <v>3.3</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -5070,12 +5070,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S39B</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -5084,7 +5084,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -5100,25 +5100,25 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>SF-LITHO_ALIGN</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>LITHO_ALIGN</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.004</v>
+        <v>3.310001</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F67" t="inlineStr">
@@ -5130,25 +5130,25 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>SF-LITHO_COAT</t>
+          <t>S39B</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>LITHO_COAT</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.0254</v>
+        <v>0</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F68" t="inlineStr">
@@ -5160,7 +5160,7 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SF-LITHO_DEV</t>
+          <t>SF-LITHO_ALIGN</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
@@ -5170,11 +5170,11 @@
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>LITHO_DEV</t>
+          <t>LITHO_ALIGN</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.008</v>
+        <v>0.004</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -5190,7 +5190,7 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>SF-LITHO_STUB</t>
+          <t>SF-LITHO_COAT</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
@@ -5200,11 +5200,11 @@
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>LITHO_STUB</t>
+          <t>LITHO_COAT</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0</v>
+        <v>0.0254</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -5220,7 +5220,7 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SF-SOLAR_PV_CELL</t>
+          <t>SF-LITHO_DEV</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -5230,11 +5230,11 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>SOLAR_PV_CELL</t>
+          <t>LITHO_DEV</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.3917</v>
+        <v>0.008</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -5250,7 +5250,7 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SF-WAFER_FAB</t>
+          <t>SF-LITHO_STUB</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
@@ -5260,11 +5260,11 @@
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>LITHO_STUB</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.4069</v>
+        <v>0</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SF-WET_BENCH</t>
+          <t>SF-SOLAR_PV_CELL</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -5290,11 +5290,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>SOLAR_PV_CELL</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.2066</v>
+        <v>0.3917</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -5310,12 +5310,12 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>STOCK_TO_FAB</t>
+          <t>SF-WAFER_FAB</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
-          <t>METAL_STORE</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C74" t="inlineStr">
@@ -5324,11 +5324,11 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.226363</v>
+        <v>0.4069</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F74" t="inlineStr">
@@ -5340,20 +5340,80 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>SF-WET_BENCH</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>WET_BENCH</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0.2066</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>STOCK_TO_FAB</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>METAL_STORE</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>WAFER_FAB</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>0.226363</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
           <t>UPW_TO_FAB</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>HDR_UPW</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>FAB_UPW_TANK</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>null</t>
         </is>
@@ -14002,7 +14062,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H75"/>
+  <dimension ref="A1:H77"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -14657,7 +14717,7 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>IA-ASU-CO2</t>
+          <t>IA-AR-CZ</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
@@ -14667,11 +14727,11 @@
       </c>
       <c r="C26" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D26" t="n">
-        <v>21.581514</v>
+        <v>0.535819</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -14687,21 +14747,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>IA-ASU-N2</t>
+          <t>IA-AR-CZ-BACK</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
+          <t>WAFER_FAB</t>
+        </is>
+      </c>
+      <c r="C27" t="inlineStr">
+        <is>
           <t>CRYO_ASU</t>
         </is>
       </c>
-      <c r="C27" t="inlineStr">
-        <is>
-          <t>CRYO_N2</t>
-        </is>
-      </c>
       <c r="D27" t="n">
-        <v>196.588594</v>
+        <v>0.535819</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -14717,7 +14777,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>IA-ASU-O2</t>
+          <t>IA-ASU-CO2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -14727,11 +14787,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.063683</v>
+        <v>21.581514</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -14747,21 +14807,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>IA-BED-VAP</t>
+          <t>IA-ASU-N2</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="C29" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="D29" t="n">
-        <v>67.443215</v>
+        <v>196.588594</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -14777,21 +14837,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>IA-CO2-RET</t>
+          <t>IA-ASU-O2</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0</v>
+        <v>0.063683</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -14807,21 +14867,21 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>IA-ELY-H2</t>
+          <t>IA-BED-VAP</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>H2O_ELYZ</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="D31" t="n">
-        <v>9.357675</v>
+        <v>67.443215</v>
       </c>
       <c r="E31" t="inlineStr">
         <is>
@@ -14837,21 +14897,21 @@
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>IA-ELY-H2O</t>
+          <t>IA-CO2-RET</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
         <is>
-          <t>H2O_ELYZ</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D32" t="n">
-        <v>83.620295</v>
+        <v>0</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -14867,7 +14927,7 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>IA-ELY-O2</t>
+          <t>IA-ELY-H2</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
@@ -14877,11 +14937,11 @@
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>CRYO_H2</t>
         </is>
       </c>
       <c r="D33" t="n">
-        <v>74.26262</v>
+        <v>9.357675</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -14897,21 +14957,21 @@
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>IA-H2-AIR</t>
+          <t>IA-ELY-H2O</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
         <is>
-          <t>H2_DRYER</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>H2O_ELYZ</t>
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>83.620295</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -14927,21 +14987,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>IA-HAB-VAP</t>
+          <t>IA-ELY-O2</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>H2O_ELYZ</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0</v>
+        <v>74.26262</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -14957,21 +15017,21 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>IA-HVAC-COND</t>
+          <t>IA-H2-AIR</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>H2_DRYER</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
         <is>
-          <t>ROOF_TANK</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D36" t="n">
-        <v>67.443215</v>
+        <v>0</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -14987,17 +15047,17 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IA-LEACH-ASU</t>
+          <t>IA-HAB-VAP</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="D37" t="n">
@@ -15017,21 +15077,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-MEOH-PROD</t>
+          <t>IA-HVAC-COND</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>MEOH_TANK</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>PROD_MEOH</t>
+          <t>ROOF_TANK</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>28.028914</v>
+        <v>67.443215</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -15047,21 +15107,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IA-MEOH-SHIP</t>
+          <t>IA-LEACH-ASU</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>PROD_MEOH</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>28.028914</v>
+        <v>0</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -15077,21 +15137,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IA-N2-RET</t>
+          <t>IA-MEOH-PROD</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>HDR_N2</t>
+          <t>MEOH_TANK</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>PROD_MEOH</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>28.028914</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -15107,12 +15167,12 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IA-N2-VENT</t>
+          <t>IA-MEOH-SHIP</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>CRYO_N2</t>
+          <t>PROD_MEOH</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
@@ -15121,7 +15181,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>3.09978</v>
+        <v>28.028914</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -15137,12 +15197,12 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IA-NOX-CO2</t>
+          <t>IA-N2-RET</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>HDR_N2</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
@@ -15151,7 +15211,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>21.581514</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -15167,21 +15227,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IA-NOX-N2</t>
+          <t>IA-N2-VENT</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>NOX_SCRUB</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>196.652277</v>
+        <v>3.09978</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -15197,21 +15257,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IA-O2-MAKE</t>
+          <t>IA-NOX-CO2</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>NOX_SCRUB</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>HDR_O2</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>21.581514</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -15227,21 +15287,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IA-O2-PROD</t>
+          <t>IA-NOX-N2</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>HDR_O2</t>
+          <t>NOX_SCRUB</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>PROD_O2</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>22.884294</v>
+        <v>196.652277</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -15257,17 +15317,17 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IA-O2-RET</t>
+          <t>IA-O2-MAKE</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
+          <t>CRYO_O2</t>
+        </is>
+      </c>
+      <c r="C46" t="inlineStr">
+        <is>
           <t>HDR_O2</t>
-        </is>
-      </c>
-      <c r="C46" t="inlineStr">
-        <is>
-          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D46" t="n">
@@ -15287,17 +15347,17 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IA-O2-SHIP</t>
+          <t>IA-O2-PROD</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
+          <t>HDR_O2</t>
+        </is>
+      </c>
+      <c r="C47" t="inlineStr">
+        <is>
           <t>PROD_O2</t>
-        </is>
-      </c>
-      <c r="C47" t="inlineStr">
-        <is>
-          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D47" t="n">
@@ -15317,21 +15377,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>S02</t>
+          <t>IA-O2-RET</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>HDR_O2</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>3.4</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -15347,21 +15407,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>S03</t>
+          <t>IA-O2-SHIP</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>CRYO_N2</t>
+          <t>PROD_O2</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>1.499799</v>
+        <v>22.884294</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -15377,21 +15437,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>S04</t>
+          <t>S02</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -15407,21 +15467,21 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>S18</t>
+          <t>S03</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0</v>
+        <v>1.499799</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -15437,21 +15497,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>S45</t>
+          <t>S04</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>BACKUP_GEN</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.019728</v>
+        <v>0</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -15467,21 +15527,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>S49</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>4.8</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -15497,21 +15557,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>S50</t>
+          <t>S45</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>CRYO_H2</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FUEL_CELL</t>
+          <t>BACKUP_GEN</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>38.4</v>
+        <v>0.019728</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -15527,25 +15587,25 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>S54</t>
+          <t>S49</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>CRYO_HX_Q4</t>
+          <t>CRYO_H2</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.5448</v>
+        <v>4.8</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F55" t="inlineStr">
@@ -15557,25 +15617,25 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>S55</t>
+          <t>S50</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>CRYO_DED_COOL</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>CRYO_DED_COOL</t>
+          <t>FUEL_CELL</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>4.2838</v>
+        <v>38.4</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F56" t="inlineStr">
@@ -15587,25 +15647,25 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>S56</t>
+          <t>S54</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>CRYO_HX_Q4</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>RELIEF_CRYO</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0</v>
+        <v>0.5448</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F57" t="inlineStr">
@@ -15617,51 +15677,51 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>S64</t>
+          <t>S55</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>H2_DRYER</t>
+          <t>CRYO_DED_COOL</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>CRYO_DED_COOL</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>1.975408</v>
+        <v>4.2838</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F58" t="inlineStr">
         <is>
-          <t>authority</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>S67B</t>
+          <t>S56</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>FLUE_KO</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>RELIEF_CRYO</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>14.050492</v>
+        <v>0</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -15677,21 +15737,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>S68</t>
+          <t>S64</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>H2_DRYER</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>CRYO_H2</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>78.98790099999999</v>
+        <v>1.975408</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -15700,28 +15760,28 @@
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>authority</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>S70</t>
+          <t>S67B</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>CRYO_AHU_COND_CONDENSABLE</t>
+          <t>FLUE_KO</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>FLUE_KO</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.0521</v>
+        <v>14.050492</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -15737,21 +15797,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>S73</t>
+          <t>S68</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>MEOH_SYNTH</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>44.257647</v>
+        <v>78.98790099999999</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -15767,21 +15827,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S74</t>
+          <t>S70</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>CRYO_AHU_COND_CONDENSABLE</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>MEOH_SYNTH</t>
+          <t>FLUE_KO</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>6.513355</v>
+        <v>0.0521</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -15797,21 +15857,21 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S82</t>
+          <t>S73</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
-          <t>MEOH_FC</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>MEOH_SYNTH</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>8.625641</v>
+        <v>44.257647</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -15827,21 +15887,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S83</t>
+          <t>S74</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>CRYO_H2</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>HDR_O2</t>
+          <t>MEOH_SYNTH</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>33.167875</v>
+        <v>6.513355</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -15857,21 +15917,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S84</t>
+          <t>S82</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>CRYO_N2</t>
+          <t>MEOH_FC</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
         <is>
-          <t>AIR_RECEIVER</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="D66" t="n">
-        <v>191.989014</v>
+        <v>8.625641</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -15887,21 +15947,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S85</t>
+          <t>S83</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>CRYO_CO2</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HDR_CO2</t>
+          <t>HDR_O2</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0</v>
+        <v>33.167875</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -15917,21 +15977,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S86</t>
+          <t>S84</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>RELIEF_CRYO</t>
+          <t>AIR_RECEIVER</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>191.989014</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -15947,21 +16007,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>S87</t>
+          <t>S85</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>CRYO_O2</t>
+          <t>HDR_CO2</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.641572</v>
+        <v>0</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -15977,17 +16037,17 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>S88</t>
+          <t>S86</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>CRYO_N2</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>RELIEF_CRYO</t>
         </is>
       </c>
       <c r="D70" t="n">
@@ -16007,25 +16067,25 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>SF-CRYO_AHU</t>
+          <t>S87</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>CRYO_O2</t>
         </is>
       </c>
       <c r="D71" t="n">
-        <v>0.6472</v>
+        <v>0.641572</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -16037,25 +16097,25 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>SF-CRYO_ASU</t>
+          <t>S88</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>CRYO_N2</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
         <is>
-          <t>CRYO_ASU</t>
+          <t>GROW_BED</t>
         </is>
       </c>
       <c r="D72" t="n">
-        <v>1.6572</v>
+        <v>0</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F72" t="inlineStr">
@@ -16067,7 +16127,7 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>SF-CRYO_H2</t>
+          <t>SF-CRYO_AHU</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
@@ -16077,11 +16137,11 @@
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>CRYO_H2</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.9325</v>
+        <v>0.6472</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -16097,7 +16157,7 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>SF-H2O_ELYZ</t>
+          <t>SF-CRYO_ASU</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
@@ -16107,11 +16167,11 @@
       </c>
       <c r="C74" t="inlineStr">
         <is>
-          <t>H2O_ELYZ</t>
+          <t>CRYO_ASU</t>
         </is>
       </c>
       <c r="D74" t="n">
-        <v>21.4447</v>
+        <v>1.6572</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -16127,28 +16187,88 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
+          <t>SF-CRYO_H2</t>
+        </is>
+      </c>
+      <c r="B75" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C75" t="inlineStr">
+        <is>
+          <t>CRYO_H2</t>
+        </is>
+      </c>
+      <c r="D75" t="n">
+        <v>0.9325</v>
+      </c>
+      <c r="E75" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F75" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" t="inlineStr">
+        <is>
+          <t>SF-H2O_ELYZ</t>
+        </is>
+      </c>
+      <c r="B76" t="inlineStr">
+        <is>
+          <t>SOL_ARK_60K</t>
+        </is>
+      </c>
+      <c r="C76" t="inlineStr">
+        <is>
+          <t>H2O_ELYZ</t>
+        </is>
+      </c>
+      <c r="D76" t="n">
+        <v>21.4447</v>
+      </c>
+      <c r="E76" t="inlineStr">
+        <is>
+          <t>kW</t>
+        </is>
+      </c>
+      <c r="F76" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="77">
+      <c r="A77" t="inlineStr">
+        <is>
           <t>SQ-H2O_ELYZ-Q4</t>
         </is>
       </c>
-      <c r="B75" t="inlineStr">
+      <c r="B77" t="inlineStr">
         <is>
           <t>H2O_ELYZ</t>
         </is>
       </c>
-      <c r="C75" t="inlineStr">
+      <c r="C77" t="inlineStr">
         <is>
           <t>Q4_BUS</t>
         </is>
       </c>
-      <c r="D75" t="n">
+      <c r="D77" t="n">
         <v>6.0825</v>
       </c>
-      <c r="E75" t="inlineStr">
+      <c r="E77" t="inlineStr">
         <is>
           <t>kW</t>
         </is>
       </c>
-      <c r="F75" t="inlineStr">
+      <c r="F77" t="inlineStr">
         <is>
           <t>study</t>
         </is>

</xml_diff>

<commit_message>
Standby route STOCK_TO_WIRE_DRAW sized at its rated case: the S57 copper feed for a MET_MELT outage, held in METAL_STORE (X-RTE, A-M-418)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -33,7 +33,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="DOCK" sheetId="24" state="visible" r:id="rId24"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DRIVERS'!$A$1:$L$866</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="1" hidden="1">'DRIVERS'!$A$1:$L$867</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="2" hidden="1">'TREE'!$A$1:$J$267</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="5" hidden="1">'DIGESTER'!$A$1:$H$26</definedName>
     <definedName name="_xlnm._FilterDatabase" localSheetId="6" hidden="1">'OIL'!$A$1:$H$15</definedName>
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 f020ca1e16e04ee50b378e442662905fba33e011c49bc4afa48dbf479c685e94</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 0a6171692e496fed2714827b117d16e723525197f95cf062bf100527ff419f9f</t>
         </is>
       </c>
     </row>
@@ -698,7 +698,7 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>all 865 drivers.json keys sorted by dotted path; value/units/ref/register/needs_verification/verification_test + the tree-path split columns</t>
+          <t>all 866 drivers.json keys sorted by dotted path; value/units/ref/register/needs_verification/verification_test + the tree-path split columns</t>
         </is>
       </c>
     </row>
@@ -22259,7 +22259,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:L866"/>
+  <dimension ref="A1:L867"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="46" customWidth="1" min="1" max="1"/>
@@ -48856,93 +48856,93 @@
     <row r="816">
       <c r="A816" t="inlineStr">
         <is>
-          <t>storage.default_no_heat_input_T_C</t>
+          <t>standby_outage_d</t>
         </is>
       </c>
       <c r="B816" s="4" t="n">
-        <v>40</v>
+        <v>2</v>
       </c>
       <c r="C816" t="inlineStr">
         <is>
-          <t>C</t>
+          <t>d outage of a primary unit that a standby feed route covers; the N+1 outage basis of the foundry melt backups (A-M-283)</t>
         </is>
       </c>
       <c r="E816" t="inlineStr">
         <is>
-          <t>A-M-269</t>
-        </is>
-      </c>
-      <c r="F816" t="b">
-        <v>1</v>
-      </c>
-      <c r="G816" t="inlineStr">
-        <is>
-          <t>0.4% site dry bulb 37.8 C (AQS-SITE-002) rounded up - confirm as the default</t>
-        </is>
-      </c>
-      <c r="H816" t="inlineStr">
-        <is>
-          <t>storage</t>
-        </is>
-      </c>
-      <c r="I816" t="inlineStr">
-        <is>
-          <t>default_no_heat_input_T_C</t>
+          <t>A-M-418</t>
         </is>
       </c>
     </row>
     <row r="817">
       <c r="A817" t="inlineStr">
         <is>
-          <t>storage_envelope_allowance_mm</t>
+          <t>storage.default_no_heat_input_T_C</t>
         </is>
       </c>
       <c r="B817" s="4" t="n">
-        <v>300</v>
+        <v>40</v>
       </c>
       <c r="C817" t="inlineStr">
         <is>
-          <t>mm access allowance on plan and height around the sized vessel</t>
+          <t>C</t>
         </is>
       </c>
       <c r="E817" t="inlineStr">
         <is>
-          <t>A-M-225 (sized vessel + 300 mm access becomes the unit envelope)</t>
+          <t>A-M-269</t>
+        </is>
+      </c>
+      <c r="F817" t="b">
+        <v>1</v>
+      </c>
+      <c r="G817" t="inlineStr">
+        <is>
+          <t>0.4% site dry bulb 37.8 C (AQS-SITE-002) rounded up - confirm as the default</t>
+        </is>
+      </c>
+      <c r="H817" t="inlineStr">
+        <is>
+          <t>storage</t>
+        </is>
+      </c>
+      <c r="I817" t="inlineStr">
+        <is>
+          <t>default_no_heat_input_T_C</t>
         </is>
       </c>
     </row>
     <row r="818">
       <c r="A818" t="inlineStr">
         <is>
-          <t>storage_pe_min_wall_mm</t>
+          <t>storage_envelope_allowance_mm</t>
         </is>
       </c>
       <c r="B818" s="4" t="n">
-        <v>4.75</v>
+        <v>300</v>
       </c>
       <c r="C818" t="inlineStr">
         <is>
-          <t>mm minimum PE wall (0.187 in)</t>
-        </is>
-      </c>
-      <c r="D818" t="inlineStr">
-        <is>
-          <t>ASTM_D1998</t>
+          <t>mm access allowance on plan and height around the sized vessel</t>
+        </is>
+      </c>
+      <c r="E818" t="inlineStr">
+        <is>
+          <t>A-M-225 (sized vessel + 300 mm access becomes the unit envelope)</t>
         </is>
       </c>
     </row>
     <row r="819">
       <c r="A819" t="inlineStr">
         <is>
-          <t>storage_pe_sd_MPa</t>
+          <t>storage_pe_min_wall_mm</t>
         </is>
       </c>
       <c r="B819" s="4" t="n">
-        <v>4.14</v>
+        <v>4.75</v>
       </c>
       <c r="C819" t="inlineStr">
         <is>
-          <t>MPa PE hydrostatic design stress (SD 600 psi at 23 C)</t>
+          <t>mm minimum PE wall (0.187 in)</t>
         </is>
       </c>
       <c r="D819" t="inlineStr">
@@ -48954,83 +48954,83 @@
     <row r="820">
       <c r="A820" t="inlineStr">
         <is>
-          <t>storage_round_trip</t>
+          <t>storage_pe_sd_MPa</t>
         </is>
       </c>
       <c r="B820" s="4" t="n">
-        <v>0.7</v>
+        <v>4.14</v>
       </c>
       <c r="C820" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="E820" t="inlineStr">
-        <is>
-          <t>A-M-179</t>
-        </is>
-      </c>
-      <c r="F820" t="b">
-        <v>1</v>
-      </c>
-      <c r="G820" t="inlineStr">
-        <is>
-          <t>ZNBR2 in-house stack test (X-MFG-41, AQS-TST-002): round trip at 20 mA/cm2 over the daily cycle; the 0.70 design value is held below the physics prediction until then</t>
+          <t>MPa PE hydrostatic design stress (SD 600 psi at 23 C)</t>
+        </is>
+      </c>
+      <c r="D820" t="inlineStr">
+        <is>
+          <t>ASTM_D1998</t>
         </is>
       </c>
     </row>
     <row r="821">
       <c r="A821" t="inlineStr">
         <is>
-          <t>storage_steel_allow_MPa</t>
+          <t>storage_round_trip</t>
         </is>
       </c>
       <c r="B821" s="4" t="n">
-        <v>115</v>
+        <v>0.7</v>
       </c>
       <c r="C821" t="inlineStr">
         <is>
-          <t>MPa SA-240 304L allowable stress</t>
-        </is>
-      </c>
-      <c r="D821" t="inlineStr">
-        <is>
-          <t>ASME_VIII_1_UG27</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="E821" t="inlineStr">
+        <is>
+          <t>A-M-179</t>
+        </is>
+      </c>
+      <c r="F821" t="b">
+        <v>1</v>
+      </c>
+      <c r="G821" t="inlineStr">
+        <is>
+          <t>ZNBR2 in-house stack test (X-MFG-41, AQS-TST-002): round trip at 20 mA/cm2 over the daily cycle; the 0.70 design value is held below the physics prediction until then</t>
         </is>
       </c>
     </row>
     <row r="822">
       <c r="A822" t="inlineStr">
         <is>
-          <t>storage_steel_min_wall_mm</t>
+          <t>storage_steel_allow_MPa</t>
         </is>
       </c>
       <c r="B822" s="4" t="n">
-        <v>3</v>
+        <v>115</v>
       </c>
       <c r="C822" t="inlineStr">
         <is>
-          <t>mm minimum steel wall</t>
-        </is>
-      </c>
-      <c r="E822" t="inlineStr">
-        <is>
-          <t>A-M-225</t>
+          <t>MPa SA-240 304L allowable stress</t>
+        </is>
+      </c>
+      <c r="D822" t="inlineStr">
+        <is>
+          <t>ASME_VIII_1_UG27</t>
         </is>
       </c>
     </row>
     <row r="823">
       <c r="A823" t="inlineStr">
         <is>
-          <t>storage_tank_HD</t>
+          <t>storage_steel_min_wall_mm</t>
         </is>
       </c>
       <c r="B823" s="4" t="n">
-        <v>1.5</v>
+        <v>3</v>
       </c>
       <c r="C823" t="inlineStr">
         <is>
-          <t>m/m nominal upright cylinder height over diameter</t>
+          <t>mm minimum steel wall</t>
         </is>
       </c>
       <c r="E823" t="inlineStr">
@@ -49042,15 +49042,15 @@
     <row r="824">
       <c r="A824" t="inlineStr">
         <is>
-          <t>storage_tank_fill_frac</t>
+          <t>storage_tank_HD</t>
         </is>
       </c>
       <c r="B824" s="4" t="n">
-        <v>0.8</v>
+        <v>1.5</v>
       </c>
       <c r="C824" t="inlineStr">
         <is>
-          <t>- working volume fraction (20 % freeboard and dead volume)</t>
+          <t>m/m nominal upright cylinder height over diameter</t>
         </is>
       </c>
       <c r="E824" t="inlineStr">
@@ -49062,91 +49062,83 @@
     <row r="825">
       <c r="A825" t="inlineStr">
         <is>
-          <t>struct_equip_density_kg_m3</t>
+          <t>storage_tank_fill_frac</t>
         </is>
       </c>
       <c r="B825" s="4" t="n">
-        <v>150</v>
+        <v>0.8</v>
       </c>
       <c r="C825" t="inlineStr">
         <is>
-          <t>kg/m3 empty equipment weight per envelope volume</t>
+          <t>- working volume fraction (20 % freeboard and dead volume)</t>
         </is>
       </c>
       <c r="E825" t="inlineStr">
         <is>
-          <t>A-M-184</t>
-        </is>
-      </c>
-      <c r="F825" t="b">
-        <v>1</v>
-      </c>
-      <c r="G825" t="inlineStr">
-        <is>
-          <t>Replace with CAD weights per unit as models are built</t>
+          <t>A-M-225</t>
         </is>
       </c>
     </row>
     <row r="826">
       <c r="A826" t="inlineStr">
         <is>
-          <t>struct_op_fill</t>
+          <t>struct_equip_density_kg_m3</t>
         </is>
       </c>
       <c r="B826" s="4" t="n">
-        <v>0.5</v>
+        <v>150</v>
       </c>
       <c r="C826" t="inlineStr">
         <is>
-          <t>- liquid fraction of envelope for liquid units without a stated hold-up</t>
+          <t>kg/m3 empty equipment weight per envelope volume</t>
         </is>
       </c>
       <c r="E826" t="inlineStr">
         <is>
           <t>A-M-184</t>
+        </is>
+      </c>
+      <c r="F826" t="b">
+        <v>1</v>
+      </c>
+      <c r="G826" t="inlineStr">
+        <is>
+          <t>Replace with CAD weights per unit as models are built</t>
         </is>
       </c>
     </row>
     <row r="827">
       <c r="A827" t="inlineStr">
         <is>
-          <t>struct_pv_kg_m2</t>
+          <t>struct_op_fill</t>
         </is>
       </c>
       <c r="B827" s="4" t="n">
-        <v>17</v>
+        <v>0.5</v>
       </c>
       <c r="C827" t="inlineStr">
         <is>
-          <t>kg/m2 PV modules plus ballasted racking on the roof</t>
+          <t>- liquid fraction of envelope for liquid units without a stated hold-up</t>
         </is>
       </c>
       <c r="E827" t="inlineStr">
         <is>
           <t>A-M-184</t>
-        </is>
-      </c>
-      <c r="F827" t="b">
-        <v>1</v>
-      </c>
-      <c r="G827" t="inlineStr">
-        <is>
-          <t>Weigh the in-house module and rack first article</t>
         </is>
       </c>
     </row>
     <row r="828">
       <c r="A828" t="inlineStr">
         <is>
-          <t>struct_tank_kg_m3</t>
+          <t>struct_pv_kg_m2</t>
         </is>
       </c>
       <c r="B828" s="4" t="n">
-        <v>40</v>
+        <v>17</v>
       </c>
       <c r="C828" t="inlineStr">
         <is>
-          <t>kg/m3 empty storage tank weight per envelope volume (thin shell)</t>
+          <t>kg/m2 PV modules plus ballasted racking on the roof</t>
         </is>
       </c>
       <c r="E828" t="inlineStr">
@@ -49159,90 +49151,90 @@
       </c>
       <c r="G828" t="inlineStr">
         <is>
-          <t>CAD weight per tank</t>
+          <t>Weigh the in-house module and rack first article</t>
         </is>
       </c>
     </row>
     <row r="829">
       <c r="A829" t="inlineStr">
         <is>
-          <t>substrate_drain_frac</t>
+          <t>struct_tank_kg_m3</t>
         </is>
       </c>
       <c r="B829" s="4" t="n">
-        <v>0.2</v>
+        <v>40</v>
       </c>
       <c r="C829" t="inlineStr">
         <is>
-          <t>-</t>
-        </is>
-      </c>
-      <c r="D829" t="inlineStr">
-        <is>
-          <t>PLOSONE2017_DRAIN</t>
+          <t>kg/m3 empty storage tank weight per envelope volume (thin shell)</t>
+        </is>
+      </c>
+      <c r="E829" t="inlineStr">
+        <is>
+          <t>A-M-184</t>
+        </is>
+      </c>
+      <c r="F829" t="b">
+        <v>1</v>
+      </c>
+      <c r="G829" t="inlineStr">
+        <is>
+          <t>CAD weight per tank</t>
         </is>
       </c>
     </row>
     <row r="830">
       <c r="A830" t="inlineStr">
         <is>
-          <t>upw_uv_W</t>
+          <t>substrate_drain_frac</t>
         </is>
       </c>
       <c r="B830" s="4" t="n">
-        <v>15</v>
+        <v>0.2</v>
       </c>
       <c r="C830" t="inlineStr">
         <is>
-          <t>W 185/254 nm UV lamp for TOC on the UPW loop</t>
-        </is>
-      </c>
-      <c r="E830" t="inlineStr">
-        <is>
-          <t>A-M-176</t>
+          <t>-</t>
+        </is>
+      </c>
+      <c r="D830" t="inlineStr">
+        <is>
+          <t>PLOSONE2017_DRAIN</t>
         </is>
       </c>
     </row>
     <row r="831">
       <c r="A831" t="inlineStr">
         <is>
-          <t>vent_dP_Pa</t>
+          <t>upw_uv_W</t>
         </is>
       </c>
       <c r="B831" s="4" t="n">
-        <v>500</v>
+        <v>15</v>
       </c>
       <c r="C831" t="inlineStr">
         <is>
-          <t>Pa</t>
+          <t>W 185/254 nm UV lamp for TOC on the UPW loop</t>
         </is>
       </c>
       <c r="E831" t="inlineStr">
         <is>
-          <t>A-M-155</t>
-        </is>
-      </c>
-      <c r="F831" t="b">
-        <v>1</v>
-      </c>
-      <c r="G831" t="inlineStr">
-        <is>
-          <t>see A-M-155</t>
+          <t>A-M-176</t>
         </is>
       </c>
     </row>
     <row r="832">
       <c r="A832" t="inlineStr">
         <is>
-          <t>vent_transfer_h</t>
+          <t>vent_dP_Pa</t>
         </is>
       </c>
       <c r="B832" s="4" t="n">
-        <v>1</v>
+        <v>500</v>
       </c>
       <c r="C832" t="inlineStr">
         <is>
-          <t>h</t>
+          <t>Pa</t>
         </is>
       </c>
       <c r="E832" t="inlineStr">
@@ -49262,20 +49254,20 @@
     <row r="833">
       <c r="A833" t="inlineStr">
         <is>
-          <t>vs_T_C</t>
+          <t>vent_transfer_h</t>
         </is>
       </c>
       <c r="B833" s="4" t="n">
-        <v>40</v>
+        <v>1</v>
       </c>
       <c r="C833" t="inlineStr">
         <is>
-          <t>C, vent condenser outlet</t>
+          <t>h</t>
         </is>
       </c>
       <c r="E833" t="inlineStr">
         <is>
-          <t>A-M-111</t>
+          <t>A-M-155</t>
         </is>
       </c>
       <c r="F833" t="b">
@@ -49283,27 +49275,22 @@
       </c>
       <c r="G833" t="inlineStr">
         <is>
-          <t>Vent condenser outlet temperature at design cooling water</t>
+          <t>see A-M-155</t>
         </is>
       </c>
     </row>
     <row r="834">
       <c r="A834" t="inlineStr">
         <is>
-          <t>vs_a_m2_m3</t>
+          <t>vs_T_C</t>
         </is>
       </c>
       <c r="B834" s="4" t="n">
-        <v>340</v>
+        <v>40</v>
       </c>
       <c r="C834" t="inlineStr">
         <is>
-          <t>m2/m3 specific area of 16 mm rings</t>
-        </is>
-      </c>
-      <c r="D834" t="inlineStr">
-        <is>
-          <t>PERRY9_ABS</t>
+          <t>C, vent condenser outlet</t>
         </is>
       </c>
       <c r="E834" t="inlineStr">
@@ -49316,27 +49303,27 @@
       </c>
       <c r="G834" t="inlineStr">
         <is>
-          <t>Measured ring geometry</t>
+          <t>Vent condenser outlet temperature at design cooling water</t>
         </is>
       </c>
     </row>
     <row r="835">
       <c r="A835" t="inlineStr">
         <is>
-          <t>vs_air_mg_kg</t>
+          <t>vs_a_m2_m3</t>
         </is>
       </c>
       <c r="B835" s="4" t="n">
-        <v>21.7</v>
+        <v>340</v>
       </c>
       <c r="C835" t="inlineStr">
         <is>
-          <t>mg air per kg feed (N2 13.4 + O2 8.3 at 25 C, 101.3 kPa, air-saturated fresh water)</t>
+          <t>m2/m3 specific area of 16 mm rings</t>
         </is>
       </c>
       <c r="D835" t="inlineStr">
         <is>
-          <t>WEISS1970</t>
+          <t>PERRY9_ABS</t>
         </is>
       </c>
       <c r="E835" t="inlineStr">
@@ -49349,73 +49336,78 @@
       </c>
       <c r="G835" t="inlineStr">
         <is>
-          <t>Vent gas flow meter on the column vent during commissioning</t>
+          <t>Measured ring geometry</t>
         </is>
       </c>
     </row>
     <row r="836">
       <c r="A836" t="inlineStr">
         <is>
-          <t>vs_d_over_dp</t>
+          <t>vs_air_mg_kg</t>
         </is>
       </c>
       <c r="B836" s="4" t="n">
-        <v>8</v>
+        <v>21.7</v>
       </c>
       <c r="C836" t="inlineStr">
         <is>
-          <t>column / packing diameter minimum (wall channelling)</t>
+          <t>mg air per kg feed (N2 13.4 + O2 8.3 at 25 C, 101.3 kPa, air-saturated fresh water)</t>
         </is>
       </c>
       <c r="D836" t="inlineStr">
         <is>
-          <t>PERRY9_ABS</t>
+          <t>WEISS1970</t>
+        </is>
+      </c>
+      <c r="E836" t="inlineStr">
+        <is>
+          <t>A-M-111</t>
         </is>
       </c>
       <c r="F836" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G836" t="inlineStr">
+        <is>
+          <t>Vent gas flow meter on the column vent during commissioning</t>
+        </is>
       </c>
     </row>
     <row r="837">
       <c r="A837" t="inlineStr">
         <is>
-          <t>vs_dp_mm</t>
+          <t>vs_d_over_dp</t>
         </is>
       </c>
       <c r="B837" s="4" t="n">
-        <v>16</v>
+        <v>8</v>
       </c>
       <c r="C837" t="inlineStr">
         <is>
-          <t>mm, nominal packing (in-house cut PVC tube rings)</t>
-        </is>
-      </c>
-      <c r="E837" t="inlineStr">
-        <is>
-          <t>A-M-111</t>
+          <t>column / packing diameter minimum (wall channelling)</t>
+        </is>
+      </c>
+      <c r="D837" t="inlineStr">
+        <is>
+          <t>PERRY9_ABS</t>
         </is>
       </c>
       <c r="F837" t="b">
-        <v>1</v>
-      </c>
-      <c r="G837" t="inlineStr">
-        <is>
-          <t>Pressure drop and wetting test on the cut rings</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="838">
       <c r="A838" t="inlineStr">
         <is>
-          <t>vs_margin</t>
+          <t>vs_dp_mm</t>
         </is>
       </c>
       <c r="B838" s="4" t="n">
-        <v>1.5</v>
+        <v>16</v>
       </c>
       <c r="C838" t="inlineStr">
         <is>
-          <t>packed height margin</t>
+          <t>mm, nominal packing (in-house cut PVC tube rings)</t>
         </is>
       </c>
       <c r="E838" t="inlineStr">
@@ -49428,75 +49420,73 @@
       </c>
       <c r="G838" t="inlineStr">
         <is>
-          <t>as vs_htu_m</t>
+          <t>Pressure drop and wetting test on the cut rings</t>
         </is>
       </c>
     </row>
     <row r="839">
       <c r="A839" t="inlineStr">
         <is>
-          <t>vs_mwr</t>
+          <t>vs_margin</t>
         </is>
       </c>
       <c r="B839" s="4" t="n">
-        <v>0.08</v>
+        <v>1.5</v>
       </c>
       <c r="C839" t="inlineStr">
         <is>
-          <t>m3/(m h) minimum wetting rate, packings below 75 mm</t>
-        </is>
-      </c>
-      <c r="D839" t="inlineStr">
-        <is>
-          <t>PERRY9_ABS</t>
+          <t>packed height margin</t>
+        </is>
+      </c>
+      <c r="E839" t="inlineStr">
+        <is>
+          <t>A-M-111</t>
         </is>
       </c>
       <c r="F839" t="b">
-        <v>0</v>
+        <v>1</v>
+      </c>
+      <c r="G839" t="inlineStr">
+        <is>
+          <t>as vs_htu_m</t>
+        </is>
       </c>
     </row>
     <row r="840">
       <c r="A840" t="inlineStr">
         <is>
-          <t>vs_naoh_excess</t>
+          <t>vs_mwr</t>
         </is>
       </c>
       <c r="B840" s="4" t="n">
-        <v>2</v>
+        <v>0.08</v>
       </c>
       <c r="C840" t="inlineStr">
         <is>
-          <t>mol NaOH fed / mol HCl absorbed</t>
-        </is>
-      </c>
-      <c r="E840" t="inlineStr">
-        <is>
-          <t>A-M-111</t>
+          <t>m3/(m h) minimum wetting rate, packings below 75 mm</t>
+        </is>
+      </c>
+      <c r="D840" t="inlineStr">
+        <is>
+          <t>PERRY9_ABS</t>
         </is>
       </c>
       <c r="F840" t="b">
-        <v>1</v>
-      </c>
-      <c r="G840" t="inlineStr">
-        <is>
-          <t>Sump pH above 12 at the bleed rate</t>
-        </is>
+        <v>0</v>
       </c>
     </row>
     <row r="841">
       <c r="A841" t="inlineStr">
         <is>
-          <t>vs_p_shell_case</t>
-        </is>
-      </c>
-      <c r="B841" s="4" t="inlineStr">
-        <is>
-          <t>upset</t>
-        </is>
+          <t>vs_naoh_excess</t>
+        </is>
+      </c>
+      <c r="B841" s="4" t="n">
+        <v>2</v>
       </c>
       <c r="C841" t="inlineStr">
         <is>
-          <t>design case: column bypassed, condensate at the body vapour composition (17.1 wt% HCl); normal case reported</t>
+          <t>mol NaOH fed / mol HCl absorbed</t>
         </is>
       </c>
       <c r="E841" t="inlineStr">
@@ -49509,27 +49499,24 @@
       </c>
       <c r="G841" t="inlineStr">
         <is>
-          <t>Condensate titration during start-up before the column profile forms</t>
+          <t>Sump pH above 12 at the bleed rate</t>
         </is>
       </c>
     </row>
     <row r="842">
       <c r="A842" t="inlineStr">
         <is>
-          <t>vs_y_out_ppm</t>
-        </is>
-      </c>
-      <c r="B842" s="4" t="n">
-        <v>1</v>
+          <t>vs_p_shell_case</t>
+        </is>
+      </c>
+      <c r="B842" s="4" t="inlineStr">
+        <is>
+          <t>upset</t>
+        </is>
       </c>
       <c r="C842" t="inlineStr">
         <is>
-          <t>ppmv HCl at the scrubber outlet (half the ACGIH TLV-C 2 ppm)</t>
-        </is>
-      </c>
-      <c r="D842" t="inlineStr">
-        <is>
-          <t>ACGIH_HCL</t>
+          <t>design case: column bypassed, condensate at the body vapour composition (17.1 wt% HCl); normal case reported</t>
         </is>
       </c>
       <c r="E842" t="inlineStr">
@@ -49542,70 +49529,75 @@
       </c>
       <c r="G842" t="inlineStr">
         <is>
-          <t>Outlet HCl by NIOSH 7903 sampling</t>
+          <t>Condensate titration during start-up before the column profile forms</t>
         </is>
       </c>
     </row>
     <row r="843">
       <c r="A843" t="inlineStr">
         <is>
-          <t>water_cp_kJ_kgK</t>
+          <t>vs_y_out_ppm</t>
         </is>
       </c>
       <c r="B843" s="4" t="n">
-        <v>4.18</v>
+        <v>1</v>
       </c>
       <c r="C843" t="inlineStr">
         <is>
-          <t>kJ/(kg K)</t>
+          <t>ppmv HCl at the scrubber outlet (half the ACGIH TLV-C 2 ppm)</t>
         </is>
       </c>
       <c r="D843" t="inlineStr">
         <is>
-          <t>INCROPERA7</t>
+          <t>ACGIH_HCL</t>
+        </is>
+      </c>
+      <c r="E843" t="inlineStr">
+        <is>
+          <t>A-M-111</t>
+        </is>
+      </c>
+      <c r="F843" t="b">
+        <v>1</v>
+      </c>
+      <c r="G843" t="inlineStr">
+        <is>
+          <t>Outlet HCl by NIOSH 7903 sampling</t>
         </is>
       </c>
     </row>
     <row r="844">
       <c r="A844" t="inlineStr">
         <is>
-          <t>wt_Ie</t>
+          <t>water_cp_kJ_kgK</t>
         </is>
       </c>
       <c r="B844" s="4" t="n">
-        <v>1.5</v>
+        <v>4.18</v>
       </c>
       <c r="C844" t="inlineStr">
         <is>
-          <t>- importance factor, Risk Category IV (life-support energy)</t>
-        </is>
-      </c>
-      <c r="E844" t="inlineStr">
-        <is>
-          <t>A-M-187</t>
-        </is>
-      </c>
-      <c r="F844" t="b">
-        <v>1</v>
-      </c>
-      <c r="G844" t="inlineStr">
-        <is>
-          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
+          <t>kJ/(kg K)</t>
+        </is>
+      </c>
+      <c r="D844" t="inlineStr">
+        <is>
+          <t>INCROPERA7</t>
         </is>
       </c>
     </row>
     <row r="845">
       <c r="A845" t="inlineStr">
         <is>
-          <t>wt_R</t>
+          <t>wt_Ie</t>
         </is>
       </c>
       <c r="B845" s="4" t="n">
-        <v>3</v>
+        <v>1.5</v>
       </c>
       <c r="C845" t="inlineStr">
         <is>
-          <t>- response modification, elevated-mass structure (conservative)</t>
+          <t>- importance factor, Risk Category IV (life-support energy)</t>
         </is>
       </c>
       <c r="E845" t="inlineStr">
@@ -49625,20 +49617,20 @@
     <row r="846">
       <c r="A846" t="inlineStr">
         <is>
-          <t>wt_SD1</t>
+          <t>wt_R</t>
         </is>
       </c>
       <c r="B846" s="4" t="n">
-        <v>0.08</v>
+        <v>3</v>
       </c>
       <c r="C846" t="inlineStr">
         <is>
-          <t>g design 1 s spectral acceleration = 2/3 Fv S1</t>
-        </is>
-      </c>
-      <c r="D846" t="inlineStr">
-        <is>
-          <t>ASCE7_22</t>
+          <t>- response modification, elevated-mass structure (conservative)</t>
+        </is>
+      </c>
+      <c r="E846" t="inlineStr">
+        <is>
+          <t>A-M-187</t>
         </is>
       </c>
       <c r="F846" t="b">
@@ -49646,22 +49638,22 @@
       </c>
       <c r="G846" t="inlineStr">
         <is>
-          <t>ASCE Hazard Tool lookup at the fixed parcel and site class from the geotechnical report (AQS-SITE-002 held)</t>
+          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
         </is>
       </c>
     </row>
     <row r="847">
       <c r="A847" t="inlineStr">
         <is>
-          <t>wt_SDS</t>
+          <t>wt_SD1</t>
         </is>
       </c>
       <c r="B847" s="4" t="n">
-        <v>0.107</v>
+        <v>0.08</v>
       </c>
       <c r="C847" t="inlineStr">
         <is>
-          <t>g design short-period spectral acceleration = 2/3 Fa Ss</t>
+          <t>g design 1 s spectral acceleration = 2/3 Fv S1</t>
         </is>
       </c>
       <c r="D847" t="inlineStr">
@@ -49681,20 +49673,20 @@
     <row r="848">
       <c r="A848" t="inlineStr">
         <is>
-          <t>wt_TL_s</t>
+          <t>wt_SDS</t>
         </is>
       </c>
       <c r="B848" s="4" t="n">
-        <v>8</v>
+        <v>0.107</v>
       </c>
       <c r="C848" t="inlineStr">
         <is>
-          <t>s long-period transition</t>
-        </is>
-      </c>
-      <c r="E848" t="inlineStr">
-        <is>
-          <t>A-M-187</t>
+          <t>g design short-period spectral acceleration = 2/3 Fa Ss</t>
+        </is>
+      </c>
+      <c r="D848" t="inlineStr">
+        <is>
+          <t>ASCE7_22</t>
         </is>
       </c>
       <c r="F848" t="b">
@@ -49702,22 +49694,22 @@
       </c>
       <c r="G848" t="inlineStr">
         <is>
-          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
+          <t>ASCE Hazard Tool lookup at the fixed parcel and site class from the geotechnical report (AQS-SITE-002 held)</t>
         </is>
       </c>
     </row>
     <row r="849">
       <c r="A849" t="inlineStr">
         <is>
-          <t>wt_cell_len_m</t>
+          <t>wt_TL_s</t>
         </is>
       </c>
       <c r="B849" s="4" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="C849" t="inlineStr">
         <is>
-          <t>m max reservoir cell length (sloshing; min 2 cells per level)</t>
+          <t>s long-period transition</t>
         </is>
       </c>
       <c r="E849" t="inlineStr">
@@ -49737,15 +49729,15 @@
     <row r="850">
       <c r="A850" t="inlineStr">
         <is>
-          <t>wt_core_frac</t>
+          <t>wt_cell_len_m</t>
         </is>
       </c>
       <c r="B850" s="4" t="n">
-        <v>0.15</v>
+        <v>12</v>
       </c>
       <c r="C850" t="inlineStr">
         <is>
-          <t>- plate fraction kept for stair, lift and penstock cores</t>
+          <t>m max reservoir cell length (sloshing; min 2 cells per level)</t>
         </is>
       </c>
       <c r="E850" t="inlineStr">
@@ -49765,15 +49757,15 @@
     <row r="851">
       <c r="A851" t="inlineStr">
         <is>
-          <t>wt_freeboard_m</t>
+          <t>wt_core_frac</t>
         </is>
       </c>
       <c r="B851" s="4" t="n">
-        <v>0.5</v>
+        <v>0.15</v>
       </c>
       <c r="C851" t="inlineStr">
         <is>
-          <t>m freeboard, lower reservoir</t>
+          <t>- plate fraction kept for stair, lift and penstock cores</t>
         </is>
       </c>
       <c r="E851" t="inlineStr">
@@ -49793,15 +49785,15 @@
     <row r="852">
       <c r="A852" t="inlineStr">
         <is>
-          <t>wt_level_clear_mm</t>
+          <t>wt_freeboard_m</t>
         </is>
       </c>
       <c r="B852" s="4" t="n">
-        <v>6000</v>
+        <v>0.5</v>
       </c>
       <c r="C852" t="inlineStr">
         <is>
-          <t>mm reservoir storey floor-to-floor</t>
+          <t>m freeboard, lower reservoir</t>
         </is>
       </c>
       <c r="E852" t="inlineStr">
@@ -49821,63 +49813,63 @@
     <row r="853">
       <c r="A853" t="inlineStr">
         <is>
-          <t>wt_life_per_shop</t>
+          <t>wt_level_clear_mm</t>
         </is>
       </c>
       <c r="B853" s="4" t="n">
-        <v>2</v>
+        <v>6000</v>
       </c>
       <c r="C853" t="inlineStr">
         <is>
-          <t>- HAB/FARM levels added per added shop level as the building grows (owner rule, Q-009)</t>
+          <t>mm reservoir storey floor-to-floor</t>
         </is>
       </c>
       <c r="E853" t="inlineStr">
         <is>
           <t>A-M-187</t>
+        </is>
+      </c>
+      <c r="F853" t="b">
+        <v>1</v>
+      </c>
+      <c r="G853" t="inlineStr">
+        <is>
+          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
         </is>
       </c>
     </row>
     <row r="854">
       <c r="A854" t="inlineStr">
         <is>
-          <t>wt_penstock_loss_frac</t>
+          <t>wt_life_per_shop</t>
         </is>
       </c>
       <c r="B854" s="4" t="n">
-        <v>0.05</v>
+        <v>2</v>
       </c>
       <c r="C854" t="inlineStr">
         <is>
-          <t>- penstock friction as fraction of head</t>
+          <t>- HAB/FARM levels added per added shop level as the building grows (owner rule, Q-009)</t>
         </is>
       </c>
       <c r="E854" t="inlineStr">
         <is>
           <t>A-M-187</t>
-        </is>
-      </c>
-      <c r="F854" t="b">
-        <v>1</v>
-      </c>
-      <c r="G854" t="inlineStr">
-        <is>
-          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
         </is>
       </c>
     </row>
     <row r="855">
       <c r="A855" t="inlineStr">
         <is>
-          <t>wt_water_max_m</t>
+          <t>wt_penstock_loss_frac</t>
         </is>
       </c>
       <c r="B855" s="4" t="n">
-        <v>4.5</v>
+        <v>0.05</v>
       </c>
       <c r="C855" t="inlineStr">
         <is>
-          <t>m max water depth per reservoir level (slab load 44 kPa)</t>
+          <t>- penstock friction as fraction of head</t>
         </is>
       </c>
       <c r="E855" t="inlineStr">
@@ -49897,15 +49889,15 @@
     <row r="856">
       <c r="A856" t="inlineStr">
         <is>
-          <t>wt_wind_ms</t>
+          <t>wt_water_max_m</t>
         </is>
       </c>
       <c r="B856" s="4" t="n">
-        <v>50</v>
+        <v>4.5</v>
       </c>
       <c r="C856" t="inlineStr">
         <is>
-          <t>m/s basic wind speed</t>
+          <t>m max water depth per reservoir level (slab load 44 kPa)</t>
         </is>
       </c>
       <c r="E856" t="inlineStr">
@@ -49925,20 +49917,20 @@
     <row r="857">
       <c r="A857" t="inlineStr">
         <is>
-          <t>xfmr_Z_pu</t>
+          <t>wt_wind_ms</t>
         </is>
       </c>
       <c r="B857" s="4" t="n">
-        <v>0.0575</v>
+        <v>50</v>
       </c>
       <c r="C857" t="inlineStr">
         <is>
-          <t>pu pad-mount transformer impedance</t>
-        </is>
-      </c>
-      <c r="D857" t="inlineStr">
-        <is>
-          <t>IEEE_C57_12_34</t>
+          <t>m/s basic wind speed</t>
+        </is>
+      </c>
+      <c r="E857" t="inlineStr">
+        <is>
+          <t>A-M-187</t>
         </is>
       </c>
       <c r="F857" t="b">
@@ -49946,70 +49938,70 @@
       </c>
       <c r="G857" t="inlineStr">
         <is>
-          <t>Transformer nameplate</t>
+          <t>Structural and geotechnical design of the reservoir floors and the site seismic and wind study</t>
         </is>
       </c>
     </row>
     <row r="858">
       <c r="A858" t="inlineStr">
         <is>
-          <t>zeolite5A_CO2_wt_frac</t>
+          <t>xfmr_Z_pu</t>
         </is>
       </c>
       <c r="B858" s="4" t="n">
-        <v>0.01</v>
+        <v>0.0575</v>
       </c>
       <c r="C858" t="inlineStr">
         <is>
-          <t>kg/kg at 0.4 kPa</t>
+          <t>pu pad-mount transformer impedance</t>
         </is>
       </c>
       <c r="D858" t="inlineStr">
         <is>
-          <t>NASA_5A1998</t>
+          <t>IEEE_C57_12_34</t>
+        </is>
+      </c>
+      <c r="F858" t="b">
+        <v>1</v>
+      </c>
+      <c r="G858" t="inlineStr">
+        <is>
+          <t>Transformer nameplate</t>
         </is>
       </c>
     </row>
     <row r="859">
       <c r="A859" t="inlineStr">
         <is>
-          <t>znbr_ASR_ohm_cm2</t>
+          <t>zeolite5A_CO2_wt_frac</t>
         </is>
       </c>
       <c r="B859" s="4" t="n">
-        <v>5</v>
+        <v>0.01</v>
       </c>
       <c r="C859" t="inlineStr">
         <is>
-          <t>ohm cm2 cell area-specific resistance</t>
-        </is>
-      </c>
-      <c r="E859" t="inlineStr">
-        <is>
-          <t>A-M-179</t>
-        </is>
-      </c>
-      <c r="F859" t="b">
-        <v>1</v>
-      </c>
-      <c r="G859" t="inlineStr">
-        <is>
-          <t>ZNBR2 stack test (X-MFG-41, AQS-TST-002)</t>
+          <t>kg/kg at 0.4 kPa</t>
+        </is>
+      </c>
+      <c r="D859" t="inlineStr">
+        <is>
+          <t>NASA_5A1998</t>
         </is>
       </c>
     </row>
     <row r="860">
       <c r="A860" t="inlineStr">
         <is>
-          <t>znbr_aux_frac</t>
+          <t>znbr_ASR_ohm_cm2</t>
         </is>
       </c>
       <c r="B860" s="4" t="n">
-        <v>0.03</v>
+        <v>5</v>
       </c>
       <c r="C860" t="inlineStr">
         <is>
-          <t>- pump and control energy as a fraction of throughput</t>
+          <t>ohm cm2 cell area-specific resistance</t>
         </is>
       </c>
       <c r="E860" t="inlineStr">
@@ -50029,68 +50021,68 @@
     <row r="861">
       <c r="A861" t="inlineStr">
         <is>
-          <t>znbr_cell_V</t>
+          <t>znbr_aux_frac</t>
         </is>
       </c>
       <c r="B861" s="4" t="n">
-        <v>1.82</v>
+        <v>0.03</v>
       </c>
       <c r="C861" t="inlineStr">
         <is>
-          <t>V</t>
-        </is>
-      </c>
-      <c r="D861" t="inlineStr">
-        <is>
-          <t>SAND2000-0893</t>
+          <t>- pump and control energy as a fraction of throughput</t>
+        </is>
+      </c>
+      <c r="E861" t="inlineStr">
+        <is>
+          <t>A-M-179</t>
+        </is>
+      </c>
+      <c r="F861" t="b">
+        <v>1</v>
+      </c>
+      <c r="G861" t="inlineStr">
+        <is>
+          <t>ZNBR2 stack test (X-MFG-41, AQS-TST-002)</t>
         </is>
       </c>
     </row>
     <row r="862">
       <c r="A862" t="inlineStr">
         <is>
-          <t>znbr_charge_h</t>
+          <t>znbr_cell_V</t>
         </is>
       </c>
       <c r="B862" s="4" t="n">
-        <v>6</v>
+        <v>1.82</v>
       </c>
       <c r="C862" t="inlineStr">
         <is>
-          <t>h/d</t>
-        </is>
-      </c>
-      <c r="E862" t="inlineStr">
-        <is>
-          <t>A-M-135</t>
-        </is>
-      </c>
-      <c r="F862" t="b">
-        <v>1</v>
-      </c>
-      <c r="G862" t="inlineStr">
-        <is>
-          <t>see A-M-135</t>
+          <t>V</t>
+        </is>
+      </c>
+      <c r="D862" t="inlineStr">
+        <is>
+          <t>SAND2000-0893</t>
         </is>
       </c>
     </row>
     <row r="863">
       <c r="A863" t="inlineStr">
         <is>
-          <t>znbr_crossover_loss</t>
+          <t>znbr_charge_h</t>
         </is>
       </c>
       <c r="B863" s="4" t="n">
-        <v>0.05</v>
+        <v>6</v>
       </c>
       <c r="C863" t="inlineStr">
         <is>
-          <t>- coulombic loss to Br2 crossover and self-discharge over the day</t>
+          <t>h/d</t>
         </is>
       </c>
       <c r="E863" t="inlineStr">
         <is>
-          <t>A-M-179</t>
+          <t>A-M-135</t>
         </is>
       </c>
       <c r="F863" t="b">
@@ -50098,42 +50090,50 @@
       </c>
       <c r="G863" t="inlineStr">
         <is>
-          <t>ZNBR2 stack test (X-MFG-41, AQS-TST-002)</t>
+          <t>see A-M-135</t>
         </is>
       </c>
     </row>
     <row r="864">
       <c r="A864" t="inlineStr">
         <is>
-          <t>znbr_her_mL_h_cm2</t>
+          <t>znbr_crossover_loss</t>
         </is>
       </c>
       <c r="B864" s="4" t="n">
-        <v>0.055</v>
+        <v>0.05</v>
       </c>
       <c r="C864" t="inlineStr">
         <is>
-          <t>mL/h/cm2 at 20 mA/cm2</t>
-        </is>
-      </c>
-      <c r="D864" t="inlineStr">
-        <is>
-          <t>ZBFB_REVIEW2023</t>
+          <t>- coulombic loss to Br2 crossover and self-discharge over the day</t>
+        </is>
+      </c>
+      <c r="E864" t="inlineStr">
+        <is>
+          <t>A-M-179</t>
+        </is>
+      </c>
+      <c r="F864" t="b">
+        <v>1</v>
+      </c>
+      <c r="G864" t="inlineStr">
+        <is>
+          <t>ZNBR2 stack test (X-MFG-41, AQS-TST-002)</t>
         </is>
       </c>
     </row>
     <row r="865">
       <c r="A865" t="inlineStr">
         <is>
-          <t>znbr_j_mA_cm2</t>
+          <t>znbr_her_mL_h_cm2</t>
         </is>
       </c>
       <c r="B865" s="4" t="n">
-        <v>20</v>
+        <v>0.055</v>
       </c>
       <c r="C865" t="inlineStr">
         <is>
-          <t>mA/cm2</t>
+          <t>mL/h/cm2 at 20 mA/cm2</t>
         </is>
       </c>
       <c r="D865" t="inlineStr">
@@ -50145,25 +50145,45 @@
     <row r="866">
       <c r="A866" t="inlineStr">
         <is>
+          <t>znbr_j_mA_cm2</t>
+        </is>
+      </c>
+      <c r="B866" s="4" t="n">
+        <v>20</v>
+      </c>
+      <c r="C866" t="inlineStr">
+        <is>
+          <t>mA/cm2</t>
+        </is>
+      </c>
+      <c r="D866" t="inlineStr">
+        <is>
+          <t>ZBFB_REVIEW2023</t>
+        </is>
+      </c>
+    </row>
+    <row r="867">
+      <c r="A867" t="inlineStr">
+        <is>
           <t>znbr_oc_corr_mL_h_cm2</t>
         </is>
       </c>
-      <c r="B866" s="4" t="n">
+      <c r="B867" s="4" t="n">
         <v>0.0032</v>
       </c>
-      <c r="C866" t="inlineStr">
+      <c r="C867" t="inlineStr">
         <is>
           <t>mL/h/cm2</t>
         </is>
       </c>
-      <c r="D866" t="inlineStr">
+      <c r="D867" t="inlineStr">
         <is>
           <t>ZBFB_REVIEW2023</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:L866"/>
+  <autoFilter ref="A1:L867"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>

</xml_diff>

<commit_message>
Recover every element first and take raw ore only for the shortfall: recovery records on each ore-taking unit, a generated per-element inventory (AQS-PAR-001 7.2) and a test that flags excess ore; the acid kiln also recovers the free-acid sulfur and the causticiser takes its lime from the acid residue (A-M-423, batch 35)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 048924eca4b2883db6fbe7eefce5ed9897a43874148f64fb223d943967cd6078</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 8a86220e5069046ba1637994dfd0725c4b5bea2473b8b817d64c5a1216f63f06</t>
         </is>
       </c>
     </row>
@@ -6191,7 +6191,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>4.836867</v>
+        <v>4.835643</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -6971,7 +6971,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>11.636366</v>
+        <v>11.635142</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -17074,7 +17074,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.079758</v>
+        <v>0.086872</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -17134,7 +17134,7 @@
         </is>
       </c>
       <c r="D30" t="n">
-        <v>0.08300299999999999</v>
+        <v>0.077462</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -17839,7 +17839,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.487201</v>
+        <v>0.475115</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -20584,7 +20584,7 @@
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.9654</v>
+        <v>0.966</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -21934,7 +21934,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1.1935</v>
+        <v>1.1929</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -55765,7 +55765,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>53.366007</v>
+        <v>53.367231</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -55885,7 +55885,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.29871</v>
+        <v>0.259355</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -55915,7 +55915,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.028933</v>
+        <v>0</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -56215,7 +56215,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.12089</v>
+        <v>0.126417</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -56575,7 +56575,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.018487</v>
+        <v>0.012935</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -57551,7 +57551,7 @@
         <v>26</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>15.6893</v>
+        <v>15.6887</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
@@ -58097,7 +58097,7 @@
         <v>16</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>10.441</v>
+        <v>10.4404</v>
       </c>
       <c r="I35" t="n">
         <v>6</v>
@@ -58136,7 +58136,7 @@
         <v>6</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>9.691000000000001</v>
+        <v>9.6904</v>
       </c>
       <c r="I36" t="n">
         <v>5</v>
@@ -58370,7 +58370,7 @@
         <v>1</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>1.1935</v>
+        <v>1.1929</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
@@ -65715,7 +65715,7 @@
         <v>11</v>
       </c>
       <c r="H232" s="5" t="n">
-        <v>2.3542</v>
+        <v>2.3548</v>
       </c>
       <c r="I232" t="n">
         <v>7</v>
@@ -65754,7 +65754,7 @@
         <v>5</v>
       </c>
       <c r="H233" s="5" t="n">
-        <v>2.2303</v>
+        <v>2.2309</v>
       </c>
       <c r="I233" t="n">
         <v>5</v>
@@ -65793,7 +65793,7 @@
         <v>1</v>
       </c>
       <c r="H234" s="5" t="n">
-        <v>0.9654</v>
+        <v>0.966</v>
       </c>
       <c r="I234" t="n">
         <v>1</v>
@@ -70061,7 +70061,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H199"/>
+  <dimension ref="A1:H200"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -70726,7 +70726,7 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>1.1935</v>
+        <v>1.1929</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -73543,7 +73543,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>53.366007</v>
+        <v>53.367231</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -73979,12 +73979,12 @@
     <row r="136">
       <c r="A136" t="inlineStr">
         <is>
-          <t>IA-LIMESTONE-MU</t>
+          <t>IA-LIME-TO-NAOH</t>
         </is>
       </c>
       <c r="B136" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>ACID_PLANT</t>
         </is>
       </c>
       <c r="C136" t="inlineStr">
@@ -73993,7 +73993,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.028933</v>
+        <v>0.022373</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -74009,21 +74009,21 @@
     <row r="137">
       <c r="A137" t="inlineStr">
         <is>
-          <t>IA-NA-PURGE</t>
+          <t>IA-LIMESTONE-MU</t>
         </is>
       </c>
       <c r="B137" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C137" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="D137" t="n">
-        <v>0.641991</v>
+        <v>0</v>
       </c>
       <c r="E137" t="inlineStr">
         <is>
@@ -74039,7 +74039,7 @@
     <row r="138">
       <c r="A138" t="inlineStr">
         <is>
-          <t>IA-NA-RECYCLE</t>
+          <t>IA-NA-PURGE</t>
         </is>
       </c>
       <c r="B138" t="inlineStr">
@@ -74049,11 +74049,11 @@
       </c>
       <c r="C138" t="inlineStr">
         <is>
-          <t>NAOH_PLANT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D138" t="n">
-        <v>5.777917</v>
+        <v>0.641991</v>
       </c>
       <c r="E138" t="inlineStr">
         <is>
@@ -74069,21 +74069,21 @@
     <row r="139">
       <c r="A139" t="inlineStr">
         <is>
-          <t>IA-NAOH-CL2-SHIP</t>
+          <t>IA-NA-RECYCLE</t>
         </is>
       </c>
       <c r="B139" t="inlineStr">
         <is>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="C139" t="inlineStr">
+        <is>
           <t>NAOH_PLANT</t>
         </is>
       </c>
-      <c r="C139" t="inlineStr">
-        <is>
-          <t>NORTH_DOCK</t>
-        </is>
-      </c>
       <c r="D139" t="n">
-        <v>3.505031</v>
+        <v>5.777917</v>
       </c>
       <c r="E139" t="inlineStr">
         <is>
@@ -74099,7 +74099,7 @@
     <row r="140">
       <c r="A140" t="inlineStr">
         <is>
-          <t>IA-NAOH-H2</t>
+          <t>IA-NAOH-CL2-SHIP</t>
         </is>
       </c>
       <c r="B140" t="inlineStr">
@@ -74109,11 +74109,11 @@
       </c>
       <c r="C140" t="inlineStr">
         <is>
-          <t>HDR_H2</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D140" t="n">
-        <v>0.09965499999999999</v>
+        <v>3.505031</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -74129,21 +74129,21 @@
     <row r="141">
       <c r="A141" t="inlineStr">
         <is>
-          <t>IA-NAOH-H2O</t>
+          <t>IA-NAOH-H2</t>
         </is>
       </c>
       <c r="B141" t="inlineStr">
         <is>
-          <t>GW_INTAKE</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="C141" t="inlineStr">
         <is>
-          <t>NAOH_PLANT</t>
+          <t>HDR_H2</t>
         </is>
       </c>
       <c r="D141" t="n">
-        <v>14.237076</v>
+        <v>0.09965499999999999</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -74159,21 +74159,21 @@
     <row r="142">
       <c r="A142" t="inlineStr">
         <is>
-          <t>IA-NAOH-LIQ</t>
+          <t>IA-NAOH-H2O</t>
         </is>
       </c>
       <c r="B142" t="inlineStr">
         <is>
+          <t>GW_INTAKE</t>
+        </is>
+      </c>
+      <c r="C142" t="inlineStr">
+        <is>
           <t>NAOH_PLANT</t>
         </is>
       </c>
-      <c r="C142" t="inlineStr">
-        <is>
-          <t>EVAP_BASE</t>
-        </is>
-      </c>
       <c r="D142" t="n">
-        <v>16.750724</v>
+        <v>14.237076</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -74189,12 +74189,12 @@
     <row r="143">
       <c r="A143" t="inlineStr">
         <is>
-          <t>IA-NAOH-MU</t>
+          <t>IA-NAOH-LIQ</t>
         </is>
       </c>
       <c r="B143" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="C143" t="inlineStr">
@@ -74203,7 +74203,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>0</v>
+        <v>16.750724</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -74219,21 +74219,21 @@
     <row r="144">
       <c r="A144" t="inlineStr">
         <is>
-          <t>IA-NAOH-RESIDUE</t>
+          <t>IA-NAOH-MU</t>
         </is>
       </c>
       <c r="B144" t="inlineStr">
         <is>
-          <t>NAOH_PLANT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C144" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="D144" t="n">
-        <v>0.12089</v>
+        <v>0</v>
       </c>
       <c r="E144" t="inlineStr">
         <is>
@@ -74249,7 +74249,7 @@
     <row r="145">
       <c r="A145" t="inlineStr">
         <is>
-          <t>IA-NAOH-VENT</t>
+          <t>IA-NAOH-RESIDUE</t>
         </is>
       </c>
       <c r="B145" t="inlineStr">
@@ -74259,11 +74259,11 @@
       </c>
       <c r="C145" t="inlineStr">
         <is>
-          <t>ATMOS</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.487201</v>
+        <v>0.126417</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -74279,21 +74279,21 @@
     <row r="146">
       <c r="A146" t="inlineStr">
         <is>
-          <t>IA-NUT-LEACH</t>
+          <t>IA-NAOH-VENT</t>
         </is>
       </c>
       <c r="B146" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="C146" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ATMOS</t>
         </is>
       </c>
       <c r="D146" t="n">
-        <v>82.317318</v>
+        <v>0.475115</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -74309,21 +74309,21 @@
     <row r="147">
       <c r="A147" t="inlineStr">
         <is>
-          <t>IA-PHOS-SRC</t>
+          <t>IA-NUT-LEACH</t>
         </is>
       </c>
       <c r="B147" t="inlineStr">
         <is>
+          <t>NUTRIENT_DOSE</t>
+        </is>
+      </c>
+      <c r="C147" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C147" t="inlineStr">
-        <is>
-          <t>WS_PHOS</t>
-        </is>
-      </c>
       <c r="D147" t="n">
-        <v>0.62</v>
+        <v>82.317318</v>
       </c>
       <c r="E147" t="inlineStr">
         <is>
@@ -74339,21 +74339,21 @@
     <row r="148">
       <c r="A148" t="inlineStr">
         <is>
-          <t>IA-PLAST-01</t>
+          <t>IA-PHOS-SRC</t>
         </is>
       </c>
       <c r="B148" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C148" t="inlineStr">
         <is>
-          <t>OIL_DRYER</t>
+          <t>WS_PHOS</t>
         </is>
       </c>
       <c r="D148" t="n">
-        <v>33</v>
+        <v>0.62</v>
       </c>
       <c r="E148" t="inlineStr">
         <is>
@@ -74369,29 +74369,37 @@
     <row r="149">
       <c r="A149" t="inlineStr">
         <is>
-          <t>IA-POL-01</t>
+          <t>IA-PLAST-01</t>
         </is>
       </c>
       <c r="B149" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="C149" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>OIL_DRYER</t>
+        </is>
+      </c>
+      <c r="D149" t="n">
+        <v>33</v>
+      </c>
+      <c r="E149" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F149" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="150">
       <c r="A150" t="inlineStr">
         <is>
-          <t>IA-POL-02</t>
+          <t>IA-POL-01</t>
         </is>
       </c>
       <c r="B150" t="inlineStr">
@@ -74401,27 +74409,19 @@
       </c>
       <c r="C150" t="inlineStr">
         <is>
-          <t>CONTINUOUS_RECYCLE</t>
-        </is>
-      </c>
-      <c r="D150" t="n">
-        <v>3302.941356</v>
-      </c>
-      <c r="E150" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="F150" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="151">
       <c r="A151" t="inlineStr">
         <is>
-          <t>IA-POL-CAKE</t>
+          <t>IA-POL-02</t>
         </is>
       </c>
       <c r="B151" t="inlineStr">
@@ -74431,11 +74431,11 @@
       </c>
       <c r="C151" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>CONTINUOUS_RECYCLE</t>
         </is>
       </c>
       <c r="D151" t="n">
-        <v>217.369993</v>
+        <v>3302.941356</v>
       </c>
       <c r="E151" t="inlineStr">
         <is>
@@ -74451,21 +74451,21 @@
     <row r="152">
       <c r="A152" t="inlineStr">
         <is>
-          <t>IA-REC-01</t>
+          <t>IA-POL-CAKE</t>
         </is>
       </c>
       <c r="B152" t="inlineStr">
         <is>
-          <t>CONTINUOUS_RECYCLE</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="C152" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D152" t="n">
-        <v>3302.941356</v>
+        <v>217.369993</v>
       </c>
       <c r="E152" t="inlineStr">
         <is>
@@ -74481,21 +74481,21 @@
     <row r="153">
       <c r="A153" t="inlineStr">
         <is>
-          <t>IA-SCRUB-SRC</t>
+          <t>IA-REC-01</t>
         </is>
       </c>
       <c r="B153" t="inlineStr">
         <is>
+          <t>CONTINUOUS_RECYCLE</t>
+        </is>
+      </c>
+      <c r="C153" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C153" t="inlineStr">
-        <is>
-          <t>ACID_POLISH_SCRUB</t>
-        </is>
-      </c>
       <c r="D153" t="n">
-        <v>27.342833</v>
+        <v>3302.941356</v>
       </c>
       <c r="E153" t="inlineStr">
         <is>
@@ -74511,21 +74511,21 @@
     <row r="154">
       <c r="A154" t="inlineStr">
         <is>
-          <t>IA-SI-FUME</t>
+          <t>IA-SCRUB-SRC</t>
         </is>
       </c>
       <c r="B154" t="inlineStr">
         <is>
-          <t>SI_REDUCE</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C154" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>ACID_POLISH_SCRUB</t>
         </is>
       </c>
       <c r="D154" t="n">
-        <v>0.142429</v>
+        <v>27.342833</v>
       </c>
       <c r="E154" t="inlineStr">
         <is>
@@ -74541,12 +74541,12 @@
     <row r="155">
       <c r="A155" t="inlineStr">
         <is>
-          <t>IA-SI-PURGE</t>
+          <t>IA-SI-FUME</t>
         </is>
       </c>
       <c r="B155" t="inlineStr">
         <is>
-          <t>SI_REFINE</t>
+          <t>SI_REDUCE</t>
         </is>
       </c>
       <c r="C155" t="inlineStr">
@@ -74555,7 +74555,7 @@
         </is>
       </c>
       <c r="D155" t="n">
-        <v>0.259039</v>
+        <v>0.142429</v>
       </c>
       <c r="E155" t="inlineStr">
         <is>
@@ -74571,12 +74571,12 @@
     <row r="156">
       <c r="A156" t="inlineStr">
         <is>
-          <t>IA-SIC-RET</t>
+          <t>IA-SI-PURGE</t>
         </is>
       </c>
       <c r="B156" t="inlineStr">
         <is>
-          <t>NUTRIENT_DOSE</t>
+          <t>SI_REFINE</t>
         </is>
       </c>
       <c r="C156" t="inlineStr">
@@ -74585,7 +74585,7 @@
         </is>
       </c>
       <c r="D156" t="n">
-        <v>0.466189</v>
+        <v>0.259039</v>
       </c>
       <c r="E156" t="inlineStr">
         <is>
@@ -74601,21 +74601,21 @@
     <row r="157">
       <c r="A157" t="inlineStr">
         <is>
-          <t>IA-SINK-01</t>
+          <t>IA-SIC-RET</t>
         </is>
       </c>
       <c r="B157" t="inlineStr">
         <is>
+          <t>NUTRIENT_DOSE</t>
+        </is>
+      </c>
+      <c r="C157" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C157" t="inlineStr">
-        <is>
-          <t>FLOAT_SINK</t>
-        </is>
-      </c>
       <c r="D157" t="n">
-        <v>376.1</v>
+        <v>0.466189</v>
       </c>
       <c r="E157" t="inlineStr">
         <is>
@@ -74631,25 +74631,25 @@
     <row r="158">
       <c r="A158" t="inlineStr">
         <is>
-          <t>IA-TRIM-HX5</t>
+          <t>IA-SINK-01</t>
         </is>
       </c>
       <c r="B158" t="inlineStr">
         <is>
-          <t>RECTIFIER</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C158" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="D158" t="n">
-        <v>15.882</v>
+        <v>376.1</v>
       </c>
       <c r="E158" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F158" t="inlineStr">
@@ -74661,25 +74661,25 @@
     <row r="159">
       <c r="A159" t="inlineStr">
         <is>
-          <t>IA-TRONA-MU</t>
+          <t>IA-TRIM-HX5</t>
         </is>
       </c>
       <c r="B159" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>RECTIFIER</t>
         </is>
       </c>
       <c r="C159" t="inlineStr">
         <is>
-          <t>NAOH_PLANT</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D159" t="n">
-        <v>0.919575</v>
+        <v>15.882</v>
       </c>
       <c r="E159" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F159" t="inlineStr">
@@ -74691,21 +74691,21 @@
     <row r="160">
       <c r="A160" t="inlineStr">
         <is>
-          <t>IA-UPW-REJ</t>
+          <t>IA-TRONA-MU</t>
         </is>
       </c>
       <c r="B160" t="inlineStr">
         <is>
-          <t>BMED_UPW_POLISH</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C160" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="D160" t="n">
-        <v>6.045005</v>
+        <v>0.919575</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -74721,12 +74721,12 @@
     <row r="161">
       <c r="A161" t="inlineStr">
         <is>
-          <t>IA-VCD-BD</t>
+          <t>IA-UPW-REJ</t>
         </is>
       </c>
       <c r="B161" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>BMED_UPW_POLISH</t>
         </is>
       </c>
       <c r="C161" t="inlineStr">
@@ -74735,7 +74735,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>6.709424</v>
+        <v>6.045005</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -74751,21 +74751,21 @@
     <row r="162">
       <c r="A162" t="inlineStr">
         <is>
-          <t>IA-VS-NAOH</t>
+          <t>IA-VCD-BD</t>
         </is>
       </c>
       <c r="B162" t="inlineStr">
         <is>
-          <t>BMED_BASE</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C162" t="inlineStr">
         <is>
-          <t>EVAP_ACID_VS</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D162" t="n">
-        <v>0.0005</v>
+        <v>6.709424</v>
       </c>
       <c r="E162" t="inlineStr">
         <is>
@@ -74781,21 +74781,21 @@
     <row r="163">
       <c r="A163" t="inlineStr">
         <is>
-          <t>IA-VS-OFF</t>
+          <t>IA-VS-NAOH</t>
         </is>
       </c>
       <c r="B163" t="inlineStr">
         <is>
+          <t>BMED_BASE</t>
+        </is>
+      </c>
+      <c r="C163" t="inlineStr">
+        <is>
           <t>EVAP_ACID_VS</t>
         </is>
       </c>
-      <c r="C163" t="inlineStr">
-        <is>
-          <t>ALK_SCRUBBER</t>
-        </is>
-      </c>
       <c r="D163" t="n">
-        <v>0.0292</v>
+        <v>0.0005</v>
       </c>
       <c r="E163" t="inlineStr">
         <is>
@@ -74811,7 +74811,7 @@
     <row r="164">
       <c r="A164" t="inlineStr">
         <is>
-          <t>IA-VS-SPENT</t>
+          <t>IA-VS-OFF</t>
         </is>
       </c>
       <c r="B164" t="inlineStr">
@@ -74821,11 +74821,11 @@
       </c>
       <c r="C164" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>ALK_SCRUBBER</t>
         </is>
       </c>
       <c r="D164" t="n">
-        <v>0.0005999999999999999</v>
+        <v>0.0292</v>
       </c>
       <c r="E164" t="inlineStr">
         <is>
@@ -74841,21 +74841,21 @@
     <row r="165">
       <c r="A165" t="inlineStr">
         <is>
-          <t>IA-WET-FLOAT-01</t>
+          <t>IA-VS-SPENT</t>
         </is>
       </c>
       <c r="B165" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="C165" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="D165" t="n">
-        <v>343.1</v>
+        <v>0.0005999999999999999</v>
       </c>
       <c r="E165" t="inlineStr">
         <is>
@@ -74871,21 +74871,21 @@
     <row r="166">
       <c r="A166" t="inlineStr">
         <is>
-          <t>IA-ZNBR-MU</t>
+          <t>IA-WET-FLOAT-01</t>
         </is>
       </c>
       <c r="B166" t="inlineStr">
         <is>
+          <t>FLOAT_SINK</t>
+        </is>
+      </c>
+      <c r="C166" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C166" t="inlineStr">
-        <is>
-          <t>ZNBR2</t>
-        </is>
-      </c>
       <c r="D166" t="n">
-        <v>8.486482000000001</v>
+        <v>343.1</v>
       </c>
       <c r="E166" t="inlineStr">
         <is>
@@ -74901,64 +74901,64 @@
     <row r="167">
       <c r="A167" t="inlineStr">
         <is>
-          <t>LI_TO_GREASE</t>
+          <t>IA-ZNBR-MU</t>
         </is>
       </c>
       <c r="B167" t="inlineStr">
         <is>
-          <t>LI_RECOVER</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C167" t="inlineStr">
         <is>
-          <t>GREASE_LI</t>
+          <t>ZNBR2</t>
+        </is>
+      </c>
+      <c r="D167" t="n">
+        <v>8.486482000000001</v>
+      </c>
+      <c r="E167" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F167" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="168">
       <c r="A168" t="inlineStr">
         <is>
-          <t>MG_POT_CL2</t>
+          <t>LI_TO_GREASE</t>
         </is>
       </c>
       <c r="B168" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>LI_RECOVER</t>
         </is>
       </c>
       <c r="C168" t="inlineStr">
         <is>
-          <t>CRU</t>
-        </is>
-      </c>
-      <c r="D168" t="n">
-        <v>0</v>
-      </c>
-      <c r="E168" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREASE_LI</t>
         </is>
       </c>
       <c r="F168" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="169">
       <c r="A169" t="inlineStr">
         <is>
-          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
+          <t>MG_POT_CL2</t>
         </is>
       </c>
       <c r="B169" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="C169" t="inlineStr">
@@ -74983,7 +74983,7 @@
     <row r="170">
       <c r="A170" t="inlineStr">
         <is>
-          <t>MO_CELL_RAFFINATE</t>
+          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
         </is>
       </c>
       <c r="B170" t="inlineStr">
@@ -74993,7 +74993,7 @@
       </c>
       <c r="C170" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D170" t="n">
@@ -75013,39 +75013,47 @@
     <row r="171">
       <c r="A171" t="inlineStr">
         <is>
-          <t>PCA_TO_GREASE</t>
+          <t>MO_CELL_RAFFINATE</t>
         </is>
       </c>
       <c r="B171" t="inlineStr">
         <is>
-          <t>P_CA</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="C171" t="inlineStr">
         <is>
-          <t>GREASE_CA</t>
+          <t>POLISH_BANK</t>
+        </is>
+      </c>
+      <c r="D171" t="n">
+        <v>0</v>
+      </c>
+      <c r="E171" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F171" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="172">
       <c r="A172" t="inlineStr">
         <is>
-          <t>POLISH_TO_LI</t>
+          <t>PCA_TO_GREASE</t>
         </is>
       </c>
       <c r="B172" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>P_CA</t>
         </is>
       </c>
       <c r="C172" t="inlineStr">
         <is>
-          <t>LI_RECOVER</t>
+          <t>GREASE_CA</t>
         </is>
       </c>
       <c r="F172" t="inlineStr">
@@ -75057,51 +75065,43 @@
     <row r="173">
       <c r="A173" t="inlineStr">
         <is>
-          <t>POLYF_RECLAIM</t>
+          <t>POLISH_TO_LI</t>
         </is>
       </c>
       <c r="B173" t="inlineStr">
         <is>
-          <t>POLY_F</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="C173" t="inlineStr">
         <is>
-          <t>F_RECOVER</t>
-        </is>
-      </c>
-      <c r="D173" t="n">
-        <v>0.02</v>
-      </c>
-      <c r="E173" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>LI_RECOVER</t>
         </is>
       </c>
       <c r="F173" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="174">
       <c r="A174" t="inlineStr">
         <is>
-          <t>POLY_TO_WET</t>
+          <t>POLYF_RECLAIM</t>
         </is>
       </c>
       <c r="B174" t="inlineStr">
         <is>
-          <t>POLY_STOCK</t>
+          <t>POLY_F</t>
         </is>
       </c>
       <c r="C174" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>F_RECOVER</t>
         </is>
       </c>
       <c r="D174" t="n">
-        <v>0.026739</v>
+        <v>0.02</v>
       </c>
       <c r="E174" t="inlineStr">
         <is>
@@ -75117,21 +75117,21 @@
     <row r="175">
       <c r="A175" t="inlineStr">
         <is>
-          <t>S08</t>
+          <t>POLY_TO_WET</t>
         </is>
       </c>
       <c r="B175" t="inlineStr">
         <is>
+          <t>POLY_STOCK</t>
+        </is>
+      </c>
+      <c r="C175" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C175" t="inlineStr">
-        <is>
-          <t>MFG_SHOP</t>
-        </is>
-      </c>
       <c r="D175" t="n">
-        <v>41.996408</v>
+        <v>0.026739</v>
       </c>
       <c r="E175" t="inlineStr">
         <is>
@@ -75147,21 +75147,21 @@
     <row r="176">
       <c r="A176" t="inlineStr">
         <is>
-          <t>S09</t>
+          <t>S08</t>
         </is>
       </c>
       <c r="B176" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C176" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D176" t="n">
-        <v>9.277184</v>
+        <v>41.996408</v>
       </c>
       <c r="E176" t="inlineStr">
         <is>
@@ -75177,21 +75177,21 @@
     <row r="177">
       <c r="A177" t="inlineStr">
         <is>
-          <t>S10</t>
+          <t>S09</t>
         </is>
       </c>
       <c r="B177" t="inlineStr">
         <is>
+          <t>BMED_ACID</t>
+        </is>
+      </c>
+      <c r="C177" t="inlineStr">
+        <is>
           <t>WET_BENCH</t>
         </is>
       </c>
-      <c r="C177" t="inlineStr">
-        <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
       <c r="D177" t="n">
-        <v>79.11577699999999</v>
+        <v>9.277184</v>
       </c>
       <c r="E177" t="inlineStr">
         <is>
@@ -75207,12 +75207,12 @@
     <row r="178">
       <c r="A178" t="inlineStr">
         <is>
-          <t>S100</t>
+          <t>S10</t>
         </is>
       </c>
       <c r="B178" t="inlineStr">
         <is>
-          <t>Q4_BUS</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="C178" t="inlineStr">
@@ -75221,11 +75221,11 @@
         </is>
       </c>
       <c r="D178" t="n">
-        <v>0.5322</v>
+        <v>79.11577699999999</v>
       </c>
       <c r="E178" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F178" t="inlineStr">
@@ -75237,12 +75237,12 @@
     <row r="179">
       <c r="A179" t="inlineStr">
         <is>
-          <t>S16</t>
+          <t>S100</t>
         </is>
       </c>
       <c r="B179" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>Q4_BUS</t>
         </is>
       </c>
       <c r="C179" t="inlineStr">
@@ -75251,11 +75251,11 @@
         </is>
       </c>
       <c r="D179" t="n">
-        <v>11.636366</v>
+        <v>0.5322</v>
       </c>
       <c r="E179" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F179" t="inlineStr">
@@ -75267,25 +75267,25 @@
     <row r="180">
       <c r="A180" t="inlineStr">
         <is>
-          <t>S17-BMED</t>
+          <t>S16</t>
         </is>
       </c>
       <c r="B180" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="C180" t="inlineStr">
         <is>
-          <t>BMED_ACID</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D180" t="n">
-        <v>5.6267</v>
+        <v>11.635142</v>
       </c>
       <c r="E180" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F180" t="inlineStr">
@@ -75297,25 +75297,25 @@
     <row r="181">
       <c r="A181" t="inlineStr">
         <is>
-          <t>S19</t>
+          <t>S17-BMED</t>
         </is>
       </c>
       <c r="B181" t="inlineStr">
         <is>
-          <t>BAGHOUSE</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C181" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>BMED_ACID</t>
         </is>
       </c>
       <c r="D181" t="n">
-        <v>0</v>
+        <v>5.6267</v>
       </c>
       <c r="E181" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F181" t="inlineStr">
@@ -75327,12 +75327,12 @@
     <row r="182">
       <c r="A182" t="inlineStr">
         <is>
-          <t>S28</t>
+          <t>S19</t>
         </is>
       </c>
       <c r="B182" t="inlineStr">
         <is>
-          <t>VCD_TRAIN</t>
+          <t>BAGHOUSE</t>
         </is>
       </c>
       <c r="C182" t="inlineStr">
@@ -75341,7 +75341,7 @@
         </is>
       </c>
       <c r="D182" t="n">
-        <v>17.877059</v>
+        <v>0</v>
       </c>
       <c r="E182" t="inlineStr">
         <is>
@@ -75357,12 +75357,12 @@
     <row r="183">
       <c r="A183" t="inlineStr">
         <is>
-          <t>S39</t>
+          <t>S28</t>
         </is>
       </c>
       <c r="B183" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>VCD_TRAIN</t>
         </is>
       </c>
       <c r="C183" t="inlineStr">
@@ -75371,7 +75371,7 @@
         </is>
       </c>
       <c r="D183" t="n">
-        <v>3.310001</v>
+        <v>17.877059</v>
       </c>
       <c r="E183" t="inlineStr">
         <is>
@@ -75387,21 +75387,21 @@
     <row r="184">
       <c r="A184" t="inlineStr">
         <is>
-          <t>S66</t>
+          <t>S39</t>
         </is>
       </c>
       <c r="B184" t="inlineStr">
         <is>
-          <t>ACID_POLISH_SCRUB</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C184" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D184" t="n">
-        <v>27.372033</v>
+        <v>3.310001</v>
       </c>
       <c r="E184" t="inlineStr">
         <is>
@@ -75417,21 +75417,21 @@
     <row r="185">
       <c r="A185" t="inlineStr">
         <is>
-          <t>S68</t>
+          <t>S66</t>
         </is>
       </c>
       <c r="B185" t="inlineStr">
         <is>
-          <t>CRYO_AHU</t>
+          <t>ACID_POLISH_SCRUB</t>
         </is>
       </c>
       <c r="C185" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D185" t="n">
-        <v>78.98790099999999</v>
+        <v>27.372033</v>
       </c>
       <c r="E185" t="inlineStr">
         <is>
@@ -75447,12 +75447,12 @@
     <row r="186">
       <c r="A186" t="inlineStr">
         <is>
-          <t>S72</t>
+          <t>S68</t>
         </is>
       </c>
       <c r="B186" t="inlineStr">
         <is>
-          <t>MET_SCRUB</t>
+          <t>CRYO_AHU</t>
         </is>
       </c>
       <c r="C186" t="inlineStr">
@@ -75461,7 +75461,7 @@
         </is>
       </c>
       <c r="D186" t="n">
-        <v>2.4442</v>
+        <v>78.98790099999999</v>
       </c>
       <c r="E186" t="inlineStr">
         <is>
@@ -75477,21 +75477,21 @@
     <row r="187">
       <c r="A187" t="inlineStr">
         <is>
-          <t>SALT_TO_FLUX</t>
+          <t>S72</t>
         </is>
       </c>
       <c r="B187" t="inlineStr">
         <is>
-          <t>SALT_FEED</t>
+          <t>MET_SCRUB</t>
         </is>
       </c>
       <c r="C187" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D187" t="n">
-        <v>0</v>
+        <v>2.4442</v>
       </c>
       <c r="E187" t="inlineStr">
         <is>
@@ -75507,25 +75507,25 @@
     <row r="188">
       <c r="A188" t="inlineStr">
         <is>
-          <t>SF-EVAP_ACID</t>
+          <t>SALT_TO_FLUX</t>
         </is>
       </c>
       <c r="B188" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>SALT_FEED</t>
         </is>
       </c>
       <c r="C188" t="inlineStr">
         <is>
-          <t>EVAP_ACID</t>
+          <t>FLUX_PREP</t>
         </is>
       </c>
       <c r="D188" t="n">
-        <v>1.498</v>
+        <v>0</v>
       </c>
       <c r="E188" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F188" t="inlineStr">
@@ -75537,7 +75537,7 @@
     <row r="189">
       <c r="A189" t="inlineStr">
         <is>
-          <t>SF-EVAP_ACID_VS</t>
+          <t>SF-EVAP_ACID</t>
         </is>
       </c>
       <c r="B189" t="inlineStr">
@@ -75547,11 +75547,11 @@
       </c>
       <c r="C189" t="inlineStr">
         <is>
-          <t>EVAP_ACID_VS</t>
+          <t>EVAP_ACID</t>
         </is>
       </c>
       <c r="D189" t="n">
-        <v>0.0238</v>
+        <v>1.498</v>
       </c>
       <c r="E189" t="inlineStr">
         <is>
@@ -75567,7 +75567,7 @@
     <row r="190">
       <c r="A190" t="inlineStr">
         <is>
-          <t>SF-EVAP_BASE</t>
+          <t>SF-EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="B190" t="inlineStr">
@@ -75577,11 +75577,11 @@
       </c>
       <c r="C190" t="inlineStr">
         <is>
-          <t>EVAP_BASE</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="D190" t="n">
-        <v>1.349</v>
+        <v>0.0238</v>
       </c>
       <c r="E190" t="inlineStr">
         <is>
@@ -75597,7 +75597,7 @@
     <row r="191">
       <c r="A191" t="inlineStr">
         <is>
-          <t>SF-LEACH_CSTR_1</t>
+          <t>SF-EVAP_BASE</t>
         </is>
       </c>
       <c r="B191" t="inlineStr">
@@ -75607,11 +75607,11 @@
       </c>
       <c r="C191" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="D191" t="n">
-        <v>0.75</v>
+        <v>1.349</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -75627,7 +75627,7 @@
     <row r="192">
       <c r="A192" t="inlineStr">
         <is>
-          <t>SF-NAOH_PLANT</t>
+          <t>SF-LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="B192" t="inlineStr">
@@ -75637,11 +75637,11 @@
       </c>
       <c r="C192" t="inlineStr">
         <is>
-          <t>NAOH_PLANT</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D192" t="n">
-        <v>1.1935</v>
+        <v>0.75</v>
       </c>
       <c r="E192" t="inlineStr">
         <is>
@@ -75657,21 +75657,21 @@
     <row r="193">
       <c r="A193" t="inlineStr">
         <is>
-          <t>SQ-EVAP_ACID</t>
+          <t>SF-NAOH_PLANT</t>
         </is>
       </c>
       <c r="B193" t="inlineStr">
         <is>
-          <t>EVAP_ACID</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C193" t="inlineStr">
         <is>
-          <t>HEAT_SINK</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1.498</v>
+        <v>1.1929</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -75687,12 +75687,12 @@
     <row r="194">
       <c r="A194" t="inlineStr">
         <is>
-          <t>SQ-EVAP_ACID_VS</t>
+          <t>SQ-EVAP_ACID</t>
         </is>
       </c>
       <c r="B194" t="inlineStr">
         <is>
-          <t>EVAP_ACID_VS</t>
+          <t>EVAP_ACID</t>
         </is>
       </c>
       <c r="C194" t="inlineStr">
@@ -75701,7 +75701,7 @@
         </is>
       </c>
       <c r="D194" t="n">
-        <v>0.0238</v>
+        <v>1.498</v>
       </c>
       <c r="E194" t="inlineStr">
         <is>
@@ -75717,12 +75717,12 @@
     <row r="195">
       <c r="A195" t="inlineStr">
         <is>
-          <t>SQ-EVAP_BASE</t>
+          <t>SQ-EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="B195" t="inlineStr">
         <is>
-          <t>EVAP_BASE</t>
+          <t>EVAP_ACID_VS</t>
         </is>
       </c>
       <c r="C195" t="inlineStr">
@@ -75731,7 +75731,7 @@
         </is>
       </c>
       <c r="D195" t="n">
-        <v>1.349</v>
+        <v>0.0238</v>
       </c>
       <c r="E195" t="inlineStr">
         <is>
@@ -75747,25 +75747,25 @@
     <row r="196">
       <c r="A196" t="inlineStr">
         <is>
-          <t>TFE_HCL_TO_CRU</t>
+          <t>SQ-EVAP_BASE</t>
         </is>
       </c>
       <c r="B196" t="inlineStr">
         <is>
-          <t>TFE_SYN</t>
+          <t>EVAP_BASE</t>
         </is>
       </c>
       <c r="C196" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>HEAT_SINK</t>
         </is>
       </c>
       <c r="D196" t="n">
-        <v>0.327654</v>
+        <v>1.349</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F196" t="inlineStr">
@@ -75777,12 +75777,12 @@
     <row r="197">
       <c r="A197" t="inlineStr">
         <is>
-          <t>TI_CELL_CL2_TO_CRU</t>
+          <t>TFE_HCL_TO_CRU</t>
         </is>
       </c>
       <c r="B197" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>TFE_SYN</t>
         </is>
       </c>
       <c r="C197" t="inlineStr">
@@ -75791,7 +75791,7 @@
         </is>
       </c>
       <c r="D197" t="n">
-        <v>0</v>
+        <v>0.327654</v>
       </c>
       <c r="E197" t="inlineStr">
         <is>
@@ -75807,7 +75807,7 @@
     <row r="198">
       <c r="A198" t="inlineStr">
         <is>
-          <t>TI_CELL_SLAG_RETURN</t>
+          <t>TI_CELL_CL2_TO_CRU</t>
         </is>
       </c>
       <c r="B198" t="inlineStr">
@@ -75817,7 +75817,7 @@
       </c>
       <c r="C198" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D198" t="n">
@@ -75837,28 +75837,58 @@
     <row r="199">
       <c r="A199" t="inlineStr">
         <is>
+          <t>TI_CELL_SLAG_RETURN</t>
+        </is>
+      </c>
+      <c r="B199" t="inlineStr">
+        <is>
+          <t>TI_CELL</t>
+        </is>
+      </c>
+      <c r="C199" t="inlineStr">
+        <is>
+          <t>LEACH_CSTR_1</t>
+        </is>
+      </c>
+      <c r="D199" t="n">
+        <v>0</v>
+      </c>
+      <c r="E199" t="inlineStr">
+        <is>
+          <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F199" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="200">
+      <c r="A200" t="inlineStr">
+        <is>
           <t>VDF_HCL_TO_CRU</t>
         </is>
       </c>
-      <c r="B199" t="inlineStr">
+      <c r="B200" t="inlineStr">
         <is>
           <t>VDF_SYN</t>
         </is>
       </c>
-      <c r="C199" t="inlineStr">
+      <c r="C200" t="inlineStr">
         <is>
           <t>CRU</t>
         </is>
       </c>
-      <c r="D199" t="n">
+      <c r="D200" t="n">
         <v>0.42605</v>
       </c>
-      <c r="E199" t="inlineStr">
+      <c r="E200" t="inlineStr">
         <is>
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F199" t="inlineStr">
+      <c r="F200" t="inlineStr">
         <is>
           <t>study</t>
         </is>
@@ -76434,7 +76464,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.024432</v>
+        <v>0.025656</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -77198,7 +77228,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>4.836867</v>
+        <v>4.835643</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -79049,7 +79079,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H63"/>
+  <dimension ref="A1:H64"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -79111,7 +79141,7 @@
         </is>
       </c>
       <c r="B2" s="8" t="n">
-        <v>0.9654</v>
+        <v>0.966</v>
       </c>
       <c r="C2" t="inlineStr">
         <is>
@@ -79537,7 +79567,7 @@
         </is>
       </c>
       <c r="D18" t="n">
-        <v>0.024432</v>
+        <v>0.025656</v>
       </c>
       <c r="E18" t="inlineStr">
         <is>
@@ -79807,7 +79837,7 @@
         </is>
       </c>
       <c r="D27" t="n">
-        <v>0.079758</v>
+        <v>0.086872</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -79867,7 +79897,7 @@
         </is>
       </c>
       <c r="D29" t="n">
-        <v>0.08300299999999999</v>
+        <v>0.077462</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -80107,7 +80137,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.29871</v>
+        <v>0.259355</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -80123,21 +80153,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-SULFUR-MU</t>
+          <t>IA-LIME-TO-NAOH</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>ACID_PLANT</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>ACID_PLANT</t>
+          <t>NAOH_PLANT</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.018487</v>
+        <v>0.022373</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -80153,21 +80183,21 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>MEOH_TO_OLEFIN</t>
+          <t>IA-SULFUR-MU</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>MEOH_SYNTH</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
         <is>
-          <t>POLY_OLEFIN</t>
+          <t>ACID_PLANT</t>
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0</v>
+        <v>0.012935</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -80183,21 +80213,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>MEOH_TO_TFE</t>
+          <t>MEOH_TO_OLEFIN</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>MEOH_TANK</t>
+          <t>MEOH_SYNTH</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>TFE_SYN</t>
+          <t>POLY_OLEFIN</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.064071</v>
+        <v>0</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -80213,7 +80243,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>MEOH_TO_VDF</t>
+          <t>MEOH_TO_TFE</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -80223,11 +80253,11 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>VDF_SYN</t>
+          <t>TFE_SYN</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.150117</v>
+        <v>0.064071</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -80243,21 +80273,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>OIL_TO_OLEFIN</t>
+          <t>MEOH_TO_VDF</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>MEOH_TANK</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>POLY_OLEFIN</t>
+          <t>VDF_SYN</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0</v>
+        <v>0.150117</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -80273,21 +80303,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>OLEFIN_TO_PELLET</t>
+          <t>OIL_TO_OLEFIN</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
+          <t>OIL_FRAC</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
           <t>POLY_OLEFIN</t>
         </is>
       </c>
-      <c r="C43" t="inlineStr">
-        <is>
-          <t>PELLET</t>
-        </is>
-      </c>
       <c r="D43" t="n">
-        <v>0.294127</v>
+        <v>0</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -80303,17 +80333,17 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>PELLET_TO_STOCK</t>
+          <t>OLEFIN_TO_PELLET</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
+          <t>POLY_OLEFIN</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
           <t>PELLET</t>
-        </is>
-      </c>
-      <c r="C44" t="inlineStr">
-        <is>
-          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="D44" t="n">
@@ -80333,21 +80363,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>POLYF_RECLAIM</t>
+          <t>PELLET_TO_STOCK</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>POLY_F</t>
+          <t>PELLET</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>F_RECOVER</t>
+          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>0.02</v>
+        <v>0.294127</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -80363,7 +80393,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>POLYF_TO_FILM</t>
+          <t>POLYF_RECLAIM</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -80373,11 +80403,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>FILM_CAST</t>
+          <t>F_RECOVER</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>0.14</v>
+        <v>0.02</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -80393,7 +80423,7 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>POLYF_TO_PELLET</t>
+          <t>POLYF_TO_FILM</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
@@ -80403,11 +80433,11 @@
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>PELLET</t>
+          <t>FILM_CAST</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0</v>
+        <v>0.14</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -80423,7 +80453,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>POLYF_TO_POWDER</t>
+          <t>POLYF_TO_PELLET</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -80433,11 +80463,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>POWDER_RESIN</t>
+          <t>PELLET</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0.09</v>
+        <v>0</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -80453,21 +80483,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>POLY_TO_FAB</t>
+          <t>POLYF_TO_POWDER</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>POLY_STOCK</t>
+          <t>POLY_F</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>POWDER_RESIN</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>0</v>
+        <v>0.09</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -80483,7 +80513,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>POLY_TO_MFG</t>
+          <t>POLY_TO_FAB</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -80493,11 +80523,11 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>0.267388</v>
+        <v>0</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -80513,7 +80543,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>POLY_TO_WET</t>
+          <t>POLY_TO_MFG</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -80523,11 +80553,11 @@
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D51" t="n">
-        <v>0.026739</v>
+        <v>0.267388</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -80543,21 +80573,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>POWDER_TO_STOCK</t>
+          <t>POLY_TO_WET</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>POWDER_RESIN</t>
+          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>POLY_STOCK</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.09</v>
+        <v>0.026739</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -80573,25 +80603,25 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>SF-ACID_PLANT</t>
+          <t>POWDER_TO_STOCK</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>POWDER_RESIN</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>ACID_PLANT</t>
+          <t>POLY_STOCK</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.9654</v>
+        <v>0.09</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F53" t="inlineStr">
@@ -80603,7 +80633,7 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>SF-FILM_CAST</t>
+          <t>SF-ACID_PLANT</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
@@ -80613,11 +80643,11 @@
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>FILM_CAST</t>
+          <t>ACID_PLANT</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.1087</v>
+        <v>0.966</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -80633,7 +80663,7 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>SF-HF_GEN</t>
+          <t>SF-FILM_CAST</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
@@ -80643,11 +80673,11 @@
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>HF_GEN</t>
+          <t>FILM_CAST</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.3083</v>
+        <v>0.1087</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -80663,7 +80693,7 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>SF-POLY_F</t>
+          <t>SF-HF_GEN</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
@@ -80673,11 +80703,11 @@
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>POLY_F</t>
+          <t>HF_GEN</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.0449</v>
+        <v>0.3083</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -80693,7 +80723,7 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>SF-POWDER_RESIN</t>
+          <t>SF-POLY_F</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
@@ -80703,11 +80733,11 @@
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>POWDER_RESIN</t>
+          <t>POLY_F</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.0152</v>
+        <v>0.0449</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -80723,7 +80753,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>SF-TFE_SYN</t>
+          <t>SF-POWDER_RESIN</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -80733,11 +80763,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>TFE_SYN</t>
+          <t>POWDER_RESIN</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.3989</v>
+        <v>0.0152</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -80753,7 +80783,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>SF-VDF_SYN</t>
+          <t>SF-TFE_SYN</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -80763,11 +80793,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>VDF_SYN</t>
+          <t>TFE_SYN</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.5128</v>
+        <v>0.3989</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -80783,25 +80813,25 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>TFE_HCL_TO_CRU</t>
+          <t>SF-VDF_SYN</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>TFE_SYN</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>VDF_SYN</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.327654</v>
+        <v>0.5128</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
@@ -80813,7 +80843,7 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>TFE_TO_POLY_F</t>
+          <t>TFE_HCL_TO_CRU</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
@@ -80823,11 +80853,11 @@
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>POLY_F</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.1</v>
+        <v>0.327654</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -80843,21 +80873,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>VDF_HCL_TO_CRU</t>
+          <t>TFE_TO_POLY_F</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>VDF_SYN</t>
+          <t>TFE_SYN</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>POLY_F</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>0.42605</v>
+        <v>0.1</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -80873,28 +80903,58 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
+          <t>VDF_HCL_TO_CRU</t>
+        </is>
+      </c>
+      <c r="B63" t="inlineStr">
+        <is>
+          <t>VDF_SYN</t>
+        </is>
+      </c>
+      <c r="C63" t="inlineStr">
+        <is>
+          <t>CRU</t>
+        </is>
+      </c>
+      <c r="D63" t="n">
+        <v>0.42605</v>
+      </c>
+      <c r="E63" t="inlineStr">
+        <is>
+          <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F63" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="64">
+      <c r="A64" t="inlineStr">
+        <is>
           <t>VDF_TO_POLY_F</t>
         </is>
       </c>
-      <c r="B63" t="inlineStr">
+      <c r="B64" t="inlineStr">
         <is>
           <t>VDF_SYN</t>
         </is>
       </c>
-      <c r="C63" t="inlineStr">
+      <c r="C64" t="inlineStr">
         <is>
           <t>POLY_F</t>
         </is>
       </c>
-      <c r="D63" t="n">
+      <c r="D64" t="n">
         <v>0.15</v>
       </c>
-      <c r="E63" t="inlineStr">
+      <c r="E64" t="inlineStr">
         <is>
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F63" t="inlineStr">
+      <c r="F64" t="inlineStr">
         <is>
           <t>study</t>
         </is>

</xml_diff>

<commit_message>
Make the pattern wax on site: the make-up is the plant C19-C28 paraffin cut after the dewax reclaim, the C19-C28 export falls by the draw; retire IA-WAX-MU (A-M-424, batch 36)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 8a86220e5069046ba1637994dfd0725c4b5bea2473b8b817d64c5a1216f63f06</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 d1045fd2b6907caf0d7ab1fa04d00dbe8b943fef94332e354ea6e0a7da176f95</t>
         </is>
       </c>
     </row>
@@ -7626,7 +7626,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H134"/>
+  <dimension ref="A1:H135"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -8870,21 +8870,21 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>CAST_SCRAP_TO_IND</t>
+          <t>C19_TO_WAX</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
         <is>
-          <t>CAST_LINE</t>
+          <t>PROD_C19_C28</t>
         </is>
       </c>
       <c r="C40" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>WAX_PATTERN</t>
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0</v>
+        <v>0.2</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -8900,7 +8900,7 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>CAST_TO_EXTRUDE</t>
+          <t>CAST_SCRAP_TO_IND</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
@@ -8910,7 +8910,7 @@
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>EXTRUDE</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D41" t="n">
@@ -8930,7 +8930,7 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>CAST_TO_ROLL</t>
+          <t>CAST_TO_EXTRUDE</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
@@ -8940,11 +8940,11 @@
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>ROLL</t>
+          <t>EXTRUDE</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -8960,21 +8960,21 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>CA_POT_TO_IND</t>
+          <t>CAST_TO_ROLL</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
         <is>
-          <t>CA_POT</t>
+          <t>CAST_LINE</t>
         </is>
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>ROLL</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.055069</v>
+        <v>3</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -8990,21 +8990,21 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>COMB_OFFGAS</t>
+          <t>CA_POT_TO_IND</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
         <is>
-          <t>COMB_HEAT</t>
+          <t>CA_POT</t>
         </is>
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>MET_SCRUB</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0</v>
+        <v>0.055069</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -9020,21 +9020,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>CONT_TO_ROLL</t>
+          <t>COMB_OFFGAS</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>CONT_CAST</t>
+          <t>COMB_HEAT</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>ROLL</t>
+          <t>MET_SCRUB</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>10</v>
+        <v>0</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -9050,7 +9050,7 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>CONT_TO_STOCK</t>
+          <t>CONT_TO_ROLL</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
@@ -9060,11 +9060,11 @@
       </c>
       <c r="C46" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>ROLL</t>
         </is>
       </c>
       <c r="D46" t="n">
-        <v>21.7125</v>
+        <v>10</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -9080,21 +9080,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>CR_TO_IND</t>
+          <t>CONT_TO_STOCK</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>CR_CELL</t>
+          <t>CONT_CAST</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.25</v>
+        <v>21.7125</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -9110,21 +9110,21 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>DRAW_TO_STOCK</t>
+          <t>CR_TO_IND</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>CR_CELL</t>
         </is>
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -9140,17 +9140,17 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>EW9_LIQUOR_TO_MO</t>
+          <t>DRAW_TO_STOCK</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>EW_9</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="D49" t="n">
@@ -9170,7 +9170,7 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>EW_METALS_TO_IND</t>
+          <t>EW9_LIQUOR_TO_MO</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
@@ -9180,7 +9180,7 @@
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="D50" t="n">
@@ -9200,17 +9200,17 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>EXTRUDE_TO_STOCK</t>
+          <t>EW_METALS_TO_IND</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
         <is>
-          <t>EXTRUDE</t>
+          <t>EW_9</t>
         </is>
       </c>
       <c r="C51" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D51" t="n">
@@ -9230,17 +9230,17 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>FLOAT_SINK_GRIT_TO_TI</t>
+          <t>EXTRUDE_TO_STOCK</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>EXTRUDE</t>
         </is>
       </c>
       <c r="C52" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="D52" t="n">
@@ -9260,21 +9260,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>FLUX_TO_IND</t>
+          <t>FLOAT_SINK_GRIT_TO_TI</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.039781</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -9290,21 +9290,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>FOUNDRY_SLAG_TO_LEACH</t>
+          <t>FLUX_TO_IND</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
+          <t>FLUX_PREP</t>
+        </is>
+      </c>
+      <c r="C54" t="inlineStr">
+        <is>
           <t>IND_MELT</t>
         </is>
       </c>
-      <c r="C54" t="inlineStr">
-        <is>
-          <t>LEACH_CSTR_1</t>
-        </is>
-      </c>
       <c r="D54" t="n">
-        <v>0.356466</v>
+        <v>0.039781</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -9320,21 +9320,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IA-ALCL3-MU</t>
+          <t>FOUNDRY_SLAG_TO_LEACH</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="C55" t="inlineStr">
         <is>
-          <t>AL_POT</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D55" t="n">
-        <v>49.419232</v>
+        <v>0.356466</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -9350,21 +9350,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IA-BURNOUT-VENT</t>
+          <t>IA-ALCL3-MU</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
-          <t>SHELL_BURNOUT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C56" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>AL_POT</t>
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.2</v>
+        <v>49.419232</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -9380,21 +9380,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IA-C-CR</t>
+          <t>IA-BURNOUT-VENT</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>OIL_PYRO</t>
+          <t>SHELL_BURNOUT</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>CR_CELL</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>0.101911</v>
+        <v>0.2</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -9410,7 +9410,7 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IA-C-MO</t>
+          <t>IA-C-CR</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
@@ -9420,11 +9420,11 @@
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>CR_CELL</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.013807</v>
+        <v>0.101911</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -9440,7 +9440,7 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>IA-C-TI</t>
+          <t>IA-C-MO</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
@@ -9450,11 +9450,11 @@
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="D59" t="n">
-        <v>0.295205</v>
+        <v>0.013807</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -9470,21 +9470,21 @@
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>IA-CA-CL2-SHIP</t>
+          <t>IA-C-TI</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>CA_POT</t>
+          <t>OIL_PYRO</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.097428</v>
+        <v>0.295205</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -9500,21 +9500,21 @@
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>IA-CACL2-MU</t>
+          <t>IA-CA-CL2-SHIP</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
+          <t>CA_POT</t>
+        </is>
+      </c>
+      <c r="C61" t="inlineStr">
+        <is>
           <t>NORTH_DOCK</t>
         </is>
       </c>
-      <c r="C61" t="inlineStr">
-        <is>
-          <t>CA_POT</t>
-        </is>
-      </c>
       <c r="D61" t="n">
-        <v>0.152497</v>
+        <v>0.097428</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -9530,21 +9530,21 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>IA-CL2-MG-TI</t>
+          <t>IA-CACL2-MU</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>CA_POT</t>
         </is>
       </c>
       <c r="D62" t="n">
-        <v>1.481313</v>
+        <v>0.152497</v>
       </c>
       <c r="E62" t="inlineStr">
         <is>
@@ -9560,21 +9560,21 @@
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>IA-CL2-SHIP</t>
+          <t>IA-CL2-MG-TI</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>AL_POT</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D63" t="n">
-        <v>39.205574</v>
+        <v>1.481313</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -9590,7 +9590,7 @@
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>IA-CL2-SIREF</t>
+          <t>IA-CL2-SHIP</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
@@ -9600,11 +9600,11 @@
       </c>
       <c r="C64" t="inlineStr">
         <is>
-          <t>SI_REFINE</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.213658</v>
+        <v>39.205574</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -9620,21 +9620,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>IA-CR-VENT</t>
+          <t>IA-CL2-SIREF</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>CR_CELL</t>
+          <t>AL_POT</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>SI_REFINE</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.2173</v>
+        <v>0.213658</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -9650,21 +9650,21 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>IA-CR2O3-MU</t>
+          <t>IA-CR-VENT</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
+          <t>CR_CELL</t>
+        </is>
+      </c>
+      <c r="C66" t="inlineStr">
+        <is>
           <t>NORTH_DOCK</t>
         </is>
       </c>
-      <c r="C66" t="inlineStr">
-        <is>
-          <t>CR_CELL</t>
-        </is>
-      </c>
       <c r="D66" t="n">
-        <v>0.365389</v>
+        <v>0.2173</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -9680,21 +9680,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>IA-KROLL-CO</t>
+          <t>IA-CR2O3-MU</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>CR_CELL</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.629453</v>
+        <v>0.365389</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -9710,7 +9710,7 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>IA-KROLL-FLUX</t>
+          <t>IA-KROLL-CO</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
@@ -9720,11 +9720,11 @@
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.039781</v>
+        <v>0.629453</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -9740,21 +9740,21 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>IA-METAL-SHIP</t>
+          <t>IA-KROLL-FLUX</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>METAL_STORE</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>FLUX_PREP</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>10.8125</v>
+        <v>0.039781</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -9770,21 +9770,21 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>IA-MG-TI</t>
+          <t>IA-METAL-SHIP</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>METAL_STORE</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D70" t="n">
-        <v>0.507761</v>
+        <v>10.8125</v>
       </c>
       <c r="E70" t="inlineStr">
         <is>
@@ -9800,21 +9800,21 @@
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>IA-MGCL2-KROLL</t>
+          <t>IA-MG-TI</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
         <is>
+          <t>MG_POT</t>
+        </is>
+      </c>
+      <c r="C71" t="inlineStr">
+        <is>
           <t>TI_CELL</t>
         </is>
       </c>
-      <c r="C71" t="inlineStr">
-        <is>
-          <t>MG_POT</t>
-        </is>
-      </c>
       <c r="D71" t="n">
-        <v>1.949292</v>
+        <v>0.507761</v>
       </c>
       <c r="E71" t="inlineStr">
         <is>
@@ -9830,12 +9830,12 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
-          <t>IA-MGCL2-MU</t>
+          <t>IA-MGCL2-KROLL</t>
         </is>
       </c>
       <c r="B72" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="C72" t="inlineStr">
@@ -9844,7 +9844,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.039782</v>
+        <v>1.949292</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -9860,21 +9860,21 @@
     <row r="73">
       <c r="A73" t="inlineStr">
         <is>
-          <t>IA-MO-VENT</t>
+          <t>IA-MGCL2-MU</t>
         </is>
       </c>
       <c r="B73" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C73" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="D73" t="n">
-        <v>0.045073</v>
+        <v>0.039782</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -9890,21 +9890,21 @@
     <row r="74">
       <c r="A74" t="inlineStr">
         <is>
-          <t>IA-MOO3-MU</t>
+          <t>IA-MO-VENT</t>
         </is>
       </c>
       <c r="B74" t="inlineStr">
         <is>
+          <t>MO_CELL</t>
+        </is>
+      </c>
+      <c r="C74" t="inlineStr">
+        <is>
           <t>NORTH_DOCK</t>
         </is>
       </c>
-      <c r="C74" t="inlineStr">
-        <is>
-          <t>MO_CELL</t>
-        </is>
-      </c>
       <c r="D74" t="n">
-        <v>0.093766</v>
+        <v>0.045073</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -9920,21 +9920,21 @@
     <row r="75">
       <c r="A75" t="inlineStr">
         <is>
-          <t>IA-SHELL-EXPORT</t>
+          <t>IA-MOO3-MU</t>
         </is>
       </c>
       <c r="B75" t="inlineStr">
         <is>
-          <t>SHELL_BREAK</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C75" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="D75" t="n">
-        <v>1</v>
+        <v>0.093766</v>
       </c>
       <c r="E75" t="inlineStr">
         <is>
@@ -9950,7 +9950,7 @@
     <row r="76">
       <c r="A76" t="inlineStr">
         <is>
-          <t>IA-SHELL-RECLAIM</t>
+          <t>IA-SHELL-EXPORT</t>
         </is>
       </c>
       <c r="B76" t="inlineStr">
@@ -9960,11 +9960,11 @@
       </c>
       <c r="C76" t="inlineStr">
         <is>
-          <t>SHELL_BUILD</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D76" t="n">
-        <v>7</v>
+        <v>1</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -9980,21 +9980,21 @@
     <row r="77">
       <c r="A77" t="inlineStr">
         <is>
-          <t>IA-SI-EG</t>
+          <t>IA-SHELL-RECLAIM</t>
         </is>
       </c>
       <c r="B77" t="inlineStr">
         <is>
-          <t>SI_REFINE</t>
+          <t>SHELL_BREAK</t>
         </is>
       </c>
       <c r="C77" t="inlineStr">
         <is>
-          <t>METAL_STORE</t>
+          <t>SHELL_BUILD</t>
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.226363</v>
+        <v>7</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -10010,12 +10010,12 @@
     <row r="78">
       <c r="A78" t="inlineStr">
         <is>
-          <t>IA-SI-IMPORT</t>
+          <t>IA-SI-EG</t>
         </is>
       </c>
       <c r="B78" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>SI_REFINE</t>
         </is>
       </c>
       <c r="C78" t="inlineStr">
@@ -10024,7 +10024,7 @@
         </is>
       </c>
       <c r="D78" t="n">
-        <v>0</v>
+        <v>0.226363</v>
       </c>
       <c r="E78" t="inlineStr">
         <is>
@@ -10040,7 +10040,7 @@
     <row r="79">
       <c r="A79" t="inlineStr">
         <is>
-          <t>IA-SILICA-MU</t>
+          <t>IA-SI-IMPORT</t>
         </is>
       </c>
       <c r="B79" t="inlineStr">
@@ -10050,11 +10050,11 @@
       </c>
       <c r="C79" t="inlineStr">
         <is>
-          <t>SHELL_BUILD</t>
+          <t>METAL_STORE</t>
         </is>
       </c>
       <c r="D79" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E79" t="inlineStr">
         <is>
@@ -10070,21 +10070,21 @@
     <row r="80">
       <c r="A80" t="inlineStr">
         <is>
-          <t>IA-STOCK-STORE</t>
+          <t>IA-SILICA-MU</t>
         </is>
       </c>
       <c r="B80" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C80" t="inlineStr">
         <is>
-          <t>METAL_STORE</t>
+          <t>SHELL_BUILD</t>
         </is>
       </c>
       <c r="D80" t="n">
-        <v>36.7125</v>
+        <v>1</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -10100,21 +10100,21 @@
     <row r="81">
       <c r="A81" t="inlineStr">
         <is>
-          <t>IA-TIO2-MU</t>
+          <t>IA-STOCK-STORE</t>
         </is>
       </c>
       <c r="B81" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="C81" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>METAL_STORE</t>
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.834247</v>
+        <v>36.7125</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -10130,7 +10130,7 @@
     <row r="82">
       <c r="A82" t="inlineStr">
         <is>
-          <t>IA-WAX-MU</t>
+          <t>IA-TIO2-MU</t>
         </is>
       </c>
       <c r="B82" t="inlineStr">
@@ -10140,11 +10140,11 @@
       </c>
       <c r="C82" t="inlineStr">
         <is>
-          <t>WAX_PATTERN</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.2</v>
+        <v>0.834247</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -10160,25 +10160,25 @@
     <row r="83">
       <c r="A83" t="inlineStr">
         <is>
-          <t>IND_HEAT_TO_HX</t>
+          <t>IA-WAX-MU</t>
         </is>
       </c>
       <c r="B83" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="C83" t="inlineStr">
         <is>
-          <t>MET_HX_Q4</t>
+          <t>WAX_PATTERN</t>
         </is>
       </c>
       <c r="D83" t="n">
-        <v>1.063</v>
+        <v>0</v>
       </c>
       <c r="E83" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F83" t="inlineStr">
@@ -10190,7 +10190,7 @@
     <row r="84">
       <c r="A84" t="inlineStr">
         <is>
-          <t>IND_MELT_TO_CAST</t>
+          <t>IND_HEAT_TO_HX</t>
         </is>
       </c>
       <c r="B84" t="inlineStr">
@@ -10200,15 +10200,15 @@
       </c>
       <c r="C84" t="inlineStr">
         <is>
-          <t>CAST_LINE</t>
+          <t>MET_HX_Q4</t>
         </is>
       </c>
       <c r="D84" t="n">
-        <v>3</v>
+        <v>1.063</v>
       </c>
       <c r="E84" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F84" t="inlineStr">
@@ -10220,7 +10220,7 @@
     <row r="85">
       <c r="A85" t="inlineStr">
         <is>
-          <t>IND_TO_ATOM</t>
+          <t>IND_MELT_TO_CAST</t>
         </is>
       </c>
       <c r="B85" t="inlineStr">
@@ -10230,11 +10230,11 @@
       </c>
       <c r="C85" t="inlineStr">
         <is>
-          <t>GAS_ATOMIZER</t>
+          <t>CAST_LINE</t>
         </is>
       </c>
       <c r="D85" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="E85" t="inlineStr">
         <is>
@@ -10250,7 +10250,7 @@
     <row r="86">
       <c r="A86" t="inlineStr">
         <is>
-          <t>IND_TO_CONT</t>
+          <t>IND_TO_ATOM</t>
         </is>
       </c>
       <c r="B86" t="inlineStr">
@@ -10260,11 +10260,11 @@
       </c>
       <c r="C86" t="inlineStr">
         <is>
-          <t>CONT_CAST</t>
+          <t>GAS_ATOMIZER</t>
         </is>
       </c>
       <c r="D86" t="n">
-        <v>31.7125</v>
+        <v>0</v>
       </c>
       <c r="E86" t="inlineStr">
         <is>
@@ -10280,7 +10280,7 @@
     <row r="87">
       <c r="A87" t="inlineStr">
         <is>
-          <t>IND_TO_INV</t>
+          <t>IND_TO_CONT</t>
         </is>
       </c>
       <c r="B87" t="inlineStr">
@@ -10290,11 +10290,11 @@
       </c>
       <c r="C87" t="inlineStr">
         <is>
-          <t>INV_CAST</t>
+          <t>CONT_CAST</t>
         </is>
       </c>
       <c r="D87" t="n">
-        <v>2</v>
+        <v>31.7125</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -10310,21 +10310,21 @@
     <row r="88">
       <c r="A88" t="inlineStr">
         <is>
-          <t>INV_TO_BREAK</t>
+          <t>IND_TO_INV</t>
         </is>
       </c>
       <c r="B88" t="inlineStr">
         <is>
+          <t>IND_MELT</t>
+        </is>
+      </c>
+      <c r="C88" t="inlineStr">
+        <is>
           <t>INV_CAST</t>
         </is>
       </c>
-      <c r="C88" t="inlineStr">
-        <is>
-          <t>SHELL_BREAK</t>
-        </is>
-      </c>
       <c r="D88" t="n">
-        <v>10</v>
+        <v>2</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -10340,21 +10340,21 @@
     <row r="89">
       <c r="A89" t="inlineStr">
         <is>
-          <t>METALS_TO_IND_MELT</t>
+          <t>INV_TO_BREAK</t>
         </is>
       </c>
       <c r="B89" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>INV_CAST</t>
         </is>
       </c>
       <c r="C89" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>SHELL_BREAK</t>
         </is>
       </c>
       <c r="D89" t="n">
-        <v>0.5</v>
+        <v>10</v>
       </c>
       <c r="E89" t="inlineStr">
         <is>
@@ -10370,12 +10370,12 @@
     <row r="90">
       <c r="A90" t="inlineStr">
         <is>
-          <t>MFG_SCRAP_TO_IND</t>
+          <t>METALS_TO_IND_MELT</t>
         </is>
       </c>
       <c r="B90" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="C90" t="inlineStr">
@@ -10384,7 +10384,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>26.161616</v>
+        <v>0.5</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -10400,21 +10400,21 @@
     <row r="91">
       <c r="A91" t="inlineStr">
         <is>
-          <t>MG_POT_CL2</t>
+          <t>MFG_SCRAP_TO_IND</t>
         </is>
       </c>
       <c r="B91" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="C91" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D91" t="n">
-        <v>0</v>
+        <v>26.161616</v>
       </c>
       <c r="E91" t="inlineStr">
         <is>
@@ -10430,7 +10430,7 @@
     <row r="92">
       <c r="A92" t="inlineStr">
         <is>
-          <t>MG_POT_TO_IND</t>
+          <t>MG_POT_CL2</t>
         </is>
       </c>
       <c r="B92" t="inlineStr">
@@ -10440,7 +10440,7 @@
       </c>
       <c r="C92" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D92" t="n">
@@ -10460,17 +10460,17 @@
     <row r="93">
       <c r="A93" t="inlineStr">
         <is>
-          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
+          <t>MG_POT_TO_IND</t>
         </is>
       </c>
       <c r="B93" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="C93" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D93" t="n">
@@ -10490,7 +10490,7 @@
     <row r="94">
       <c r="A94" t="inlineStr">
         <is>
-          <t>MO_CELL_RAFFINATE</t>
+          <t>MO_CELL_ANODE_GAS_TO_CRU</t>
         </is>
       </c>
       <c r="B94" t="inlineStr">
@@ -10500,7 +10500,7 @@
       </c>
       <c r="C94" t="inlineStr">
         <is>
-          <t>POLISH_BANK</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D94" t="n">
@@ -10520,7 +10520,7 @@
     <row r="95">
       <c r="A95" t="inlineStr">
         <is>
-          <t>MO_TO_IND</t>
+          <t>MO_CELL_RAFFINATE</t>
         </is>
       </c>
       <c r="B95" t="inlineStr">
@@ -10530,11 +10530,11 @@
       </c>
       <c r="C95" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>POLISH_BANK</t>
         </is>
       </c>
       <c r="D95" t="n">
-        <v>0.0625</v>
+        <v>0</v>
       </c>
       <c r="E95" t="inlineStr">
         <is>
@@ -10550,21 +10550,21 @@
     <row r="96">
       <c r="A96" t="inlineStr">
         <is>
-          <t>ROLL_TO_STOCK</t>
+          <t>MO_TO_IND</t>
         </is>
       </c>
       <c r="B96" t="inlineStr">
         <is>
-          <t>ROLL</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="C96" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D96" t="n">
-        <v>13</v>
+        <v>0.0625</v>
       </c>
       <c r="E96" t="inlineStr">
         <is>
@@ -10580,21 +10580,21 @@
     <row r="97">
       <c r="A97" t="inlineStr">
         <is>
-          <t>SALT_TO_FLUX</t>
+          <t>ROLL_TO_STOCK</t>
         </is>
       </c>
       <c r="B97" t="inlineStr">
         <is>
-          <t>SALT_FEED</t>
+          <t>ROLL</t>
         </is>
       </c>
       <c r="C97" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="D97" t="n">
-        <v>0</v>
+        <v>13</v>
       </c>
       <c r="E97" t="inlineStr">
         <is>
@@ -10610,25 +10610,25 @@
     <row r="98">
       <c r="A98" t="inlineStr">
         <is>
-          <t>SF-AL_POT</t>
+          <t>SALT_TO_FLUX</t>
         </is>
       </c>
       <c r="B98" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>SALT_FEED</t>
         </is>
       </c>
       <c r="C98" t="inlineStr">
         <is>
-          <t>AL_POT</t>
+          <t>FLUX_PREP</t>
         </is>
       </c>
       <c r="D98" t="n">
-        <v>5.6578</v>
+        <v>0</v>
       </c>
       <c r="E98" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F98" t="inlineStr">
@@ -10640,7 +10640,7 @@
     <row r="99">
       <c r="A99" t="inlineStr">
         <is>
-          <t>SF-CA_POT</t>
+          <t>SF-AL_POT</t>
         </is>
       </c>
       <c r="B99" t="inlineStr">
@@ -10650,11 +10650,11 @@
       </c>
       <c r="C99" t="inlineStr">
         <is>
-          <t>CA_POT</t>
+          <t>AL_POT</t>
         </is>
       </c>
       <c r="D99" t="n">
-        <v>0.1221</v>
+        <v>5.6578</v>
       </c>
       <c r="E99" t="inlineStr">
         <is>
@@ -10670,7 +10670,7 @@
     <row r="100">
       <c r="A100" t="inlineStr">
         <is>
-          <t>SF-COMB_HEAT</t>
+          <t>SF-CA_POT</t>
         </is>
       </c>
       <c r="B100" t="inlineStr">
@@ -10680,11 +10680,11 @@
       </c>
       <c r="C100" t="inlineStr">
         <is>
-          <t>COMB_HEAT</t>
+          <t>CA_POT</t>
         </is>
       </c>
       <c r="D100" t="n">
-        <v>0.05</v>
+        <v>0.1221</v>
       </c>
       <c r="E100" t="inlineStr">
         <is>
@@ -10700,7 +10700,7 @@
     <row r="101">
       <c r="A101" t="inlineStr">
         <is>
-          <t>SF-CR_CELL</t>
+          <t>SF-COMB_HEAT</t>
         </is>
       </c>
       <c r="B101" t="inlineStr">
@@ -10710,11 +10710,11 @@
       </c>
       <c r="C101" t="inlineStr">
         <is>
-          <t>CR_CELL</t>
+          <t>COMB_HEAT</t>
         </is>
       </c>
       <c r="D101" t="n">
-        <v>0.16</v>
+        <v>0.05</v>
       </c>
       <c r="E101" t="inlineStr">
         <is>
@@ -10730,7 +10730,7 @@
     <row r="102">
       <c r="A102" t="inlineStr">
         <is>
-          <t>SF-DRAW</t>
+          <t>SF-CR_CELL</t>
         </is>
       </c>
       <c r="B102" t="inlineStr">
@@ -10740,11 +10740,11 @@
       </c>
       <c r="C102" t="inlineStr">
         <is>
-          <t>DRAW</t>
+          <t>CR_CELL</t>
         </is>
       </c>
       <c r="D102" t="n">
-        <v>0</v>
+        <v>0.16</v>
       </c>
       <c r="E102" t="inlineStr">
         <is>
@@ -10760,7 +10760,7 @@
     <row r="103">
       <c r="A103" t="inlineStr">
         <is>
-          <t>SF-EXTRUDE</t>
+          <t>SF-DRAW</t>
         </is>
       </c>
       <c r="B103" t="inlineStr">
@@ -10770,7 +10770,7 @@
       </c>
       <c r="C103" t="inlineStr">
         <is>
-          <t>EXTRUDE</t>
+          <t>DRAW</t>
         </is>
       </c>
       <c r="D103" t="n">
@@ -10790,7 +10790,7 @@
     <row r="104">
       <c r="A104" t="inlineStr">
         <is>
-          <t>SF-FLUX_PREP</t>
+          <t>SF-EXTRUDE</t>
         </is>
       </c>
       <c r="B104" t="inlineStr">
@@ -10800,11 +10800,11 @@
       </c>
       <c r="C104" t="inlineStr">
         <is>
-          <t>FLUX_PREP</t>
+          <t>EXTRUDE</t>
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.1</v>
+        <v>0</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -10820,7 +10820,7 @@
     <row r="105">
       <c r="A105" t="inlineStr">
         <is>
-          <t>SF-FORGE</t>
+          <t>SF-FLUX_PREP</t>
         </is>
       </c>
       <c r="B105" t="inlineStr">
@@ -10830,11 +10830,11 @@
       </c>
       <c r="C105" t="inlineStr">
         <is>
-          <t>FORGE</t>
+          <t>FLUX_PREP</t>
         </is>
       </c>
       <c r="D105" t="n">
-        <v>0</v>
+        <v>0.1</v>
       </c>
       <c r="E105" t="inlineStr">
         <is>
@@ -10850,7 +10850,7 @@
     <row r="106">
       <c r="A106" t="inlineStr">
         <is>
-          <t>SF-IND_MELT</t>
+          <t>SF-FORGE</t>
         </is>
       </c>
       <c r="B106" t="inlineStr">
@@ -10860,11 +10860,11 @@
       </c>
       <c r="C106" t="inlineStr">
         <is>
-          <t>IND_MELT</t>
+          <t>FORGE</t>
         </is>
       </c>
       <c r="D106" t="n">
-        <v>0.8854</v>
+        <v>0</v>
       </c>
       <c r="E106" t="inlineStr">
         <is>
@@ -10880,7 +10880,7 @@
     <row r="107">
       <c r="A107" t="inlineStr">
         <is>
-          <t>SF-INV_CAST</t>
+          <t>SF-IND_MELT</t>
         </is>
       </c>
       <c r="B107" t="inlineStr">
@@ -10890,11 +10890,11 @@
       </c>
       <c r="C107" t="inlineStr">
         <is>
-          <t>INV_CAST</t>
+          <t>IND_MELT</t>
         </is>
       </c>
       <c r="D107" t="n">
-        <v>0.15</v>
+        <v>0.8854</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -10910,7 +10910,7 @@
     <row r="108">
       <c r="A108" t="inlineStr">
         <is>
-          <t>SF-MG_POT</t>
+          <t>SF-INV_CAST</t>
         </is>
       </c>
       <c r="B108" t="inlineStr">
@@ -10920,11 +10920,11 @@
       </c>
       <c r="C108" t="inlineStr">
         <is>
-          <t>MG_POT</t>
+          <t>INV_CAST</t>
         </is>
       </c>
       <c r="D108" t="n">
-        <v>0.3375</v>
+        <v>0.15</v>
       </c>
       <c r="E108" t="inlineStr">
         <is>
@@ -10940,7 +10940,7 @@
     <row r="109">
       <c r="A109" t="inlineStr">
         <is>
-          <t>SF-MO_CELL</t>
+          <t>SF-MG_POT</t>
         </is>
       </c>
       <c r="B109" t="inlineStr">
@@ -10950,11 +10950,11 @@
       </c>
       <c r="C109" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>MG_POT</t>
         </is>
       </c>
       <c r="D109" t="n">
-        <v>0.1141</v>
+        <v>0.3375</v>
       </c>
       <c r="E109" t="inlineStr">
         <is>
@@ -10970,7 +10970,7 @@
     <row r="110">
       <c r="A110" t="inlineStr">
         <is>
-          <t>SF-RES_HEAT</t>
+          <t>SF-MO_CELL</t>
         </is>
       </c>
       <c r="B110" t="inlineStr">
@@ -10980,11 +10980,11 @@
       </c>
       <c r="C110" t="inlineStr">
         <is>
-          <t>RES_HEAT</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="D110" t="n">
-        <v>0</v>
+        <v>0.1141</v>
       </c>
       <c r="E110" t="inlineStr">
         <is>
@@ -11000,7 +11000,7 @@
     <row r="111">
       <c r="A111" t="inlineStr">
         <is>
-          <t>SF-RF_HEAT</t>
+          <t>SF-RES_HEAT</t>
         </is>
       </c>
       <c r="B111" t="inlineStr">
@@ -11010,7 +11010,7 @@
       </c>
       <c r="C111" t="inlineStr">
         <is>
-          <t>RF_HEAT</t>
+          <t>RES_HEAT</t>
         </is>
       </c>
       <c r="D111" t="n">
@@ -11030,7 +11030,7 @@
     <row r="112">
       <c r="A112" t="inlineStr">
         <is>
-          <t>SF-SHELL_BREAK</t>
+          <t>SF-RF_HEAT</t>
         </is>
       </c>
       <c r="B112" t="inlineStr">
@@ -11040,11 +11040,11 @@
       </c>
       <c r="C112" t="inlineStr">
         <is>
-          <t>SHELL_BREAK</t>
+          <t>RF_HEAT</t>
         </is>
       </c>
       <c r="D112" t="n">
-        <v>0.4</v>
+        <v>0</v>
       </c>
       <c r="E112" t="inlineStr">
         <is>
@@ -11060,7 +11060,7 @@
     <row r="113">
       <c r="A113" t="inlineStr">
         <is>
-          <t>SF-SHELL_BUILD</t>
+          <t>SF-SHELL_BREAK</t>
         </is>
       </c>
       <c r="B113" t="inlineStr">
@@ -11070,11 +11070,11 @@
       </c>
       <c r="C113" t="inlineStr">
         <is>
-          <t>SHELL_BUILD</t>
+          <t>SHELL_BREAK</t>
         </is>
       </c>
       <c r="D113" t="n">
-        <v>0.3</v>
+        <v>0.4</v>
       </c>
       <c r="E113" t="inlineStr">
         <is>
@@ -11090,7 +11090,7 @@
     <row r="114">
       <c r="A114" t="inlineStr">
         <is>
-          <t>SF-SHELL_BURNOUT</t>
+          <t>SF-SHELL_BUILD</t>
         </is>
       </c>
       <c r="B114" t="inlineStr">
@@ -11100,11 +11100,11 @@
       </c>
       <c r="C114" t="inlineStr">
         <is>
-          <t>SHELL_BURNOUT</t>
+          <t>SHELL_BUILD</t>
         </is>
       </c>
       <c r="D114" t="n">
-        <v>0.25</v>
+        <v>0.3</v>
       </c>
       <c r="E114" t="inlineStr">
         <is>
@@ -11120,7 +11120,7 @@
     <row r="115">
       <c r="A115" t="inlineStr">
         <is>
-          <t>SF-SINTER</t>
+          <t>SF-SHELL_BURNOUT</t>
         </is>
       </c>
       <c r="B115" t="inlineStr">
@@ -11130,11 +11130,11 @@
       </c>
       <c r="C115" t="inlineStr">
         <is>
-          <t>SINTER</t>
+          <t>SHELL_BURNOUT</t>
         </is>
       </c>
       <c r="D115" t="n">
-        <v>0</v>
+        <v>0.25</v>
       </c>
       <c r="E115" t="inlineStr">
         <is>
@@ -11150,7 +11150,7 @@
     <row r="116">
       <c r="A116" t="inlineStr">
         <is>
-          <t>SF-TI_CELL</t>
+          <t>SF-SINTER</t>
         </is>
       </c>
       <c r="B116" t="inlineStr">
@@ -11160,11 +11160,11 @@
       </c>
       <c r="C116" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>SINTER</t>
         </is>
       </c>
       <c r="D116" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E116" t="inlineStr">
         <is>
@@ -11180,7 +11180,7 @@
     <row r="117">
       <c r="A117" t="inlineStr">
         <is>
-          <t>SF-VAC_CAST</t>
+          <t>SF-TI_CELL</t>
         </is>
       </c>
       <c r="B117" t="inlineStr">
@@ -11190,11 +11190,11 @@
       </c>
       <c r="C117" t="inlineStr">
         <is>
-          <t>VAC_CAST</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D117" t="n">
-        <v>0</v>
+        <v>0.5</v>
       </c>
       <c r="E117" t="inlineStr">
         <is>
@@ -11210,7 +11210,7 @@
     <row r="118">
       <c r="A118" t="inlineStr">
         <is>
-          <t>SF-VAC_IND</t>
+          <t>SF-VAC_CAST</t>
         </is>
       </c>
       <c r="B118" t="inlineStr">
@@ -11220,7 +11220,7 @@
       </c>
       <c r="C118" t="inlineStr">
         <is>
-          <t>VAC_IND</t>
+          <t>VAC_CAST</t>
         </is>
       </c>
       <c r="D118" t="n">
@@ -11240,7 +11240,7 @@
     <row r="119">
       <c r="A119" t="inlineStr">
         <is>
-          <t>SF-WAX_PATTERN</t>
+          <t>SF-VAC_IND</t>
         </is>
       </c>
       <c r="B119" t="inlineStr">
@@ -11250,11 +11250,11 @@
       </c>
       <c r="C119" t="inlineStr">
         <is>
-          <t>WAX_PATTERN</t>
+          <t>VAC_IND</t>
         </is>
       </c>
       <c r="D119" t="n">
-        <v>0.5</v>
+        <v>0</v>
       </c>
       <c r="E119" t="inlineStr">
         <is>
@@ -11270,25 +11270,25 @@
     <row r="120">
       <c r="A120" t="inlineStr">
         <is>
-          <t>SHELL_TO_BURNOUT</t>
+          <t>SF-WAX_PATTERN</t>
         </is>
       </c>
       <c r="B120" t="inlineStr">
         <is>
-          <t>SHELL_BUILD</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C120" t="inlineStr">
         <is>
-          <t>SHELL_BURNOUT</t>
+          <t>WAX_PATTERN</t>
         </is>
       </c>
       <c r="D120" t="n">
-        <v>10</v>
+        <v>0.5</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F120" t="inlineStr">
@@ -11300,21 +11300,21 @@
     <row r="121">
       <c r="A121" t="inlineStr">
         <is>
-          <t>SHELL_TO_GLASS</t>
+          <t>SHELL_TO_BURNOUT</t>
         </is>
       </c>
       <c r="B121" t="inlineStr">
         <is>
-          <t>SHELL_BREAK</t>
+          <t>SHELL_BUILD</t>
         </is>
       </c>
       <c r="C121" t="inlineStr">
         <is>
-          <t>GLASS_MILL</t>
+          <t>SHELL_BURNOUT</t>
         </is>
       </c>
       <c r="D121" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -11330,17 +11330,17 @@
     <row r="122">
       <c r="A122" t="inlineStr">
         <is>
-          <t>SINTER_TO_STOCK</t>
+          <t>SHELL_TO_GLASS</t>
         </is>
       </c>
       <c r="B122" t="inlineStr">
         <is>
-          <t>SINTER</t>
+          <t>SHELL_BREAK</t>
         </is>
       </c>
       <c r="C122" t="inlineStr">
         <is>
-          <t>STOCK_OUT</t>
+          <t>GLASS_MILL</t>
         </is>
       </c>
       <c r="D122" t="n">
@@ -11360,21 +11360,21 @@
     <row r="123">
       <c r="A123" t="inlineStr">
         <is>
-          <t>STOCK_TO_FAB</t>
+          <t>SINTER_TO_STOCK</t>
         </is>
       </c>
       <c r="B123" t="inlineStr">
         <is>
-          <t>METAL_STORE</t>
+          <t>SINTER</t>
         </is>
       </c>
       <c r="C123" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>STOCK_OUT</t>
         </is>
       </c>
       <c r="D123" t="n">
-        <v>0.226363</v>
+        <v>0</v>
       </c>
       <c r="E123" t="inlineStr">
         <is>
@@ -11390,7 +11390,7 @@
     <row r="124">
       <c r="A124" t="inlineStr">
         <is>
-          <t>STOCK_TO_MFG</t>
+          <t>STOCK_TO_FAB</t>
         </is>
       </c>
       <c r="B124" t="inlineStr">
@@ -11400,11 +11400,11 @@
       </c>
       <c r="C124" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="D124" t="n">
-        <v>25.9</v>
+        <v>0.226363</v>
       </c>
       <c r="E124" t="inlineStr">
         <is>
@@ -11420,7 +11420,7 @@
     <row r="125">
       <c r="A125" t="inlineStr">
         <is>
-          <t>STOCK_TO_WIRE_DRAW</t>
+          <t>STOCK_TO_MFG</t>
         </is>
       </c>
       <c r="B125" t="inlineStr">
@@ -11430,11 +11430,11 @@
       </c>
       <c r="C125" t="inlineStr">
         <is>
-          <t>WIRE_DRAW</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D125" t="n">
-        <v>0</v>
+        <v>25.9</v>
       </c>
       <c r="E125" t="inlineStr">
         <is>
@@ -11450,17 +11450,17 @@
     <row r="126">
       <c r="A126" t="inlineStr">
         <is>
-          <t>TI_CELL_CL2_TO_CRU</t>
+          <t>STOCK_TO_WIRE_DRAW</t>
         </is>
       </c>
       <c r="B126" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>METAL_STORE</t>
         </is>
       </c>
       <c r="C126" t="inlineStr">
         <is>
-          <t>CRU</t>
+          <t>WIRE_DRAW</t>
         </is>
       </c>
       <c r="D126" t="n">
@@ -11480,7 +11480,7 @@
     <row r="127">
       <c r="A127" t="inlineStr">
         <is>
-          <t>TI_CELL_SLAG_RETURN</t>
+          <t>TI_CELL_CL2_TO_CRU</t>
         </is>
       </c>
       <c r="B127" t="inlineStr">
@@ -11490,7 +11490,7 @@
       </c>
       <c r="C127" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>CRU</t>
         </is>
       </c>
       <c r="D127" t="n">
@@ -11510,25 +11510,25 @@
     <row r="128">
       <c r="A128" t="inlineStr">
         <is>
-          <t>VAC_HEAT_TO_HX</t>
+          <t>TI_CELL_SLAG_RETURN</t>
         </is>
       </c>
       <c r="B128" t="inlineStr">
         <is>
-          <t>VAC_IND</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="C128" t="inlineStr">
         <is>
-          <t>MET_HX_Q4</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="D128" t="n">
-        <v>0.638</v>
+        <v>0</v>
       </c>
       <c r="E128" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F128" t="inlineStr">
@@ -11540,25 +11540,25 @@
     <row r="129">
       <c r="A129" t="inlineStr">
         <is>
-          <t>VAC_IND_TI</t>
+          <t>VAC_HEAT_TO_HX</t>
         </is>
       </c>
       <c r="B129" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>VAC_IND</t>
         </is>
       </c>
       <c r="C129" t="inlineStr">
         <is>
-          <t>VAC_IND</t>
+          <t>MET_HX_Q4</t>
         </is>
       </c>
       <c r="D129" t="n">
-        <v>0</v>
+        <v>0.638</v>
       </c>
       <c r="E129" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F129" t="inlineStr">
@@ -11570,17 +11570,17 @@
     <row r="130">
       <c r="A130" t="inlineStr">
         <is>
-          <t>VAC_IND_TO_VAC_CAST</t>
+          <t>VAC_IND_TI</t>
         </is>
       </c>
       <c r="B130" t="inlineStr">
         <is>
+          <t>TI_CELL</t>
+        </is>
+      </c>
+      <c r="C130" t="inlineStr">
+        <is>
           <t>VAC_IND</t>
-        </is>
-      </c>
-      <c r="C130" t="inlineStr">
-        <is>
-          <t>VAC_CAST</t>
         </is>
       </c>
       <c r="D130" t="n">
@@ -11600,7 +11600,7 @@
     <row r="131">
       <c r="A131" t="inlineStr">
         <is>
-          <t>VAC_TO_INV</t>
+          <t>VAC_IND_TO_VAC_CAST</t>
         </is>
       </c>
       <c r="B131" t="inlineStr">
@@ -11610,7 +11610,7 @@
       </c>
       <c r="C131" t="inlineStr">
         <is>
-          <t>INV_CAST</t>
+          <t>VAC_CAST</t>
         </is>
       </c>
       <c r="D131" t="n">
@@ -11630,21 +11630,21 @@
     <row r="132">
       <c r="A132" t="inlineStr">
         <is>
-          <t>WAX_RECLAIM_TO_PATTERN</t>
+          <t>VAC_TO_INV</t>
         </is>
       </c>
       <c r="B132" t="inlineStr">
         <is>
-          <t>SHELL_BURNOUT</t>
+          <t>VAC_IND</t>
         </is>
       </c>
       <c r="C132" t="inlineStr">
         <is>
-          <t>WAX_PATTERN</t>
+          <t>INV_CAST</t>
         </is>
       </c>
       <c r="D132" t="n">
-        <v>1.8</v>
+        <v>0</v>
       </c>
       <c r="E132" t="inlineStr">
         <is>
@@ -11660,7 +11660,7 @@
     <row r="133">
       <c r="A133" t="inlineStr">
         <is>
-          <t>WAX_TO_OIL</t>
+          <t>WAX_RECLAIM_TO_PATTERN</t>
         </is>
       </c>
       <c r="B133" t="inlineStr">
@@ -11670,11 +11670,11 @@
       </c>
       <c r="C133" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>WAX_PATTERN</t>
         </is>
       </c>
       <c r="D133" t="n">
-        <v>0</v>
+        <v>1.8</v>
       </c>
       <c r="E133" t="inlineStr">
         <is>
@@ -11690,28 +11690,58 @@
     <row r="134">
       <c r="A134" t="inlineStr">
         <is>
+          <t>WAX_TO_OIL</t>
+        </is>
+      </c>
+      <c r="B134" t="inlineStr">
+        <is>
+          <t>SHELL_BURNOUT</t>
+        </is>
+      </c>
+      <c r="C134" t="inlineStr">
+        <is>
+          <t>OIL_FRAC</t>
+        </is>
+      </c>
+      <c r="D134" t="n">
+        <v>0</v>
+      </c>
+      <c r="E134" t="inlineStr">
+        <is>
+          <t>kg/d</t>
+        </is>
+      </c>
+      <c r="F134" t="inlineStr">
+        <is>
+          <t>study</t>
+        </is>
+      </c>
+    </row>
+    <row r="135">
+      <c r="A135" t="inlineStr">
+        <is>
           <t>WAX_TO_SHELL</t>
         </is>
       </c>
-      <c r="B134" t="inlineStr">
+      <c r="B135" t="inlineStr">
         <is>
           <t>WAX_PATTERN</t>
         </is>
       </c>
-      <c r="C134" t="inlineStr">
+      <c r="C135" t="inlineStr">
         <is>
           <t>SHELL_BUILD</t>
         </is>
       </c>
-      <c r="D134" t="n">
+      <c r="D135" t="n">
         <v>2</v>
       </c>
-      <c r="E134" t="inlineStr">
+      <c r="E135" t="inlineStr">
         <is>
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F134" t="inlineStr">
+      <c r="F135" t="inlineStr">
         <is>
           <t>study</t>
         </is>
@@ -55465,7 +55495,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2.218146</v>
+        <v>2.018146</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -56665,7 +56695,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.2</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -75906,7 +75936,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H72"/>
+  <dimension ref="A1:H73"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="24" customWidth="1" min="1" max="1"/>
@@ -76390,21 +76420,21 @@
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>C29_RECYCLE</t>
+          <t>C19_TO_WAX</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>PROD_C29</t>
+          <t>PROD_C19_C28</t>
         </is>
       </c>
       <c r="C21" t="inlineStr">
         <is>
-          <t>C29_RECYCLE</t>
+          <t>WAX_PATTERN</t>
         </is>
       </c>
       <c r="D21" t="n">
-        <v>5.873266</v>
+        <v>0.2</v>
       </c>
       <c r="E21" t="inlineStr">
         <is>
@@ -76420,17 +76450,17 @@
     <row r="22">
       <c r="A22" t="inlineStr">
         <is>
-          <t>C29_TO_PYRO</t>
+          <t>C29_RECYCLE</t>
         </is>
       </c>
       <c r="B22" t="inlineStr">
         <is>
+          <t>PROD_C29</t>
+        </is>
+      </c>
+      <c r="C22" t="inlineStr">
+        <is>
           <t>C29_RECYCLE</t>
-        </is>
-      </c>
-      <c r="C22" t="inlineStr">
-        <is>
-          <t>OIL_PYRO</t>
         </is>
       </c>
       <c r="D22" t="n">
@@ -76450,21 +76480,21 @@
     <row r="23">
       <c r="A23" t="inlineStr">
         <is>
-          <t>CHAR_TO_ACID</t>
+          <t>C29_TO_PYRO</t>
         </is>
       </c>
       <c r="B23" t="inlineStr">
         <is>
+          <t>C29_RECYCLE</t>
+        </is>
+      </c>
+      <c r="C23" t="inlineStr">
+        <is>
           <t>OIL_PYRO</t>
         </is>
       </c>
-      <c r="C23" t="inlineStr">
-        <is>
-          <t>ACID_PLANT</t>
-        </is>
-      </c>
       <c r="D23" t="n">
-        <v>0.025656</v>
+        <v>5.873266</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -76480,7 +76510,7 @@
     <row r="24">
       <c r="A24" t="inlineStr">
         <is>
-          <t>CHAR_TO_SI</t>
+          <t>CHAR_TO_ACID</t>
         </is>
       </c>
       <c r="B24" t="inlineStr">
@@ -76490,11 +76520,11 @@
       </c>
       <c r="C24" t="inlineStr">
         <is>
-          <t>SI_REDUCE</t>
+          <t>ACID_PLANT</t>
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.227778</v>
+        <v>0.025656</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -76510,21 +76540,21 @@
     <row r="25">
       <c r="A25" t="inlineStr">
         <is>
-          <t>CUT-1</t>
+          <t>CHAR_TO_SI</t>
         </is>
       </c>
       <c r="B25" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>OIL_PYRO</t>
         </is>
       </c>
       <c r="C25" t="inlineStr">
         <is>
-          <t>PROD_C5_C10</t>
+          <t>SI_REDUCE</t>
         </is>
       </c>
       <c r="D25" t="n">
-        <v>7.424773</v>
+        <v>0.227778</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -76540,21 +76570,21 @@
     <row r="26">
       <c r="A26" t="inlineStr">
         <is>
-          <t>CUT-1-OUT</t>
+          <t>CUT-1</t>
         </is>
       </c>
       <c r="B26" t="inlineStr">
         <is>
+          <t>OIL_FRAC</t>
+        </is>
+      </c>
+      <c r="C26" t="inlineStr">
+        <is>
           <t>PROD_C5_C10</t>
         </is>
       </c>
-      <c r="C26" t="inlineStr">
-        <is>
-          <t>BACKUP_GEN</t>
-        </is>
-      </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>7.424773</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -76570,21 +76600,21 @@
     <row r="27">
       <c r="A27" t="inlineStr">
         <is>
-          <t>CUT-2</t>
+          <t>CUT-1-OUT</t>
         </is>
       </c>
       <c r="B27" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>PROD_C5_C10</t>
         </is>
       </c>
       <c r="C27" t="inlineStr">
         <is>
-          <t>PROD_C11_C18</t>
+          <t>BACKUP_GEN</t>
         </is>
       </c>
       <c r="D27" t="n">
-        <v>9.918820999999999</v>
+        <v>0</v>
       </c>
       <c r="E27" t="inlineStr">
         <is>
@@ -76600,7 +76630,7 @@
     <row r="28">
       <c r="A28" t="inlineStr">
         <is>
-          <t>CUT-3</t>
+          <t>CUT-2</t>
         </is>
       </c>
       <c r="B28" t="inlineStr">
@@ -76610,11 +76640,11 @@
       </c>
       <c r="C28" t="inlineStr">
         <is>
-          <t>PROD_C19_C28</t>
+          <t>PROD_C11_C18</t>
         </is>
       </c>
       <c r="D28" t="n">
-        <v>6.165705</v>
+        <v>9.918820999999999</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -76630,21 +76660,21 @@
     <row r="29">
       <c r="A29" t="inlineStr">
         <is>
-          <t>CUT-3-OUT</t>
+          <t>CUT-3</t>
         </is>
       </c>
       <c r="B29" t="inlineStr">
         <is>
+          <t>OIL_FRAC</t>
+        </is>
+      </c>
+      <c r="C29" t="inlineStr">
+        <is>
           <t>PROD_C19_C28</t>
         </is>
       </c>
-      <c r="C29" t="inlineStr">
-        <is>
-          <t>MFG_SHOP</t>
-        </is>
-      </c>
       <c r="D29" t="n">
-        <v>3.947559</v>
+        <v>6.165705</v>
       </c>
       <c r="E29" t="inlineStr">
         <is>
@@ -76660,21 +76690,21 @@
     <row r="30">
       <c r="A30" t="inlineStr">
         <is>
-          <t>CUT-4</t>
+          <t>CUT-3-OUT</t>
         </is>
       </c>
       <c r="B30" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>PROD_C19_C28</t>
         </is>
       </c>
       <c r="C30" t="inlineStr">
         <is>
-          <t>PROD_C29</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D30" t="n">
-        <v>5.873266</v>
+        <v>3.947559</v>
       </c>
       <c r="E30" t="inlineStr">
         <is>
@@ -76690,34 +76720,42 @@
     <row r="31">
       <c r="A31" t="inlineStr">
         <is>
-          <t>GREASE_CA_TO_MFG</t>
+          <t>CUT-4</t>
         </is>
       </c>
       <c r="B31" t="inlineStr">
         <is>
-          <t>GREASE_CA</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="C31" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>PROD_C29</t>
+        </is>
+      </c>
+      <c r="D31" t="n">
+        <v>5.873266</v>
+      </c>
+      <c r="E31" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F31" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="32">
       <c r="A32" t="inlineStr">
         <is>
-          <t>GREASE_LI_TO_MFG</t>
+          <t>GREASE_CA_TO_MFG</t>
         </is>
       </c>
       <c r="B32" t="inlineStr">
         <is>
-          <t>GREASE_LI</t>
+          <t>GREASE_CA</t>
         </is>
       </c>
       <c r="C32" t="inlineStr">
@@ -76734,37 +76772,29 @@
     <row r="33">
       <c r="A33" t="inlineStr">
         <is>
-          <t>HL-AFTERBURNER-Q1-A</t>
+          <t>GREASE_LI_TO_MFG</t>
         </is>
       </c>
       <c r="B33" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
+          <t>GREASE_LI</t>
         </is>
       </c>
       <c r="C33" t="inlineStr">
         <is>
-          <t>Q1_A</t>
-        </is>
-      </c>
-      <c r="D33" t="n">
-        <v>1.383</v>
-      </c>
-      <c r="E33" t="inlineStr">
-        <is>
-          <t>kW</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="F33" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="34">
       <c r="A34" t="inlineStr">
         <is>
-          <t>HL-AFTERBURNER-Q1-B</t>
+          <t>HL-AFTERBURNER-Q1-A</t>
         </is>
       </c>
       <c r="B34" t="inlineStr">
@@ -76774,7 +76804,7 @@
       </c>
       <c r="C34" t="inlineStr">
         <is>
-          <t>Q1_B</t>
+          <t>Q1_A</t>
         </is>
       </c>
       <c r="D34" t="n">
@@ -76794,21 +76824,21 @@
     <row r="35">
       <c r="A35" t="inlineStr">
         <is>
-          <t>HL-Q3-A-HX4</t>
+          <t>HL-AFTERBURNER-Q1-B</t>
         </is>
       </c>
       <c r="B35" t="inlineStr">
         <is>
-          <t>Q3_A</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="C35" t="inlineStr">
         <is>
-          <t>OIL_DRYER</t>
+          <t>Q1_B</t>
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.0553</v>
+        <v>1.383</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -76824,12 +76854,12 @@
     <row r="36">
       <c r="A36" t="inlineStr">
         <is>
-          <t>HL-Q3-B-HX4</t>
+          <t>HL-Q3-A-HX4</t>
         </is>
       </c>
       <c r="B36" t="inlineStr">
         <is>
-          <t>Q3_B</t>
+          <t>Q3_A</t>
         </is>
       </c>
       <c r="C36" t="inlineStr">
@@ -76854,25 +76884,25 @@
     <row r="37">
       <c r="A37" t="inlineStr">
         <is>
-          <t>IA-AB-FLUE</t>
+          <t>HL-Q3-B-HX4</t>
         </is>
       </c>
       <c r="B37" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
+          <t>Q3_B</t>
         </is>
       </c>
       <c r="C37" t="inlineStr">
         <is>
-          <t>AFTERBURNER_FLUE</t>
+          <t>OIL_DRYER</t>
         </is>
       </c>
       <c r="D37" t="n">
-        <v>7.096878</v>
+        <v>0.0553</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
-          <t>kg/d</t>
+          <t>kW</t>
         </is>
       </c>
       <c r="F37" t="inlineStr">
@@ -76884,21 +76914,21 @@
     <row r="38">
       <c r="A38" t="inlineStr">
         <is>
-          <t>IA-AB-O2</t>
+          <t>IA-AB-FLUE</t>
         </is>
       </c>
       <c r="B38" t="inlineStr">
         <is>
-          <t>HDR_O2</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="C38" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
+          <t>AFTERBURNER_FLUE</t>
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.528278</v>
+        <v>7.096878</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>
@@ -76914,12 +76944,12 @@
     <row r="39">
       <c r="A39" t="inlineStr">
         <is>
-          <t>IA-BLK-CAKE</t>
+          <t>IA-AB-O2</t>
         </is>
       </c>
       <c r="B39" t="inlineStr">
         <is>
-          <t>BLACK_DIGEST</t>
+          <t>HDR_O2</t>
         </is>
       </c>
       <c r="C39" t="inlineStr">
@@ -76928,7 +76958,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.67</v>
+        <v>0.528278</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -76944,7 +76974,7 @@
     <row r="40">
       <c r="A40" t="inlineStr">
         <is>
-          <t>IA-BLK-GAS</t>
+          <t>IA-BLK-CAKE</t>
         </is>
       </c>
       <c r="B40" t="inlineStr">
@@ -76958,7 +76988,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.09859999999999999</v>
+        <v>0.67</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -76974,21 +77004,21 @@
     <row r="41">
       <c r="A41" t="inlineStr">
         <is>
-          <t>IA-BLOW-IN</t>
+          <t>IA-BLK-GAS</t>
         </is>
       </c>
       <c r="B41" t="inlineStr">
         <is>
-          <t>PROD_C11_C18</t>
+          <t>BLACK_DIGEST</t>
         </is>
       </c>
       <c r="C41" t="inlineStr">
         <is>
-          <t>BLOW_MOLD</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="D41" t="n">
-        <v>8.407159</v>
+        <v>0.09859999999999999</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -77004,21 +77034,21 @@
     <row r="42">
       <c r="A42" t="inlineStr">
         <is>
-          <t>IA-C-CR</t>
+          <t>IA-BLOW-IN</t>
         </is>
       </c>
       <c r="B42" t="inlineStr">
         <is>
-          <t>OIL_PYRO</t>
+          <t>PROD_C11_C18</t>
         </is>
       </c>
       <c r="C42" t="inlineStr">
         <is>
-          <t>CR_CELL</t>
+          <t>BLOW_MOLD</t>
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.101911</v>
+        <v>8.407159</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -77034,7 +77064,7 @@
     <row r="43">
       <c r="A43" t="inlineStr">
         <is>
-          <t>IA-C-MO</t>
+          <t>IA-C-CR</t>
         </is>
       </c>
       <c r="B43" t="inlineStr">
@@ -77044,11 +77074,11 @@
       </c>
       <c r="C43" t="inlineStr">
         <is>
-          <t>MO_CELL</t>
+          <t>CR_CELL</t>
         </is>
       </c>
       <c r="D43" t="n">
-        <v>0.013807</v>
+        <v>0.101911</v>
       </c>
       <c r="E43" t="inlineStr">
         <is>
@@ -77064,7 +77094,7 @@
     <row r="44">
       <c r="A44" t="inlineStr">
         <is>
-          <t>IA-C-TI</t>
+          <t>IA-C-MO</t>
         </is>
       </c>
       <c r="B44" t="inlineStr">
@@ -77074,11 +77104,11 @@
       </c>
       <c r="C44" t="inlineStr">
         <is>
-          <t>TI_CELL</t>
+          <t>MO_CELL</t>
         </is>
       </c>
       <c r="D44" t="n">
-        <v>0.295205</v>
+        <v>0.013807</v>
       </c>
       <c r="E44" t="inlineStr">
         <is>
@@ -77094,21 +77124,21 @@
     <row r="45">
       <c r="A45" t="inlineStr">
         <is>
-          <t>IA-C11-SHIP</t>
+          <t>IA-C-TI</t>
         </is>
       </c>
       <c r="B45" t="inlineStr">
         <is>
-          <t>PROD_C11_C18</t>
+          <t>OIL_PYRO</t>
         </is>
       </c>
       <c r="C45" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>TI_CELL</t>
         </is>
       </c>
       <c r="D45" t="n">
-        <v>1.511662</v>
+        <v>0.295205</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -77124,12 +77154,12 @@
     <row r="46">
       <c r="A46" t="inlineStr">
         <is>
-          <t>IA-C19-SHIP</t>
+          <t>IA-C11-SHIP</t>
         </is>
       </c>
       <c r="B46" t="inlineStr">
         <is>
-          <t>PROD_C19_C28</t>
+          <t>PROD_C11_C18</t>
         </is>
       </c>
       <c r="C46" t="inlineStr">
@@ -77138,7 +77168,7 @@
         </is>
       </c>
       <c r="D46" t="n">
-        <v>2.218146</v>
+        <v>1.511662</v>
       </c>
       <c r="E46" t="inlineStr">
         <is>
@@ -77154,21 +77184,21 @@
     <row r="47">
       <c r="A47" t="inlineStr">
         <is>
-          <t>IA-C5-POLY</t>
+          <t>IA-C19-SHIP</t>
         </is>
       </c>
       <c r="B47" t="inlineStr">
         <is>
-          <t>PROD_C5_C10</t>
+          <t>PROD_C19_C28</t>
         </is>
       </c>
       <c r="C47" t="inlineStr">
         <is>
-          <t>POLY_OLEFIN</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D47" t="n">
-        <v>0.294127</v>
+        <v>2.018146</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -77184,7 +77214,7 @@
     <row r="48">
       <c r="A48" t="inlineStr">
         <is>
-          <t>IA-C5-SHIP</t>
+          <t>IA-C5-POLY</t>
         </is>
       </c>
       <c r="B48" t="inlineStr">
@@ -77194,11 +77224,11 @@
       </c>
       <c r="C48" t="inlineStr">
         <is>
-          <t>NORTH_DOCK</t>
+          <t>POLY_OLEFIN</t>
         </is>
       </c>
       <c r="D48" t="n">
-        <v>7.130646</v>
+        <v>0.294127</v>
       </c>
       <c r="E48" t="inlineStr">
         <is>
@@ -77214,21 +77244,21 @@
     <row r="49">
       <c r="A49" t="inlineStr">
         <is>
-          <t>IA-CHAR</t>
+          <t>IA-C5-SHIP</t>
         </is>
       </c>
       <c r="B49" t="inlineStr">
         <is>
-          <t>OIL_PYRO</t>
+          <t>PROD_C5_C10</t>
         </is>
       </c>
       <c r="C49" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>NORTH_DOCK</t>
         </is>
       </c>
       <c r="D49" t="n">
-        <v>4.835643</v>
+        <v>7.130646</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -77244,21 +77274,21 @@
     <row r="50">
       <c r="A50" t="inlineStr">
         <is>
-          <t>IA-FEED-01</t>
+          <t>IA-CHAR</t>
         </is>
       </c>
       <c r="B50" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>OIL_PYRO</t>
         </is>
       </c>
       <c r="C50" t="inlineStr">
         <is>
-          <t>LEACH_CSTR_1</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="D50" t="n">
-        <v>102.680001</v>
+        <v>4.835643</v>
       </c>
       <c r="E50" t="inlineStr">
         <is>
@@ -77274,7 +77304,7 @@
     <row r="51">
       <c r="A51" t="inlineStr">
         <is>
-          <t>IA-HOP-01</t>
+          <t>IA-FEED-01</t>
         </is>
       </c>
       <c r="B51" t="inlineStr">
@@ -77288,7 +77318,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>530.73594</v>
+        <v>102.680001</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -77304,21 +77334,21 @@
     <row r="52">
       <c r="A52" t="inlineStr">
         <is>
-          <t>IA-LEACH-HOP</t>
+          <t>IA-HOP-01</t>
         </is>
       </c>
       <c r="B52" t="inlineStr">
         <is>
+          <t>HOPPER</t>
+        </is>
+      </c>
+      <c r="C52" t="inlineStr">
+        <is>
           <t>LEACH_CSTR_1</t>
         </is>
       </c>
-      <c r="C52" t="inlineStr">
-        <is>
-          <t>HOPPER</t>
-        </is>
-      </c>
       <c r="D52" t="n">
-        <v>35.355</v>
+        <v>530.73594</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -77334,21 +77364,21 @@
     <row r="53">
       <c r="A53" t="inlineStr">
         <is>
-          <t>IA-LITHO-OUT</t>
+          <t>IA-LEACH-HOP</t>
         </is>
       </c>
       <c r="B53" t="inlineStr">
         <is>
-          <t>LITHO_DEV</t>
+          <t>LEACH_CSTR_1</t>
         </is>
       </c>
       <c r="C53" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.987499</v>
+        <v>35.355</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -77364,21 +77394,21 @@
     <row r="54">
       <c r="A54" t="inlineStr">
         <is>
-          <t>IA-OIL-01</t>
+          <t>IA-LITHO-OUT</t>
         </is>
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>OIL_DRYER</t>
+          <t>LITHO_DEV</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
         <is>
-          <t>OIL_PYRO</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D54" t="n">
-        <v>33</v>
+        <v>0.987499</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -77394,21 +77424,21 @@
     <row r="55">
       <c r="A55" t="inlineStr">
         <is>
-          <t>IA-OIL-02</t>
+          <t>IA-OIL-01</t>
         </is>
       </c>
       <c r="B55" t="inlineStr">
         <is>
+          <t>OIL_DRYER</t>
+        </is>
+      </c>
+      <c r="C55" t="inlineStr">
+        <is>
           <t>OIL_PYRO</t>
         </is>
       </c>
-      <c r="C55" t="inlineStr">
-        <is>
-          <t>OIL_FRAC</t>
-        </is>
-      </c>
       <c r="D55" t="n">
-        <v>33.373266</v>
+        <v>33</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -77424,21 +77454,21 @@
     <row r="56">
       <c r="A56" t="inlineStr">
         <is>
-          <t>IA-OIL-03</t>
+          <t>IA-OIL-02</t>
         </is>
       </c>
       <c r="B56" t="inlineStr">
         <is>
+          <t>OIL_PYRO</t>
+        </is>
+      </c>
+      <c r="C56" t="inlineStr">
+        <is>
           <t>OIL_FRAC</t>
         </is>
       </c>
-      <c r="C56" t="inlineStr">
-        <is>
-          <t>NCG_HEADER</t>
-        </is>
-      </c>
       <c r="D56" t="n">
-        <v>5</v>
+        <v>33.373266</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -77454,21 +77484,21 @@
     <row r="57">
       <c r="A57" t="inlineStr">
         <is>
-          <t>IA-PLAST-01</t>
+          <t>IA-OIL-03</t>
         </is>
       </c>
       <c r="B57" t="inlineStr">
         <is>
-          <t>FLOAT_SINK</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="C57" t="inlineStr">
         <is>
-          <t>OIL_DRYER</t>
+          <t>NCG_HEADER</t>
         </is>
       </c>
       <c r="D57" t="n">
-        <v>33</v>
+        <v>5</v>
       </c>
       <c r="E57" t="inlineStr">
         <is>
@@ -77484,21 +77514,21 @@
     <row r="58">
       <c r="A58" t="inlineStr">
         <is>
-          <t>IA-WEAR</t>
+          <t>IA-PLAST-01</t>
         </is>
       </c>
       <c r="B58" t="inlineStr">
         <is>
-          <t>HABITATION</t>
+          <t>FLOAT_SINK</t>
         </is>
       </c>
       <c r="C58" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>OIL_DRYER</t>
         </is>
       </c>
       <c r="D58" t="n">
-        <v>596.863842</v>
+        <v>33</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -77514,73 +77544,73 @@
     <row r="59">
       <c r="A59" t="inlineStr">
         <is>
-          <t>LI_TO_GREASE</t>
+          <t>IA-WEAR</t>
         </is>
       </c>
       <c r="B59" t="inlineStr">
         <is>
-          <t>LI_RECOVER</t>
+          <t>HABITATION</t>
         </is>
       </c>
       <c r="C59" t="inlineStr">
         <is>
-          <t>GREASE_LI</t>
+          <t>HOPPER</t>
+        </is>
+      </c>
+      <c r="D59" t="n">
+        <v>596.863842</v>
+      </c>
+      <c r="E59" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" t="inlineStr">
         <is>
-          <t>NCG_TO_AB</t>
+          <t>LI_TO_GREASE</t>
         </is>
       </c>
       <c r="B60" t="inlineStr">
         <is>
-          <t>NCG_HEADER</t>
+          <t>LI_RECOVER</t>
         </is>
       </c>
       <c r="C60" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
-        </is>
-      </c>
-      <c r="D60" t="n">
-        <v>5</v>
-      </c>
-      <c r="E60" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREASE_LI</t>
         </is>
       </c>
       <c r="F60" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" t="inlineStr">
         <is>
-          <t>OIL_TO_OLEFIN</t>
+          <t>NCG_TO_AB</t>
         </is>
       </c>
       <c r="B61" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>NCG_HEADER</t>
         </is>
       </c>
       <c r="C61" t="inlineStr">
         <is>
-          <t>POLY_OLEFIN</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -77596,73 +77626,73 @@
     <row r="62">
       <c r="A62" t="inlineStr">
         <is>
-          <t>PCA_TO_GREASE</t>
+          <t>OIL_TO_OLEFIN</t>
         </is>
       </c>
       <c r="B62" t="inlineStr">
         <is>
-          <t>P_CA</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="C62" t="inlineStr">
         <is>
-          <t>GREASE_CA</t>
+          <t>POLY_OLEFIN</t>
+        </is>
+      </c>
+      <c r="D62" t="n">
+        <v>0</v>
+      </c>
+      <c r="E62" t="inlineStr">
+        <is>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F62" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" t="inlineStr">
         <is>
-          <t>S11</t>
+          <t>PCA_TO_GREASE</t>
         </is>
       </c>
       <c r="B63" t="inlineStr">
         <is>
-          <t>GROW_BED</t>
+          <t>P_CA</t>
         </is>
       </c>
       <c r="C63" t="inlineStr">
         <is>
-          <t>AFTERBURNER</t>
-        </is>
-      </c>
-      <c r="D63" t="n">
-        <v>0.8</v>
-      </c>
-      <c r="E63" t="inlineStr">
-        <is>
-          <t>kg/d</t>
+          <t>GREASE_CA</t>
         </is>
       </c>
       <c r="F63" t="inlineStr">
         <is>
-          <t>study</t>
+          <t>null</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" t="inlineStr">
         <is>
-          <t>S18</t>
+          <t>S11</t>
         </is>
       </c>
       <c r="B64" t="inlineStr">
         <is>
+          <t>GROW_BED</t>
+        </is>
+      </c>
+      <c r="C64" t="inlineStr">
+        <is>
           <t>AFTERBURNER</t>
         </is>
       </c>
-      <c r="C64" t="inlineStr">
-        <is>
-          <t>CRYO_CO2</t>
-        </is>
-      </c>
       <c r="D64" t="n">
-        <v>0</v>
+        <v>0.8</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -77678,21 +77708,21 @@
     <row r="65">
       <c r="A65" t="inlineStr">
         <is>
-          <t>S38</t>
+          <t>S18</t>
         </is>
       </c>
       <c r="B65" t="inlineStr">
         <is>
-          <t>WET_BENCH</t>
+          <t>AFTERBURNER</t>
         </is>
       </c>
       <c r="C65" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>CRYO_CO2</t>
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.006</v>
+        <v>0</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -77708,12 +77738,12 @@
     <row r="66">
       <c r="A66" t="inlineStr">
         <is>
-          <t>S39B</t>
+          <t>S38</t>
         </is>
       </c>
       <c r="B66" t="inlineStr">
         <is>
-          <t>WAFER_FAB</t>
+          <t>WET_BENCH</t>
         </is>
       </c>
       <c r="C66" t="inlineStr">
@@ -77722,7 +77752,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>0.006</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -77738,21 +77768,21 @@
     <row r="67">
       <c r="A67" t="inlineStr">
         <is>
-          <t>S61</t>
+          <t>S39B</t>
         </is>
       </c>
       <c r="B67" t="inlineStr">
         <is>
-          <t>MFG_SHOP</t>
+          <t>WAFER_FAB</t>
         </is>
       </c>
       <c r="C67" t="inlineStr">
         <is>
-          <t>HOPPER</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D67" t="n">
-        <v>1.197099</v>
+        <v>0</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -77768,21 +77798,21 @@
     <row r="68">
       <c r="A68" t="inlineStr">
         <is>
-          <t>S72B</t>
+          <t>S61</t>
         </is>
       </c>
       <c r="B68" t="inlineStr">
         <is>
-          <t>MET_SCRUB</t>
+          <t>MFG_SHOP</t>
         </is>
       </c>
       <c r="C68" t="inlineStr">
         <is>
-          <t>OIL_FRAC</t>
+          <t>HOPPER</t>
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.0158</v>
+        <v>1.197099</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -77798,25 +77828,25 @@
     <row r="69">
       <c r="A69" t="inlineStr">
         <is>
-          <t>SF-OIL_PYRO</t>
+          <t>S72B</t>
         </is>
       </c>
       <c r="B69" t="inlineStr">
         <is>
-          <t>SOL_ARK_60K</t>
+          <t>MET_SCRUB</t>
         </is>
       </c>
       <c r="C69" t="inlineStr">
         <is>
-          <t>OIL_PYRO</t>
+          <t>OIL_FRAC</t>
         </is>
       </c>
       <c r="D69" t="n">
-        <v>1.664</v>
+        <v>0.0158</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>kW</t>
+          <t>kg/d</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
@@ -77828,29 +77858,37 @@
     <row r="70">
       <c r="A70" t="inlineStr">
         <is>
-          <t>WAX_TO_GREASE_CA</t>
+          <t>SF-OIL_PYRO</t>
         </is>
       </c>
       <c r="B70" t="inlineStr">
         <is>
-          <t>PROD_C19_C28</t>
+          <t>SOL_ARK_60K</t>
         </is>
       </c>
       <c r="C70" t="inlineStr">
         <is>
-          <t>GREASE_CA</t>
+          <t>OIL_PYRO</t>
+        </is>
+      </c>
+      <c r="D70" t="n">
+        <v>1.664</v>
+      </c>
+      <c r="E70" t="inlineStr">
+        <is>
+          <t>kW</t>
         </is>
       </c>
       <c r="F70" t="inlineStr">
         <is>
-          <t>null</t>
+          <t>study</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" t="inlineStr">
         <is>
-          <t>WAX_TO_GREASE_LI</t>
+          <t>WAX_TO_GREASE_CA</t>
         </is>
       </c>
       <c r="B71" t="inlineStr">
@@ -77860,7 +77898,7 @@
       </c>
       <c r="C71" t="inlineStr">
         <is>
-          <t>GREASE_LI</t>
+          <t>GREASE_CA</t>
         </is>
       </c>
       <c r="F71" t="inlineStr">
@@ -77872,28 +77910,50 @@
     <row r="72">
       <c r="A72" t="inlineStr">
         <is>
+          <t>WAX_TO_GREASE_LI</t>
+        </is>
+      </c>
+      <c r="B72" t="inlineStr">
+        <is>
+          <t>PROD_C19_C28</t>
+        </is>
+      </c>
+      <c r="C72" t="inlineStr">
+        <is>
+          <t>GREASE_LI</t>
+        </is>
+      </c>
+      <c r="F72" t="inlineStr">
+        <is>
+          <t>null</t>
+        </is>
+      </c>
+    </row>
+    <row r="73">
+      <c r="A73" t="inlineStr">
+        <is>
           <t>WAX_TO_OIL</t>
         </is>
       </c>
-      <c r="B72" t="inlineStr">
+      <c r="B73" t="inlineStr">
         <is>
           <t>SHELL_BURNOUT</t>
         </is>
       </c>
-      <c r="C72" t="inlineStr">
+      <c r="C73" t="inlineStr">
         <is>
           <t>OIL_FRAC</t>
         </is>
       </c>
-      <c r="D72" t="n">
+      <c r="D73" t="n">
         <v>0</v>
       </c>
-      <c r="E72" t="inlineStr">
+      <c r="E73" t="inlineStr">
         <is>
           <t>kg/d</t>
         </is>
       </c>
-      <c r="F72" t="inlineStr">
+      <c r="F73" t="inlineStr">
         <is>
           <t>study</t>
         </is>

</xml_diff>

<commit_message>
Decide Q-035 and Q-036 on the merits (t62u): top up the sodium hydroxide on the chlor-alkali cells with halite ore, less than half the load of causticising and no kilns, with CAUSTICIZE selectable; keep the cell hydrogen on the H2 header to the hydrogen store (A-M-426, batch 38)
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 15edcc2fe9038602a3ccc1a0fe0ae19e5060ac0b00d70f0f662c13bc5d2ea1af</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 94817999e5d0abe4eb1e6777d0c24fde5d18cd0e44526906cbe22f1fb03b04a6</t>
         </is>
       </c>
     </row>
@@ -2231,7 +2231,7 @@
         </is>
       </c>
       <c r="D45" t="n">
-        <v>2.075063</v>
+        <v>2.086136</v>
       </c>
       <c r="E45" t="inlineStr">
         <is>
@@ -2441,7 +2441,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.09965499999999999</v>
+        <v>0.110728</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -2651,7 +2651,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>22.093431</v>
+        <v>22.005555</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -2891,7 +2891,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>2.075063</v>
+        <v>2.086136</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -3071,7 +3071,7 @@
         </is>
       </c>
       <c r="D73" t="n">
-        <v>32.377012</v>
+        <v>32.289136</v>
       </c>
       <c r="E73" t="inlineStr">
         <is>
@@ -14528,7 +14528,7 @@
         </is>
       </c>
       <c r="B12" s="8" t="n">
-        <v>21.2163</v>
+        <v>21.1909</v>
       </c>
       <c r="C12" t="inlineStr">
         <is>
@@ -15061,7 +15061,7 @@
         </is>
       </c>
       <c r="D33" t="n">
-        <v>9.25802</v>
+        <v>9.246947</v>
       </c>
       <c r="E33" t="inlineStr">
         <is>
@@ -15091,7 +15091,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>82.729777</v>
+        <v>82.63082799999999</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -15121,7 +15121,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>73.471757</v>
+        <v>73.383881</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -15481,7 +15481,7 @@
         </is>
       </c>
       <c r="D47" t="n">
-        <v>22.093431</v>
+        <v>22.005555</v>
       </c>
       <c r="E47" t="inlineStr">
         <is>
@@ -15541,7 +15541,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>22.093431</v>
+        <v>22.005555</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -15871,7 +15871,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>2.075063</v>
+        <v>2.086136</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -16081,7 +16081,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>32.377012</v>
+        <v>32.289136</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -16351,7 +16351,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>21.2163</v>
+        <v>21.1909</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -16381,7 +16381,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>6.0177</v>
+        <v>6.0105</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -16907,7 +16907,7 @@
         </is>
       </c>
       <c r="B18" s="8" t="n">
-        <v>0.2353</v>
+        <v>0.2352</v>
       </c>
       <c r="C18" t="inlineStr">
         <is>
@@ -17424,7 +17424,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>82.729777</v>
+        <v>82.63082799999999</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -17779,7 +17779,7 @@
         </is>
       </c>
       <c r="D51" t="n">
-        <v>167.10916</v>
+        <v>167.010211</v>
       </c>
       <c r="E51" t="inlineStr">
         <is>
@@ -17839,7 +17839,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>14.237076</v>
+        <v>11.3154</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -17869,7 +17869,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.475115</v>
+        <v>0</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -18041,7 +18041,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>164.283721</v>
+        <v>164.184772</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -18221,7 +18221,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>174.28376</v>
+        <v>174.184811</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -18551,7 +18551,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>307.62916</v>
+        <v>307.530211</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -18930,7 +18930,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>82.50230000000001</v>
+        <v>82.1326</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -19056,7 +19056,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>352.9258</v>
+        <v>351.8354</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -19157,7 +19157,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>219.1023</v>
+        <v>218.0126</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -19842,7 +19842,7 @@
         </is>
       </c>
       <c r="D36" t="n">
-        <v>352.9258</v>
+        <v>351.8354</v>
       </c>
       <c r="E36" t="inlineStr">
         <is>
@@ -20524,7 +20524,7 @@
         </is>
       </c>
       <c r="D59" t="n">
-        <v>920.7045000000001</v>
+        <v>916.12544</v>
       </c>
       <c r="E59" t="inlineStr">
         <is>
@@ -20554,7 +20554,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>920.7045000000001</v>
+        <v>916.12544</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -21154,7 +21154,7 @@
         </is>
       </c>
       <c r="D80" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="E80" t="inlineStr">
         <is>
@@ -21214,7 +21214,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>82.50230000000001</v>
+        <v>82.1326</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -21364,7 +21364,7 @@
         </is>
       </c>
       <c r="D87" t="n">
-        <v>0.7069</v>
+        <v>0.7091</v>
       </c>
       <c r="E87" t="inlineStr">
         <is>
@@ -21454,7 +21454,7 @@
         </is>
       </c>
       <c r="D90" t="n">
-        <v>21.2163</v>
+        <v>21.1909</v>
       </c>
       <c r="E90" t="inlineStr">
         <is>
@@ -21964,7 +21964,7 @@
         </is>
       </c>
       <c r="D107" t="n">
-        <v>1.1929</v>
+        <v>0.5004</v>
       </c>
       <c r="E107" t="inlineStr">
         <is>
@@ -46914,7 +46914,7 @@
       </c>
       <c r="B723" s="4" t="inlineStr">
         <is>
-          <t>CAUSTICIZE</t>
+          <t>CHLOR_ALKALI</t>
         </is>
       </c>
       <c r="C723" t="inlineStr">
@@ -46924,7 +46924,7 @@
       </c>
       <c r="E723" t="inlineStr">
         <is>
-          <t>A-M-422</t>
+          <t>A-M-422, A-M-426</t>
         </is>
       </c>
     </row>
@@ -53400,7 +53400,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>2.262</v>
+        <v>2.2692</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -53550,7 +53550,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>6.0177</v>
+        <v>6.0105</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -54901,7 +54901,7 @@
         </is>
       </c>
       <c r="B3" s="8" t="n">
-        <v>0.7069</v>
+        <v>0.7091</v>
       </c>
       <c r="C3" t="inlineStr">
         <is>
@@ -55158,7 +55158,7 @@
         </is>
       </c>
       <c r="D14" t="n">
-        <v>2.262</v>
+        <v>2.2692</v>
       </c>
       <c r="E14" t="inlineStr">
         <is>
@@ -55210,7 +55210,7 @@
         </is>
       </c>
       <c r="D16" t="n">
-        <v>0.7069</v>
+        <v>0.7091</v>
       </c>
       <c r="E16" t="inlineStr">
         <is>
@@ -55330,7 +55330,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -55977,7 +55977,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>53.367231</v>
+        <v>56.288882</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -56037,7 +56037,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0</v>
+        <v>0.67578</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -56097,7 +56097,7 @@
         </is>
       </c>
       <c r="D28" t="n">
-        <v>0.259355</v>
+        <v>0.281728</v>
       </c>
       <c r="E28" t="inlineStr">
         <is>
@@ -56367,7 +56367,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>3.505031</v>
+        <v>3.894478</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -56427,7 +56427,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.126417</v>
+        <v>0.033789</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -56457,7 +56457,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>22.093431</v>
+        <v>22.005555</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -56847,7 +56847,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.919575</v>
+        <v>0</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -57022,7 +57022,7 @@
         <v>14</v>
       </c>
       <c r="H2" s="5" t="n">
-        <v>24.4532</v>
+        <v>24.4278</v>
       </c>
       <c r="I2" t="n">
         <v>4</v>
@@ -57061,7 +57061,7 @@
         <v>14</v>
       </c>
       <c r="H3" s="5" t="n">
-        <v>24.4532</v>
+        <v>24.4278</v>
       </c>
       <c r="I3" t="n">
         <v>4</v>
@@ -57495,7 +57495,7 @@
         <v>6</v>
       </c>
       <c r="H14" s="5" t="n">
-        <v>21.2163</v>
+        <v>21.1909</v>
       </c>
       <c r="I14" t="n">
         <v>1</v>
@@ -57612,7 +57612,7 @@
         <v>1</v>
       </c>
       <c r="H17" s="5" t="n">
-        <v>21.2163</v>
+        <v>21.1909</v>
       </c>
       <c r="I17" t="n">
         <v>1</v>
@@ -57763,7 +57763,7 @@
         <v>26</v>
       </c>
       <c r="H21" s="5" t="n">
-        <v>15.6887</v>
+        <v>14.9912</v>
       </c>
       <c r="I21" t="n">
         <v>7</v>
@@ -58309,7 +58309,7 @@
         <v>16</v>
       </c>
       <c r="H35" s="5" t="n">
-        <v>10.4404</v>
+        <v>9.742900000000001</v>
       </c>
       <c r="I35" t="n">
         <v>6</v>
@@ -58348,7 +58348,7 @@
         <v>6</v>
       </c>
       <c r="H36" s="5" t="n">
-        <v>9.6904</v>
+        <v>8.992900000000001</v>
       </c>
       <c r="I36" t="n">
         <v>5</v>
@@ -58543,7 +58543,7 @@
         <v>1</v>
       </c>
       <c r="H41" s="5" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="I41" t="n">
         <v>1</v>
@@ -58582,7 +58582,7 @@
         <v>1</v>
       </c>
       <c r="H42" s="5" t="n">
-        <v>1.1929</v>
+        <v>0.5004</v>
       </c>
       <c r="I42" t="n">
         <v>1</v>
@@ -59196,7 +59196,7 @@
         <v>10</v>
       </c>
       <c r="H58" s="5" t="n">
-        <v>670.5386</v>
+        <v>667.9888</v>
       </c>
       <c r="I58" t="n">
         <v>6</v>
@@ -59235,7 +59235,7 @@
         <v>4</v>
       </c>
       <c r="H59" s="5" t="n">
-        <v>94.50230000000001</v>
+        <v>94.1326</v>
       </c>
       <c r="I59" t="n">
         <v>2</v>
@@ -59274,7 +59274,7 @@
         <v>1</v>
       </c>
       <c r="H60" s="5" t="n">
-        <v>82.50230000000001</v>
+        <v>82.1326</v>
       </c>
       <c r="I60" t="n">
         <v>1</v>
@@ -59430,7 +59430,7 @@
         <v>3</v>
       </c>
       <c r="H64" s="5" t="n">
-        <v>356.934</v>
+        <v>355.8436</v>
       </c>
       <c r="I64" t="n">
         <v>3</v>
@@ -59547,7 +59547,7 @@
         <v>1</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>352.9258</v>
+        <v>351.8354</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
@@ -59586,7 +59586,7 @@
         <v>3</v>
       </c>
       <c r="H68" s="5" t="n">
-        <v>219.1023</v>
+        <v>218.0126</v>
       </c>
       <c r="I68" t="n">
         <v>1</v>
@@ -59664,7 +59664,7 @@
         <v>1</v>
       </c>
       <c r="H70" s="5" t="n">
-        <v>219.1023</v>
+        <v>218.0126</v>
       </c>
       <c r="I70" t="n">
         <v>1</v>
@@ -62808,7 +62808,7 @@
         <v>4</v>
       </c>
       <c r="H151" s="5" t="n">
-        <v>0.8326</v>
+        <v>0.8348</v>
       </c>
       <c r="I151" t="n">
         <v>2</v>
@@ -62847,7 +62847,7 @@
         <v>4</v>
       </c>
       <c r="H152" s="5" t="n">
-        <v>0.8326</v>
+        <v>0.8348</v>
       </c>
       <c r="I152" t="n">
         <v>2</v>
@@ -62925,7 +62925,7 @@
         <v>1</v>
       </c>
       <c r="H154" s="5" t="n">
-        <v>0.7069</v>
+        <v>0.7091</v>
       </c>
       <c r="I154" t="n">
         <v>1</v>
@@ -66619,7 +66619,7 @@
         <v>18</v>
       </c>
       <c r="H250" s="5" t="n">
-        <v>0.4045</v>
+        <v>0.4044</v>
       </c>
       <c r="I250" t="n">
         <v>4</v>
@@ -66853,7 +66853,7 @@
         <v>14</v>
       </c>
       <c r="H256" s="5" t="n">
-        <v>0.2993</v>
+        <v>0.2992</v>
       </c>
       <c r="I256" t="n">
         <v>3</v>
@@ -67399,7 +67399,7 @@
         <v>1</v>
       </c>
       <c r="H270" s="5" t="n">
-        <v>0.2353</v>
+        <v>0.2352</v>
       </c>
       <c r="I270" t="n">
         <v>1</v>
@@ -67477,7 +67477,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>219.1</v>
+        <v>218.01</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -67491,7 +67491,7 @@
       </c>
       <c r="F2" t="inlineStr">
         <is>
-          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 30x27 bays, ext 82.50 kW).</t>
+          <t>write_graph power() live derivation (A-M-234 replaced_by; A-M-258): converged bounding demand incl. the EXT_HALL extension (roof_close 35x23 bays, ext 82.13 kW).</t>
         </is>
       </c>
     </row>
@@ -67507,7 +67507,7 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>547.76</v>
+        <v>545.03</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -67552,7 +67552,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6076</v>
+        <v>6046</v>
       </c>
     </row>
     <row r="6">
@@ -67582,7 +67582,7 @@
         </is>
       </c>
       <c r="C7" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="8">
@@ -67653,7 +67653,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>352.9258</v>
+        <v>351.8354</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -67678,7 +67678,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>219.1023</v>
+        <v>218.0126</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -67781,7 +67781,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6076</v>
+        <v>6046</v>
       </c>
     </row>
     <row r="19">
@@ -67796,7 +67796,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3038</v>
+        <v>3023</v>
       </c>
     </row>
     <row r="20">
@@ -67811,7 +67811,7 @@
         </is>
       </c>
       <c r="C20" t="n">
-        <v>26712</v>
+        <v>26574</v>
       </c>
     </row>
     <row r="21">
@@ -67826,7 +67826,7 @@
         </is>
       </c>
       <c r="C21" t="n">
-        <v>1519</v>
+        <v>1512</v>
       </c>
     </row>
     <row r="22">
@@ -67856,7 +67856,7 @@
         </is>
       </c>
       <c r="C23" t="n">
-        <v>996</v>
+        <v>991</v>
       </c>
     </row>
     <row r="24">
@@ -67871,7 +67871,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3068</v>
+        <v>3053</v>
       </c>
     </row>
     <row r="25">
@@ -67886,7 +67886,7 @@
         </is>
       </c>
       <c r="C25" t="n">
-        <v>996</v>
+        <v>991</v>
       </c>
     </row>
     <row r="26">
@@ -67901,7 +67901,7 @@
         </is>
       </c>
       <c r="C26" t="n">
-        <v>220</v>
+        <v>219</v>
       </c>
     </row>
     <row r="27">
@@ -67916,7 +67916,7 @@
         </is>
       </c>
       <c r="C27" t="n">
-        <v>2580</v>
+        <v>2520</v>
       </c>
     </row>
     <row r="28">
@@ -67931,7 +67931,7 @@
         </is>
       </c>
       <c r="C28" t="n">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29">
@@ -67961,7 +67961,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2360.9</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="31">
@@ -69404,7 +69404,7 @@
         </is>
       </c>
       <c r="D54" s="8" t="n">
-        <v>2.262</v>
+        <v>2.2692</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -69554,7 +69554,7 @@
         </is>
       </c>
       <c r="D60" s="8" t="n">
-        <v>6.0177</v>
+        <v>6.0105</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -70524,7 +70524,7 @@
         </is>
       </c>
       <c r="B8" s="8" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="C8" t="inlineStr">
         <is>
@@ -70938,7 +70938,7 @@
         </is>
       </c>
       <c r="B23" s="8" t="n">
-        <v>1.1929</v>
+        <v>0.5004</v>
       </c>
       <c r="C23" t="inlineStr">
         <is>
@@ -71775,7 +71775,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>487.774</v>
+        <v>490.7946</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -72405,7 +72405,7 @@
         </is>
       </c>
       <c r="D76" t="n">
-        <v>814.213</v>
+        <v>811.1924</v>
       </c>
       <c r="E76" t="inlineStr">
         <is>
@@ -73755,7 +73755,7 @@
         </is>
       </c>
       <c r="D121" t="n">
-        <v>53.367231</v>
+        <v>56.288882</v>
       </c>
       <c r="E121" t="inlineStr">
         <is>
@@ -73785,7 +73785,7 @@
         </is>
       </c>
       <c r="D122" t="n">
-        <v>0</v>
+        <v>0.67578</v>
       </c>
       <c r="E122" t="inlineStr">
         <is>
@@ -74175,7 +74175,7 @@
         </is>
       </c>
       <c r="D135" t="n">
-        <v>167.10916</v>
+        <v>167.010211</v>
       </c>
       <c r="E135" t="inlineStr">
         <is>
@@ -74205,7 +74205,7 @@
         </is>
       </c>
       <c r="D136" t="n">
-        <v>0.022373</v>
+        <v>0</v>
       </c>
       <c r="E136" t="inlineStr">
         <is>
@@ -74325,7 +74325,7 @@
         </is>
       </c>
       <c r="D140" t="n">
-        <v>3.505031</v>
+        <v>3.894478</v>
       </c>
       <c r="E140" t="inlineStr">
         <is>
@@ -74355,7 +74355,7 @@
         </is>
       </c>
       <c r="D141" t="n">
-        <v>0.09965499999999999</v>
+        <v>0.110728</v>
       </c>
       <c r="E141" t="inlineStr">
         <is>
@@ -74385,7 +74385,7 @@
         </is>
       </c>
       <c r="D142" t="n">
-        <v>14.237076</v>
+        <v>11.3154</v>
       </c>
       <c r="E142" t="inlineStr">
         <is>
@@ -74415,7 +74415,7 @@
         </is>
       </c>
       <c r="D143" t="n">
-        <v>16.750724</v>
+        <v>13.730102</v>
       </c>
       <c r="E143" t="inlineStr">
         <is>
@@ -74475,7 +74475,7 @@
         </is>
       </c>
       <c r="D145" t="n">
-        <v>0.126417</v>
+        <v>0.033789</v>
       </c>
       <c r="E145" t="inlineStr">
         <is>
@@ -74505,7 +74505,7 @@
         </is>
       </c>
       <c r="D146" t="n">
-        <v>0.475115</v>
+        <v>0</v>
       </c>
       <c r="E146" t="inlineStr">
         <is>
@@ -74917,7 +74917,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.919575</v>
+        <v>0</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -75823,7 +75823,7 @@
         </is>
       </c>
       <c r="D191" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="E191" t="inlineStr">
         <is>
@@ -75883,7 +75883,7 @@
         </is>
       </c>
       <c r="D193" t="n">
-        <v>1.1929</v>
+        <v>0.5004</v>
       </c>
       <c r="E193" t="inlineStr">
         <is>
@@ -75973,7 +75973,7 @@
         </is>
       </c>
       <c r="D196" t="n">
-        <v>1.349</v>
+        <v>1.344</v>
       </c>
       <c r="E196" t="inlineStr">
         <is>
@@ -80379,7 +80379,7 @@
         </is>
       </c>
       <c r="D37" t="n">
-        <v>0.259355</v>
+        <v>0.281728</v>
       </c>
       <c r="E37" t="inlineStr">
         <is>
@@ -80409,7 +80409,7 @@
         </is>
       </c>
       <c r="D38" t="n">
-        <v>0.022373</v>
+        <v>0</v>
       </c>
       <c r="E38" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
Batch 42e: hold X-RTE transfer-function rates in the reconciliation; take the resist benzene feed off IA-C5-SHIP
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 53cde3c475e10dd650ae9708b5611ccf6c88c1ca606279fb7124e80398e8f076</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 08f7fff441d4abd9edd422b14df9ab48a03c1bcc2dcbd17a7db848fd04e9fb56</t>
         </is>
       </c>
     </row>
@@ -4170,7 +4170,7 @@
         </is>
       </c>
       <c r="D32" t="n">
-        <v>0.938489</v>
+        <v>1.499799</v>
       </c>
       <c r="E32" t="inlineStr">
         <is>
@@ -4230,7 +4230,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0</v>
+        <v>0.21952</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -4260,7 +4260,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>66.527242</v>
+        <v>66.500212</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -4380,7 +4380,7 @@
         </is>
       </c>
       <c r="D39" t="n">
-        <v>0.557915</v>
+        <v>0.33952</v>
       </c>
       <c r="E39" t="inlineStr">
         <is>
@@ -4410,7 +4410,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>0.557915</v>
+        <v>0.33952</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -4440,7 +4440,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0.557915</v>
+        <v>0.33952</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -4770,7 +4770,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.257613</v>
+        <v>0.09</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -4830,7 +4830,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>0.319016</v>
+        <v>0.092558</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -4860,7 +4860,7 @@
         </is>
       </c>
       <c r="D55" t="n">
-        <v>0.007976</v>
+        <v>0.011349</v>
       </c>
       <c r="E55" t="inlineStr">
         <is>
@@ -4890,7 +4890,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0</v>
+        <v>1.005233</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -4950,7 +4950,7 @@
         </is>
       </c>
       <c r="D58" t="n">
-        <v>0.000732</v>
+        <v>0.000721</v>
       </c>
       <c r="E58" t="inlineStr">
         <is>
@@ -5010,7 +5010,7 @@
         </is>
       </c>
       <c r="D60" t="n">
-        <v>0.000915</v>
+        <v>0.000938</v>
       </c>
       <c r="E60" t="inlineStr">
         <is>
@@ -5040,7 +5040,7 @@
         </is>
       </c>
       <c r="D61" t="n">
-        <v>0.00666</v>
+        <v>0.005938</v>
       </c>
       <c r="E61" t="inlineStr">
         <is>
@@ -5130,7 +5130,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>0.947336</v>
+        <v>1.350229</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -5160,7 +5160,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -5190,7 +5190,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0</v>
+        <v>0.084138</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -5250,7 +5250,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0.543843</v>
+        <v>0.14095</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -5280,7 +5280,7 @@
         </is>
       </c>
       <c r="D69" t="n">
-        <v>0.12609</v>
+        <v>0.126101</v>
       </c>
       <c r="E69" t="inlineStr">
         <is>
@@ -5370,7 +5370,7 @@
         </is>
       </c>
       <c r="D72" t="n">
-        <v>0.143533</v>
+        <v>0.144254</v>
       </c>
       <c r="E72" t="inlineStr">
         <is>
@@ -5430,7 +5430,7 @@
         </is>
       </c>
       <c r="D74" t="n">
-        <v>0.467586</v>
+        <v>0.519493</v>
       </c>
       <c r="E74" t="inlineStr">
         <is>
@@ -5520,7 +5520,7 @@
         </is>
       </c>
       <c r="D77" t="n">
-        <v>0.016578</v>
+        <v>0.149902</v>
       </c>
       <c r="E77" t="inlineStr">
         <is>
@@ -5640,7 +5640,7 @@
         </is>
       </c>
       <c r="D81" t="n">
-        <v>0.023634</v>
+        <v>0.12</v>
       </c>
       <c r="E81" t="inlineStr">
         <is>
@@ -11166,7 +11166,7 @@
         </is>
       </c>
       <c r="D82" t="n">
-        <v>0.000732</v>
+        <v>0.000721</v>
       </c>
       <c r="E82" t="inlineStr">
         <is>
@@ -11346,7 +11346,7 @@
         </is>
       </c>
       <c r="D88" t="n">
-        <v>0.12609</v>
+        <v>0.126101</v>
       </c>
       <c r="E88" t="inlineStr">
         <is>
@@ -18836,7 +18836,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.938489</v>
+        <v>1.499799</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -19573,7 +19573,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.319016</v>
+        <v>0.092558</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>
@@ -19603,7 +19603,7 @@
         </is>
       </c>
       <c r="D68" t="n">
-        <v>0</v>
+        <v>0.084138</v>
       </c>
       <c r="E68" t="inlineStr">
         <is>
@@ -57168,7 +57168,7 @@
         </is>
       </c>
       <c r="D23" t="n">
-        <v>0.00666</v>
+        <v>0.005938</v>
       </c>
       <c r="E23" t="inlineStr">
         <is>
@@ -57198,7 +57198,7 @@
         </is>
       </c>
       <c r="D24" t="n">
-        <v>0.143533</v>
+        <v>0.144254</v>
       </c>
       <c r="E24" t="inlineStr">
         <is>
@@ -58749,7 +58749,7 @@
         </is>
       </c>
       <c r="D15" t="n">
-        <v>7.635055</v>
+        <v>6.629822</v>
       </c>
       <c r="E15" t="inlineStr">
         <is>
@@ -59889,7 +59889,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.016578</v>
+        <v>0.149902</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -74371,7 +74371,7 @@
         </is>
       </c>
       <c r="D34" t="n">
-        <v>0.291339</v>
+        <v>0.283567</v>
       </c>
       <c r="E34" t="inlineStr">
         <is>
@@ -74401,7 +74401,7 @@
         </is>
       </c>
       <c r="D35" t="n">
-        <v>0.348057</v>
+        <v>0.332195</v>
       </c>
       <c r="E35" t="inlineStr">
         <is>
@@ -75255,7 +75255,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>27.487256</v>
+        <v>27.510913</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -76935,7 +76935,7 @@
         </is>
       </c>
       <c r="D120" t="n">
-        <v>66.527242</v>
+        <v>66.500212</v>
       </c>
       <c r="E120" t="inlineStr">
         <is>
@@ -78127,7 +78127,7 @@
         </is>
       </c>
       <c r="D160" t="n">
-        <v>0.007976</v>
+        <v>0.011349</v>
       </c>
       <c r="E160" t="inlineStr">
         <is>
@@ -78157,7 +78157,7 @@
         </is>
       </c>
       <c r="D161" t="n">
-        <v>0.000915</v>
+        <v>0.000938</v>
       </c>
       <c r="E161" t="inlineStr">
         <is>
@@ -80978,7 +80978,7 @@
         </is>
       </c>
       <c r="D49" t="n">
-        <v>7.635055</v>
+        <v>6.629822</v>
       </c>
       <c r="E49" t="inlineStr">
         <is>
@@ -81398,7 +81398,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>0</v>
+        <v>1.005233</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -81458,7 +81458,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.947336</v>
+        <v>1.350229</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -81488,7 +81488,7 @@
         </is>
       </c>
       <c r="D66" t="n">
-        <v>0.543843</v>
+        <v>0.14095</v>
       </c>
       <c r="E66" t="inlineStr">
         <is>
@@ -83709,7 +83709,7 @@
         </is>
       </c>
       <c r="D19" t="n">
-        <v>0.291339</v>
+        <v>0.283567</v>
       </c>
       <c r="E19" t="inlineStr">
         <is>
@@ -83739,7 +83739,7 @@
         </is>
       </c>
       <c r="D20" t="n">
-        <v>0.348057</v>
+        <v>0.332195</v>
       </c>
       <c r="E20" t="inlineStr">
         <is>
@@ -83889,7 +83889,7 @@
         </is>
       </c>
       <c r="D25" t="n">
-        <v>0.079842</v>
+        <v>0.080016</v>
       </c>
       <c r="E25" t="inlineStr">
         <is>
@@ -83919,7 +83919,7 @@
         </is>
       </c>
       <c r="D26" t="n">
-        <v>0.093912</v>
+        <v>0.093738</v>
       </c>
       <c r="E26" t="inlineStr">
         <is>
@@ -84369,7 +84369,7 @@
         </is>
       </c>
       <c r="D41" t="n">
-        <v>0</v>
+        <v>0.12</v>
       </c>
       <c r="E41" t="inlineStr">
         <is>
@@ -84699,7 +84699,7 @@
         </is>
       </c>
       <c r="D52" t="n">
-        <v>0.113634</v>
+        <v>0.09</v>
       </c>
       <c r="E52" t="inlineStr">
         <is>
@@ -84729,7 +84729,7 @@
         </is>
       </c>
       <c r="D53" t="n">
-        <v>0.023634</v>
+        <v>0.12</v>
       </c>
       <c r="E53" t="inlineStr">
         <is>
@@ -84819,7 +84819,7 @@
         </is>
       </c>
       <c r="D56" t="n">
-        <v>0.113634</v>
+        <v>0.09</v>
       </c>
       <c r="E56" t="inlineStr">
         <is>
@@ -85089,7 +85089,7 @@
         </is>
       </c>
       <c r="D65" t="n">
-        <v>0.107598</v>
+        <v>0.1</v>
       </c>
       <c r="E65" t="inlineStr">
         <is>
@@ -85149,7 +85149,7 @@
         </is>
       </c>
       <c r="D67" t="n">
-        <v>0.166036</v>
+        <v>0.15</v>
       </c>
       <c r="E67" t="inlineStr">
         <is>

</xml_diff>

<commit_message>
task-10/11 acceptance wave: CadQuery builds for all trains, GA sheet sets + build logs, envelope size recovery for 65 units; desk P4 481 -> 2
</commit_message>
<xml_diff>
--- a/docs-authority/MODEL_WORKBOOK.xlsx
+++ b/docs-authority/MODEL_WORKBOOK.xlsx
@@ -563,7 +563,7 @@
       </c>
       <c r="B5" t="inlineStr">
         <is>
-          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 dda6fec22e1d2666daa38b0e6ced69c0b98553d4a8f7c427054b6d58ef2a48d5</t>
+          <t>flow_graph/plant_flow_graph.json -- revision AC -- sha256 a68069cea430aa988f392ed5983c64b1e0fc779ac1b46b8bff45f81929bf5159</t>
         </is>
       </c>
     </row>
@@ -21695,7 +21695,7 @@
         </is>
       </c>
       <c r="B7" s="8" t="n">
-        <v>368.9079</v>
+        <v>368.9871</v>
       </c>
       <c r="C7" t="inlineStr">
         <is>
@@ -21796,7 +21796,7 @@
         </is>
       </c>
       <c r="B10" s="8" t="n">
-        <v>217.8701</v>
+        <v>217.9501</v>
       </c>
       <c r="C10" t="inlineStr">
         <is>
@@ -22601,7 +22601,7 @@
         </is>
       </c>
       <c r="D40" t="n">
-        <v>368.9079</v>
+        <v>368.9871</v>
       </c>
       <c r="E40" t="inlineStr">
         <is>
@@ -23283,7 +23283,7 @@
         </is>
       </c>
       <c r="D63" t="n">
-        <v>915.526468</v>
+        <v>915.8626410000001</v>
       </c>
       <c r="E63" t="inlineStr">
         <is>
@@ -23313,7 +23313,7 @@
         </is>
       </c>
       <c r="D64" t="n">
-        <v>915.526468</v>
+        <v>915.8626410000001</v>
       </c>
       <c r="E64" t="inlineStr">
         <is>
@@ -24513,7 +24513,7 @@
         </is>
       </c>
       <c r="D104" t="n">
-        <v>0.7388</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="E104" t="inlineStr">
         <is>
@@ -57895,7 +57895,7 @@
         </is>
       </c>
       <c r="B5" s="8" t="n">
-        <v>0.7388</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="C5" t="inlineStr">
         <is>
@@ -58921,7 +58921,7 @@
         </is>
       </c>
       <c r="D42" t="n">
-        <v>0.7388</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="E42" t="inlineStr">
         <is>
@@ -63442,7 +63442,7 @@
         <v>10</v>
       </c>
       <c r="H57" s="5" t="n">
-        <v>701.9663</v>
+        <v>702.1255</v>
       </c>
       <c r="I57" t="n">
         <v>6</v>
@@ -63676,7 +63676,7 @@
         <v>3</v>
       </c>
       <c r="H63" s="5" t="n">
-        <v>372.9161</v>
+        <v>372.9953</v>
       </c>
       <c r="I63" t="n">
         <v>3</v>
@@ -63793,7 +63793,7 @@
         <v>1</v>
       </c>
       <c r="H66" s="5" t="n">
-        <v>368.9079</v>
+        <v>368.9871</v>
       </c>
       <c r="I66" t="n">
         <v>1</v>
@@ -63832,7 +63832,7 @@
         <v>3</v>
       </c>
       <c r="H67" s="5" t="n">
-        <v>217.8701</v>
+        <v>217.9501</v>
       </c>
       <c r="I67" t="n">
         <v>1</v>
@@ -63910,7 +63910,7 @@
         <v>1</v>
       </c>
       <c r="H69" s="5" t="n">
-        <v>217.8701</v>
+        <v>217.9501</v>
       </c>
       <c r="I69" t="n">
         <v>1</v>
@@ -69335,7 +69335,7 @@
         <v>6</v>
       </c>
       <c r="H209" s="5" t="n">
-        <v>1.9595</v>
+        <v>2.0387</v>
       </c>
       <c r="I209" t="n">
         <v>4</v>
@@ -69374,7 +69374,7 @@
         <v>6</v>
       </c>
       <c r="H210" s="5" t="n">
-        <v>1.9595</v>
+        <v>2.0387</v>
       </c>
       <c r="I210" t="n">
         <v>4</v>
@@ -69530,7 +69530,7 @@
         <v>1</v>
       </c>
       <c r="H214" s="5" t="n">
-        <v>0.7388</v>
+        <v>0.8179999999999999</v>
       </c>
       <c r="I214" t="n">
         <v>1</v>
@@ -72620,7 +72620,7 @@
         </is>
       </c>
       <c r="C2" s="6" t="n">
-        <v>217.87</v>
+        <v>217.95</v>
       </c>
       <c r="D2" t="inlineStr">
         <is>
@@ -72650,7 +72650,7 @@
         </is>
       </c>
       <c r="C3" s="6" t="n">
-        <v>544.6799999999999</v>
+        <v>544.88</v>
       </c>
       <c r="D3" t="inlineStr">
         <is>
@@ -72695,7 +72695,7 @@
         </is>
       </c>
       <c r="C5" t="n">
-        <v>6042</v>
+        <v>6044</v>
       </c>
     </row>
     <row r="6">
@@ -72796,7 +72796,7 @@
         </is>
       </c>
       <c r="C12" s="8" t="n">
-        <v>368.9079</v>
+        <v>368.9871</v>
       </c>
       <c r="D12" t="inlineStr">
         <is>
@@ -72821,7 +72821,7 @@
         </is>
       </c>
       <c r="C13" s="8" t="n">
-        <v>217.8701</v>
+        <v>217.9501</v>
       </c>
       <c r="D13" t="inlineStr">
         <is>
@@ -72924,7 +72924,7 @@
         </is>
       </c>
       <c r="C18" t="n">
-        <v>6042</v>
+        <v>6044</v>
       </c>
     </row>
     <row r="19">
@@ -72939,7 +72939,7 @@
         </is>
       </c>
       <c r="C19" t="n">
-        <v>3021</v>
+        <v>3022</v>
       </c>
     </row>
     <row r="20">
@@ -73014,7 +73014,7 @@
         </is>
       </c>
       <c r="C24" t="n">
-        <v>3051</v>
+        <v>3052</v>
       </c>
     </row>
     <row r="25">
@@ -73104,7 +73104,7 @@
         </is>
       </c>
       <c r="C30" t="n">
-        <v>2302.1</v>
+        <v>2302</v>
       </c>
     </row>
     <row r="31">

</xml_diff>